<commit_message>
Add Qattan passages for review, follow-up judging excludes shown passages, router states what is asked
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RkXtRf8o9rcFbV2XzFoBFz
</commit_message>
<xml_diff>
--- a/data/register.xlsx
+++ b/data/register.xlsx
@@ -18,7 +18,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="الملخص" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'للمراجعة'!$A$1:$V$42</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'للمراجعة'!$A$1:$V$49</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'المقاطع'!$A$1:$S$16</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -660,7 +660,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V42"/>
+  <dimension ref="A1:V49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -1794,46 +1794,88 @@
       <c r="U13" s="8" t="n"/>
       <c r="V13" s="8" t="n"/>
     </row>
-    <row r="14" ht="48" customHeight="1">
+    <row r="14" ht="150" customHeight="1">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>قالب</t>
+          <t>مقطع</t>
         </is>
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>و-01</t>
+          <t>ق-10</t>
         </is>
       </c>
       <c r="C14" s="6" t="inlineStr">
         <is>
-          <t>أعلى كل صفحة</t>
-        </is>
-      </c>
-      <c r="D14" s="6" t="n"/>
-      <c r="E14" s="6" t="n"/>
-      <c r="F14" s="6" t="n"/>
-      <c r="G14" s="6" t="n"/>
+          <t>ح2</t>
+        </is>
+      </c>
+      <c r="D14" s="6" t="inlineStr">
+        <is>
+          <t>أساسي</t>
+        </is>
+      </c>
+      <c r="E14" s="6" t="inlineStr">
+        <is>
+          <t>م-03</t>
+        </is>
+      </c>
+      <c r="F14" s="6" t="inlineStr">
+        <is>
+          <t>مباحث في علوم القرآن، مناع القطان — الفصل 4: المكي والمدني — الفرق بين المكي والمدني (ص 60 حسب فهرس الكتاب) — https://quranpedia.net/book/23563</t>
+        </is>
+      </c>
+      <c r="G14" s="6" t="inlineStr">
+        <is>
+          <t>الفرق بين المكي والمدني</t>
+        </is>
+      </c>
       <c r="H14" s="6" t="n"/>
-      <c r="I14" s="6" t="n"/>
-      <c r="J14" s="6" t="n"/>
+      <c r="I14" s="6" t="inlineStr">
+        <is>
+          <t>ما الفرق بين المكي والمدني؟ | ما معنى سورة مكية؟ | ما معنى سورة مدنية؟</t>
+        </is>
+      </c>
+      <c r="J14" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
       <c r="K14" s="6" t="inlineStr">
         <is>
-          <t>«دليل» أداة تستعين بالذكاء الاصطناعي لتختار لك مقطعاً من مصادر إسلامية معتمدة راجعها مختص. لا تكتب إجابات من عندها، وقد تخطئ في الاختيار.</t>
-        </is>
-      </c>
-      <c r="L14" s="6" t="n"/>
-      <c r="M14" s="6" t="n"/>
-      <c r="N14" s="6" t="n"/>
+          <t>للعلماء في الفرق بين المكي والمدني ثلاثة آراء اصطلاحية، كل رأي منها بُنِيَ على اعتبار خاص.
+الأول: اعتبار زمن النزول، فالمكي: ما نزل قبل الهجرة وإن كان بغير مكة، والمدني: ما نزل بعد الهجرة وإن كان بغير المدينة، فما نزل بعد الهجرة ولو بمكة، أو عرفة: مدني، كالذي نزل عام الفتح، كقوله تعالى: ﴿إِنَّ اللَّهَ يَأْمُرُكُمْ أَنْ تُؤَدُّوا الْأَمَانَاتِ إِلَى أَهْلِهَا﴾ [النساء: 58]، فإنها نزلت بمكة في جوف الكعبة عام الفتح الأعظم، أو نزل بحجة الوداع كقوله تعالى: ﴿الْيَوْمَ أَكْمَلْتُ لَكُمْ دِينَكُمْ وَأَتْمَمْتُ عَلَيْكُمْ نِعْمَتِي وَرَضِيتُ لَكُمُ الْإِسْلَامَ دِينًا﴾ [المائدة: 3]، وهذا الرأي أولى من الرأيين بعده لحصره واطراده.
+[…]</t>
+        </is>
+      </c>
+      <c r="L14" s="6" t="inlineStr">
+        <is>
+          <t>معنى «مكي» و«مدني»: المكي ما نزل قبل الهجرة، والمدني ما نزل بعدها، وهو أرجح الآراء الثلاثة.</t>
+        </is>
+      </c>
+      <c r="M14" s="6" t="inlineStr">
+        <is>
+          <t>ما معنى سورة مكية ومدنية؟ | يعني إيش مكية؟ | ليش مكتوب على السورة مدنية؟ | هل المكي ما نزل في مكة فقط؟</t>
+        </is>
+      </c>
+      <c r="N14" s="6" t="inlineStr">
+        <is>
+          <t>أ</t>
+        </is>
+      </c>
       <c r="O14" s="6" t="inlineStr">
         <is>
           <t>لا</t>
         </is>
       </c>
-      <c r="P14" s="6" t="n"/>
+      <c r="P14" s="6" t="inlineStr">
+        <is>
+          <t>النساء 58 (جزء)؛ المائدة 3 (جزء) — تُعرض من المصحف.</t>
+        </is>
+      </c>
       <c r="Q14" s="6" t="inlineStr">
         <is>
-          <t>مراجعة شرعية: نعم</t>
+          <t>أخذت الرأي الأول (الذي رجّحه المؤلف) كاملاً، وقصصت الرأيين الآخرين «[…]» لأنهما يربكان المبتدئ. حذفت أرقام الحواشي.</t>
         </is>
       </c>
       <c r="R14" s="6" t="n"/>
@@ -1842,46 +1884,88 @@
       <c r="U14" s="8" t="n"/>
       <c r="V14" s="8" t="n"/>
     </row>
-    <row r="15" ht="48" customHeight="1">
+    <row r="15" ht="150" customHeight="1">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>قالب</t>
+          <t>مقطع</t>
         </is>
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>و-02</t>
+          <t>ق-05</t>
         </is>
       </c>
       <c r="C15" s="6" t="inlineStr">
         <is>
-          <t>بعد كل جزء معروض</t>
-        </is>
-      </c>
-      <c r="D15" s="6" t="n"/>
-      <c r="E15" s="6" t="n"/>
-      <c r="F15" s="6" t="n"/>
-      <c r="G15" s="6" t="n"/>
+          <t>ح5</t>
+        </is>
+      </c>
+      <c r="D15" s="6" t="inlineStr">
+        <is>
+          <t>أساسي</t>
+        </is>
+      </c>
+      <c r="E15" s="6" t="inlineStr">
+        <is>
+          <t>م-03</t>
+        </is>
+      </c>
+      <c r="F15" s="6" t="inlineStr">
+        <is>
+          <t>مباحث في علوم القرآن، مناع القطان — الفصل 4: المكي والمدني — مدخل الفصل (ص 49–50 حسب فهرس الكتاب) — https://quranpedia.net/book/23563</t>
+        </is>
+      </c>
+      <c r="G15" s="6" t="inlineStr">
+        <is>
+          <t>خصائص الآيات المكية والمدنية</t>
+        </is>
+      </c>
       <c r="H15" s="6" t="n"/>
-      <c r="I15" s="6" t="n"/>
-      <c r="J15" s="6" t="n"/>
+      <c r="I15" s="6" t="inlineStr">
+        <is>
+          <t>ما موضوعات القرآن؟ | عن ماذا يتكلم القرآن؟ | ما الرسالة الأساسية في القرآن؟</t>
+        </is>
+      </c>
+      <c r="J15" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
       <c r="K15" s="6" t="inlineStr">
         <is>
-          <t>هل أجاب هذا عن سؤالك؟  [نعم] [جزئياً] [لا]</t>
-        </is>
-      </c>
-      <c r="L15" s="6" t="n"/>
-      <c r="M15" s="6" t="n"/>
-      <c r="N15" s="6" t="n"/>
+          <t>والذي يقرأ القرآن الكريم يجد للآيات المكية خصائص ليست للآيات المدنية في وقعها ومعانيها، وإن كانت الثانية مبنية على الأولى في الأحكام والتشريع.
+[…] نزل الوحي المكي قوارع زاجرة، وشهبًا منذرة، وحججًا قاطعة، يحطم وثنيتهم في العقيدة، ويدعوهم إلى توحيد الألوهية والربوبية، ويهتك أستار فسادهم، ويسَفِّه أحلامهم، ويقيم دلائل النبوة، ويضرب الأمثلة للحياة الآخرة وما فيها من جنة ونار، ويتحداهم -على فصاحتهم- بأن يأتوا بمثل القرآن، ويسوق إليهم قصص المكذبين الغابرين عبرة وذكرى […]
+وحين تكونت الجماعة المؤمنة بالله وملائكته وكتبه ورسله واليوم الآخر وبالقدر خيره وشره، وامتُحنت في عقيدتها بأذى المشركين فصبرت وهاجرت بدينها مؤثرة ما عند الله على متع الحياة -حين تكونت هذه الجماعة- نرى الآيات المدنية طويلة المقاطع، تتناول أحكام الإسلام وحدوده، وتدعو إلى الجهاد والاستشهاد في سبيل الله، وتفصل أصول التشريع، وتضع قواعد المجتمع، وتحدد روابط الأسرة، وصلات الأفراد، وعلاقات الدول والأمم، كما تفضح المنافقين وتكشف دخيلتهم، وتجادل أهل الكتاب وتلجم أفواههم -وهذا هو الطابع العام للقرآن المدني.</t>
+        </is>
+      </c>
+      <c r="L15" s="6" t="inlineStr">
+        <is>
+          <t>أبرز موضوعات القرآن: التوحيد، ودلائل النبوة، والآخرة والجنة والنار، وقصص الأمم السابقة، ثم الأحكام وقواعد المجتمع والأسرة.</t>
+        </is>
+      </c>
+      <c r="M15" s="6" t="inlineStr">
+        <is>
+          <t>عن ماذا يتكلم القرآن؟ | ما الرسالة الأساسية في القرآن؟ | هل القرآن كتاب أحكام فقط؟ | هل يتكلم القرآن عن يوم القيامة؟ | ماذا يطلب القرآن من الإنسان؟</t>
+        </is>
+      </c>
+      <c r="N15" s="6" t="inlineStr">
+        <is>
+          <t>أ</t>
+        </is>
+      </c>
       <c r="O15" s="6" t="inlineStr">
         <is>
           <t>لا</t>
         </is>
       </c>
-      <c r="P15" s="6" t="n"/>
+      <c r="P15" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
       <c r="Q15" s="6" t="inlineStr">
         <is>
-          <t>مراجعة شرعية: لا</t>
+          <t>قصّان «[…]»: (1) وصف حال المشركين وقولهم مع آيتين، (2) وصف ألفاظ المكي وأساليبه. يغطي هذا المقطع وحده ق-05 وق-07 المخططين (التوحيد، والآخرة، والقيم)، فحذفت ق-07 من «الناقص».</t>
         </is>
       </c>
       <c r="R15" s="6" t="n"/>
@@ -1890,46 +1974,92 @@
       <c r="U15" s="8" t="n"/>
       <c r="V15" s="8" t="n"/>
     </row>
-    <row r="16" ht="48" customHeight="1">
+    <row r="16" ht="150" customHeight="1">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>قالب</t>
+          <t>مقطع</t>
         </is>
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>و-03</t>
+          <t>ق-06</t>
         </is>
       </c>
       <c r="C16" s="6" t="inlineStr">
         <is>
-          <t>بعد «جزئياً»</t>
-        </is>
-      </c>
-      <c r="D16" s="6" t="n"/>
-      <c r="E16" s="6" t="n"/>
-      <c r="F16" s="6" t="n"/>
-      <c r="G16" s="6" t="n"/>
+          <t>ح5</t>
+        </is>
+      </c>
+      <c r="D16" s="6" t="inlineStr">
+        <is>
+          <t>أساسي</t>
+        </is>
+      </c>
+      <c r="E16" s="6" t="inlineStr">
+        <is>
+          <t>م-03</t>
+        </is>
+      </c>
+      <c r="F16" s="6" t="inlineStr">
+        <is>
+          <t>مباحث في علوم القرآن، مناع القطان — الفصل 21: قصص القرآن — معنى القصص، وأنواعه، وفوائده (ص 316–317 حسب فهرس الكتاب) — https://quranpedia.net/book/23563</t>
+        </is>
+      </c>
+      <c r="G16" s="6" t="inlineStr">
+        <is>
+          <t>قصص القرآن</t>
+        </is>
+      </c>
       <c r="H16" s="6" t="n"/>
-      <c r="I16" s="6" t="n"/>
-      <c r="J16" s="6" t="n"/>
+      <c r="I16" s="6" t="inlineStr">
+        <is>
+          <t>هل في القرآن قصص؟ | ما قصص القرآن؟ | هل يذكر القرآن الأنبياء؟</t>
+        </is>
+      </c>
+      <c r="J16" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
       <c r="K16" s="6" t="inlineStr">
         <is>
-          <t>ما الذي بقي دون إجابة؟ اكتبه بكلماتك.</t>
-        </is>
-      </c>
-      <c r="L16" s="6" t="n"/>
-      <c r="M16" s="6" t="n"/>
-      <c r="N16" s="6" t="n"/>
+          <t>وقصص القرآن: أخباره عن أحوال الأمم الماضية، والنبوات السابقة، والحوادث الواقعة - وقد اشتمل القرآن على كثير من وقائع الماضي، وتاريخ الأمم، وذكر البلاد والديار، وتتبع آثار كل قوم، وحكى عنهم صورة ناطقة لما كانوا عليه.
+والقصص في القرآن ثلاثة أنواع:
+النوع الأول: قصص الأنبياء، وقد تضمن دعوتهم إلى قومهم، والمعجزات التي أيدهم الله بها، وموقف المعاندين منهم، ومراحل الدعوة وتطورها وعاقبة المؤمنين والمكذبين، كقصص نوح، وإبراهيم، وموسى، وهارون، وعيسى، ومحمد، وغيرهم من الأنبياء والمرسلين، عليهم جميعًا أفضل الصلاة والسلام.
+[…]
+النوع الثالث: قصص يتعلق بالحوادث التي وقعت في زمن رسول الله -صلى الله عليه وسلم- كغزوة بدر وأحد في سورة آل عمران، وغزوة حنين وتبوك في التوبة، وغزوة الأحزاب في سورة الأحزاب، والهجرة، والإسراء، ونحو ذلك.
+وللقصص القرآني فوائد نجمل أهمها فيما يأتي:
+1- إيضاح أسس الدعوة إلى الله، وبيان أصول الشرائع التي بعث بها كل نبي: ﴿وَمَا أَرْسَلْنَا مِنْ قَبْلِكَ مِنْ رَسُولٍ إِلَّا نُوحِي إِلَيْهِ أَنَّهُ لَا إِلَهَ إِلَّا أَنَا فَاعْبُدُونِ﴾ [الأنبياء: 25].</t>
+        </is>
+      </c>
+      <c r="L16" s="6" t="inlineStr">
+        <is>
+          <t>هل في القرآن قصص؟ نعم: قصص الأنبياء، وأحداث زمن النبي ﷺ، والغاية منها بيان أسس الدعوة إلى التوحيد.</t>
+        </is>
+      </c>
+      <c r="M16" s="6" t="inlineStr">
+        <is>
+          <t>هل القرآن فيه قصص؟ | هل يذكر القرآن موسى وعيسى؟ | ليش القرآن يحكي قصص الأنبياء؟ | هل قصص القرآن حقيقية؟</t>
+        </is>
+      </c>
+      <c r="N16" s="6" t="inlineStr">
+        <is>
+          <t>أ</t>
+        </is>
+      </c>
       <c r="O16" s="6" t="inlineStr">
         <is>
           <t>لا</t>
         </is>
       </c>
-      <c r="P16" s="6" t="n"/>
+      <c r="P16" s="6" t="inlineStr">
+        <is>
+          <t>الأنبياء 25 (كاملة) — تُعرض من المصحف.</t>
+        </is>
+      </c>
       <c r="Q16" s="6" t="inlineStr">
         <is>
-          <t>مراجعة شرعية: لا</t>
+          <t>قصّ واحد «[…]»: النوع الثاني (فيه عبارة «لم تثبت ثبوتهم» قد تُفهم خطأً، ويحسن عرضها مع شرح). من الفوائد أخذت الأولى فقط لأن البقية لم ترد في النسخة الرقمية.</t>
         </is>
       </c>
       <c r="R16" s="6" t="n"/>
@@ -1938,46 +2068,91 @@
       <c r="U16" s="8" t="n"/>
       <c r="V16" s="8" t="n"/>
     </row>
-    <row r="17" ht="48" customHeight="1">
+    <row r="17" ht="150" customHeight="1">
       <c r="A17" s="5" t="inlineStr">
         <is>
-          <t>قالب</t>
+          <t>مقطع</t>
         </is>
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>و-04</t>
+          <t>ق-15</t>
         </is>
       </c>
       <c r="C17" s="6" t="inlineStr">
         <is>
-          <t>فوق كل مقطع (يُملأ من السجل)</t>
-        </is>
-      </c>
-      <c r="D17" s="6" t="n"/>
-      <c r="E17" s="6" t="n"/>
-      <c r="F17" s="6" t="n"/>
-      <c r="G17" s="6" t="n"/>
+          <t>ح4</t>
+        </is>
+      </c>
+      <c r="D17" s="6" t="inlineStr">
+        <is>
+          <t>أساسي</t>
+        </is>
+      </c>
+      <c r="E17" s="6" t="inlineStr">
+        <is>
+          <t>م-03</t>
+        </is>
+      </c>
+      <c r="F17" s="6" t="inlineStr">
+        <is>
+          <t>مباحث في علوم القرآن، مناع القطان — الفصل 8: جمع القرآن وترتيبه — ترتيب الآيات، وسور القرآن وآياته (ص 140، 145 حسب فهرس الكتاب) — https://quranpedia.net/book/23563</t>
+        </is>
+      </c>
+      <c r="G17" s="6" t="inlineStr">
+        <is>
+          <t>السورة والآية وعدد السور</t>
+        </is>
+      </c>
       <c r="H17" s="6" t="n"/>
-      <c r="I17" s="6" t="n"/>
-      <c r="J17" s="6" t="n"/>
+      <c r="I17" s="6" t="inlineStr">
+        <is>
+          <t>ما الفرق بين السورة والآية؟ | كم عدد سور القرآن؟ | كم عدد آيات القرآن؟</t>
+        </is>
+      </c>
+      <c r="J17" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
       <c r="K17" s="6" t="inlineStr">
         <is>
-          <t>يجيب هذا المقطع عن: {يجيب_عن}</t>
-        </is>
-      </c>
-      <c r="L17" s="6" t="n"/>
-      <c r="M17" s="6" t="n"/>
-      <c r="N17" s="6" t="n"/>
+          <t>القرآن سور وآيات منها القصار والطوال، والآية: هي الجملة من كلام الله المندرجة في سورة من القرآن، والسورة: هي الجملة من آيات القرآن ذات المطلع والمقطع.
+[…]
+وتعداد السور: مائة وأربع عشرة سورة، وقيل: وثلاث عشرة بجعل الأنفال وبراءة سورة واحدة.
+أما تعداد الآيات فستة آلاف ومائتا آية، واختلفوا فيما زاد عن ذلك.
+وأطول الآيات آية الدَّيْن، وأطول السور سورة البقرة.
+وهذه التجزئة تيسر على الناس الحفظ، وتحملهم على الدراسة، وتشعر القارئ لسورة من السور بأنه قد أخذ قسطاً وافيًا وطائفة مستقلة من أصول دينه وأحكام شريعته.</t>
+        </is>
+      </c>
+      <c r="L17" s="6" t="inlineStr">
+        <is>
+          <t>ما السورة وما الآية؟ وعدد سور القرآن 114 سورة، وآياته ستة آلاف ومئتان وزيادة.</t>
+        </is>
+      </c>
+      <c r="M17" s="6" t="inlineStr">
+        <is>
+          <t>كم عدد سور القرآن؟ | ما الفرق بين السورة والآية؟ | كم آية في القرآن؟ | ما أطول سورة؟</t>
+        </is>
+      </c>
+      <c r="N17" s="6" t="inlineStr">
+        <is>
+          <t>أ</t>
+        </is>
+      </c>
       <c r="O17" s="6" t="inlineStr">
         <is>
           <t>لا</t>
         </is>
       </c>
-      <c r="P17" s="6" t="n"/>
+      <c r="P17" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
       <c r="Q17" s="6" t="inlineStr">
         <is>
-          <t>مراجعة شرعية: لا</t>
+          <t>جمعت فقرتين من موضعين: تعريف الآية والسورة (ص 140) ثم العدد (ص 145)، وبينهما «[…]». أبقيت «وقيل: وثلاث عشرة» كما في المصدر.</t>
         </is>
       </c>
       <c r="R17" s="6" t="n"/>
@@ -1986,94 +2161,185 @@
       <c r="U17" s="8" t="n"/>
       <c r="V17" s="8" t="n"/>
     </row>
-    <row r="18" ht="48" customHeight="1">
+    <row r="18" ht="150" customHeight="1">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>قالب</t>
+          <t>مقطع</t>
         </is>
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>و-05</t>
+          <t>ق-16</t>
         </is>
       </c>
       <c r="C18" s="6" t="inlineStr">
         <is>
-          <t>تحت وصف «يجيب عن»</t>
-        </is>
-      </c>
-      <c r="D18" s="6" t="n"/>
-      <c r="E18" s="6" t="n"/>
-      <c r="F18" s="6" t="n"/>
-      <c r="G18" s="6" t="n"/>
+          <t>ح4</t>
+        </is>
+      </c>
+      <c r="D18" s="6" t="inlineStr">
+        <is>
+          <t>أساسي</t>
+        </is>
+      </c>
+      <c r="E18" s="6" t="inlineStr">
+        <is>
+          <t>م-03</t>
+        </is>
+      </c>
+      <c r="F18" s="6" t="inlineStr">
+        <is>
+          <t>مباحث في علوم القرآن، مناع القطان — الفصل 8: جمع القرآن وترتيبه — ترتيب الآيات وترتيب السور (ص 140–145 حسب فهرس الكتاب) — https://quranpedia.net/book/23563</t>
+        </is>
+      </c>
+      <c r="G18" s="6" t="inlineStr">
+        <is>
+          <t>ترتيب الآيات والسور</t>
+        </is>
+      </c>
       <c r="H18" s="6" t="n"/>
-      <c r="I18" s="6" t="n"/>
-      <c r="J18" s="6" t="n"/>
+      <c r="I18" s="6" t="inlineStr">
+        <is>
+          <t>من رتّب القرآن؟ | هل ترتيب المصحف حسب النزول؟ | لماذا السور مرتبة هكذا؟</t>
+        </is>
+      </c>
+      <c r="J18" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
       <c r="K18" s="6" t="inlineStr">
         <is>
-          <t>وصف مساعد كُتب بمساعدة الذكاء الاصطناعي وراجعه صاحب المشروع. النص المعتمد هو المقتبس.</t>
-        </is>
-      </c>
-      <c r="L18" s="6" t="n"/>
-      <c r="M18" s="6" t="n"/>
-      <c r="N18" s="6" t="n"/>
+          <t>وترتيب الآيات في القرآن الكريم توقيفي عن رسول الله -صلى الله عليه وسلم- وحكى بعضهم الإجماع على ذلك […] فقد كان جبريل يتنزل بالآيات على رسول الله -صلى الله عليه وسلم- ويرشده إلى موضعها من السورة أو الآيات التي نزلت قبل، فيأمر الرسول كتبة الوحي بكتابتها في موضعها ويقول لهم: ضعوا هذه الآيات في السورة التي يُذكر فيها كذا أو كذا، أو ضعوا آية كذا في موضع كذا […]
+وكان جبريل يعارض رسول الله -صلى الله عليه وسلم- بالقرآن كل عام مرة في رمضان، وعارضه في العام الأخير من حياته مرتين، وكان ذلك العرض على الترتيب المعروف الآن.
+[…]
+وبهذا يترجح أن ترتيب السور توقيفي كترتيب الآيات.</t>
+        </is>
+      </c>
+      <c r="L18" s="6" t="inlineStr">
+        <is>
+          <t>لماذا ليس ترتيب المصحف بحسب النزول؟ لأن ترتيب الآيات بأمر النبي ﷺ عن جبريل، والراجح أن ترتيب السور كذلك.</t>
+        </is>
+      </c>
+      <c r="M18" s="6" t="inlineStr">
+        <is>
+          <t>ليش السور مو مرتبة حسب نزولها؟ | من رتب سور القرآن؟ | هل ترتيب الآيات من النبي؟ | ليش البقرة أول القرآن مع إنها مدنية؟</t>
+        </is>
+      </c>
+      <c r="N18" s="6" t="inlineStr">
+        <is>
+          <t>أ</t>
+        </is>
+      </c>
       <c r="O18" s="6" t="inlineStr">
         <is>
           <t>لا</t>
         </is>
       </c>
-      <c r="P18" s="6" t="n"/>
+      <c r="P18" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
       <c r="Q18" s="6" t="inlineStr">
         <is>
-          <t>مراجعة شرعية: لا</t>
-        </is>
-      </c>
-      <c r="R18" s="6" t="n"/>
+          <t>ثلاثة قصوص «[…]»: أسماء من حكى الإجماع، والأحاديث والآثار (ستحتاج تخريجاً)، ومناقشة الآراء الثلاثة في ترتيب السور. الخلاف في ترتيب السور مذكور في المصدر، والمقطع يعرض الراجح فقط.</t>
+        </is>
+      </c>
+      <c r="R18" s="6" t="inlineStr">
+        <is>
+          <t>المصدر يذكر خلافاً في ترتيب السور ويرجّح التوقيف. هل عرض الراجح وحده مناسب للمبتدئ؟</t>
+        </is>
+      </c>
       <c r="S18" s="8" t="n"/>
       <c r="T18" s="8" t="n"/>
       <c r="U18" s="8" t="n"/>
       <c r="V18" s="8" t="n"/>
     </row>
-    <row r="19" ht="48" customHeight="1">
+    <row r="19" ht="150" customHeight="1">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t>قالب</t>
+          <t>مقطع</t>
         </is>
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>ست-01</t>
+          <t>ق-19</t>
         </is>
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>التباس بين ح1 وح7</t>
-        </is>
-      </c>
-      <c r="D19" s="6" t="n"/>
-      <c r="E19" s="6" t="n"/>
-      <c r="F19" s="6" t="n"/>
-      <c r="G19" s="6" t="n"/>
+          <t>ح6</t>
+        </is>
+      </c>
+      <c r="D19" s="6" t="inlineStr">
+        <is>
+          <t>أساسي</t>
+        </is>
+      </c>
+      <c r="E19" s="6" t="inlineStr">
+        <is>
+          <t>م-03</t>
+        </is>
+      </c>
+      <c r="F19" s="6" t="inlineStr">
+        <is>
+          <t>مباحث في علوم القرآن، مناع القطان — الفصل 23: التفسير والتأويل — مدخل الفصل، ومعنى التفسير، وشرف التفسير (ص 334، 339 حسب فهرس الكتاب) — https://quranpedia.net/book/23563</t>
+        </is>
+      </c>
+      <c r="G19" s="6" t="inlineStr">
+        <is>
+          <t>معنى التفسير والحاجة إليه</t>
+        </is>
+      </c>
       <c r="H19" s="6" t="n"/>
-      <c r="I19" s="6" t="n"/>
-      <c r="J19" s="6" t="n"/>
+      <c r="I19" s="6" t="inlineStr">
+        <is>
+          <t>ما التفسير؟ | كيف أفهم القرآن؟ | ما معنى تفسير القرآن؟</t>
+        </is>
+      </c>
+      <c r="J19" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
       <c r="K19" s="6" t="inlineStr">
         <is>
-          <t>هل تريد تعريفاً بالقرآن ومكانته، أم الأسباب التي تجعل المسلمين يؤمنون أنه من عند الله؟</t>
-        </is>
-      </c>
-      <c r="L19" s="6" t="n"/>
-      <c r="M19" s="6" t="n"/>
-      <c r="N19" s="6" t="n"/>
+          <t>ولا يستوي الناس جميعًا في فهم ألفاظه وعباراته مع وضوح بيانه وتفصيل آياته، فإن تفاوت الإدراك بينهم أمر لا مراء فيه فالعامي يدرك من المعاني ظاهرها ومن الآيات مجملها، والذكي المتعلم يستخرج منها المعنى الرائع. وبين هذا وذاك مراتب فهم شتى، فلا غرو أن يجد القرآن من أبناء أمته اهتمامًا بالغًا في الدراسة لتفسير غريب، أو تأويل تركيب.
+[…]
+وقال الزركشي: التفسير: علم يُفهم به كتاب الله المنزل على نبيه محمد, صلى الله عليه وسلم: وبيان معانيه، واستخراج أحكامه وحكمه.
+[…]
+والتفسير من أجلِّ علوم الشريعة وأرفعها قدرًا، وهو أشرف العلوم موضوعًا وغرضًا وحاجة إليه لأن موضوعه كلام الله تعالى الذي هو ينبوع كل حكمة.</t>
+        </is>
+      </c>
+      <c r="L19" s="6" t="inlineStr">
+        <is>
+          <t>إذا قرأت ولم تفهم: الناس يتفاوتون في الفهم، والتفسير هو العلم الذي يُفهم به القرآن وتُبيَّن معانيه.</t>
+        </is>
+      </c>
+      <c r="M19" s="6" t="inlineStr">
+        <is>
+          <t>أقرأ القرآن وما أفهم، شو أسوي؟ | ما هو التفسير؟ | كيف أفهم الكلمات الصعبة في القرآن؟ | هل أحتاج تفسير لأفهم القرآن؟</t>
+        </is>
+      </c>
+      <c r="N19" s="6" t="inlineStr">
+        <is>
+          <t>أ</t>
+        </is>
+      </c>
       <c r="O19" s="6" t="inlineStr">
         <is>
           <t>لا</t>
         </is>
       </c>
-      <c r="P19" s="6" t="n"/>
+      <c r="P19" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
       <c r="Q19" s="6" t="inlineStr">
         <is>
-          <t>مراجعة شرعية: نعم</t>
+          <t>ثلاث فقرات من الفصل: المدخل، وتعريف الزركشي (حذفت تعريف أبي حيان المطوّل)، وأول جملة من «شرف التفسير». لا يرشح المصدر تفسيراً بعينه للمبتدئ؛ يبقى ق-18 في «الناقص».</t>
         </is>
       </c>
       <c r="R19" s="6" t="n"/>
@@ -2082,49 +2348,99 @@
       <c r="U19" s="8" t="n"/>
       <c r="V19" s="8" t="n"/>
     </row>
-    <row r="20" ht="48" customHeight="1">
+    <row r="20" ht="150" customHeight="1">
       <c r="A20" s="5" t="inlineStr">
         <is>
-          <t>قالب</t>
+          <t>مقطع</t>
         </is>
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>ست-02</t>
+          <t>ق-20</t>
         </is>
       </c>
       <c r="C20" s="6" t="inlineStr">
         <is>
-          <t>التباس بين ح2 وح7</t>
-        </is>
-      </c>
-      <c r="D20" s="6" t="n"/>
-      <c r="E20" s="6" t="n"/>
-      <c r="F20" s="6" t="n"/>
-      <c r="G20" s="6" t="n"/>
+          <t>ح6</t>
+        </is>
+      </c>
+      <c r="D20" s="6" t="inlineStr">
+        <is>
+          <t>أساسي</t>
+        </is>
+      </c>
+      <c r="E20" s="6" t="inlineStr">
+        <is>
+          <t>م-03</t>
+        </is>
+      </c>
+      <c r="F20" s="6" t="inlineStr">
+        <is>
+          <t>مباحث في علوم القرآن، مناع القطان — الفصل 22: ترجمة القرآن — معنى الترجمة، وحكم الترجمة الحرفية، والترجمة التفسيرية (ص 324–327 حسب فهرس الكتاب) — https://quranpedia.net/book/23563</t>
+        </is>
+      </c>
+      <c r="G20" s="6" t="inlineStr">
+        <is>
+          <t>ترجمة القرآن: هل الترجمة قرآن؟</t>
+        </is>
+      </c>
       <c r="H20" s="6" t="n"/>
-      <c r="I20" s="6" t="n"/>
-      <c r="J20" s="6" t="n"/>
+      <c r="I20" s="6" t="inlineStr">
+        <is>
+          <t>هل ترجمة القرآن تعتبر قرآناً؟ | ما الفرق بين القرآن وترجمته؟ | هل يجوز ترجمة القرآن؟</t>
+        </is>
+      </c>
+      <c r="J20" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
       <c r="K20" s="6" t="inlineStr">
         <is>
-          <t>هل تقصد كيف كان الوحي يأتي النبي ﷺ، أم لماذا يؤمن المسلمون أن القرآن من عند الله؟</t>
-        </is>
-      </c>
-      <c r="L20" s="6" t="n"/>
-      <c r="M20" s="6" t="n"/>
-      <c r="N20" s="6" t="n"/>
+          <t>والترجمة تطلق على معنيين:
+أولهما: الترجمة الحرفية: وهي نقل ألفاظ من لغة إلى نظائرها من اللغة الأخرى بحيث يكون النظم موافقًا للنظم، والترتيب موافقًا للترتيب.
+ثانيهما: الترجمة التفسيرية أو المعنوية: وهي بيان معنى الكلام بلغة أخرى من غير تقييد بترتيب كلمات الأصل أو مراعاة لنظمه.
+[…]
+ولا يقول أحد من الناس إن الكلمة من القرآن إذا ترجمت يقال فيها إنها كلام الله، فإن الله لم يتكلم إلا بما تتلوه بالعربية […]
+ويحق لنا أن نقول: إن علماء الإسلام إذا قاموا بتفسير للقرآن، يتوخى فيه أداء المعنى القريب الميسور الراجح، ثم يترجم هذا التفسير بأمانة وبراعة، فإن هذا يقال فيه: "ترجمة تفسير القرآن" أو "ترجمة تفسيرية" بمعنى شرح الكلام وبيان معناه بلغة أخرى. ولا بأس بذلك. […]
+فالمفسِّر يقول في تفسير الآية: يعني كذا، ويذكر فهمه الخاص. والمترجم يقول: معنى هذا الكلام هو عين معنى الآية، وقد عرفنا ما في ذلك.</t>
+        </is>
+      </c>
+      <c r="L20" s="6" t="inlineStr">
+        <is>
+          <t>الترجمة ليست قرآناً؛ القرآن هو النص العربي، وما يُترجم هو تفسير لمعانيه بلغة أخرى.</t>
+        </is>
+      </c>
+      <c r="M20" s="6" t="inlineStr">
+        <is>
+          <t>هل الترجمة تعتبر قرآناً؟ | أقدر أقرأ القرآن بالإنجليزي؟ | ما الفرق بين القرآن وترجمة معانيه؟ | ليش يقولون ترجمة معاني القرآن؟</t>
+        </is>
+      </c>
+      <c r="N20" s="6" t="inlineStr">
+        <is>
+          <t>أ</t>
+        </is>
+      </c>
       <c r="O20" s="6" t="inlineStr">
         <is>
           <t>لا</t>
         </is>
       </c>
-      <c r="P20" s="6" t="n"/>
+      <c r="P20" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
       <c r="Q20" s="6" t="inlineStr">
         <is>
-          <t>مراجعة شرعية: نعم</t>
-        </is>
-      </c>
-      <c r="R20" s="6" t="n"/>
+          <t>القصوص «[…]»: شرح اختلاف تراكيب اللغات، وبقية حكم الترجمة الحرفية (فيه لفظ «حرمة»)، والحديث وما بعده. «القراءة في الصلاة بغير العربية» خارج النطاق (فتوى) ولم تؤخذ.</t>
+        </is>
+      </c>
+      <c r="R20" s="6" t="inlineStr">
+        <is>
+          <t>المقطع يقتصر على أن الترجمة ليست قرآناً وأن ترجمة التفسير لا بأس بها، ولم أنقل لفظ الحكم «حرمة». هل يكفي هذا؟</t>
+        </is>
+      </c>
       <c r="S20" s="8" t="n"/>
       <c r="T20" s="8" t="n"/>
       <c r="U20" s="8" t="n"/>
@@ -2138,12 +2454,12 @@
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>ست-03</t>
+          <t>و-01</t>
         </is>
       </c>
       <c r="C21" s="6" t="inlineStr">
         <is>
-          <t>سؤال عن «نسخ مختلفة» أو تغيّر القرآن</t>
+          <t>أعلى كل صفحة</t>
         </is>
       </c>
       <c r="D21" s="6" t="n"/>
@@ -2155,7 +2471,7 @@
       <c r="J21" s="6" t="n"/>
       <c r="K21" s="6" t="inlineStr">
         <is>
-          <t>هل تسأل: هل القرآن الذي بين أيدينا هو نفسه الذي نزل على النبي ﷺ؟</t>
+          <t>«دليل» أداة تستعين بالذكاء الاصطناعي لتختار لك مقطعاً من مصادر إسلامية معتمدة راجعها مختص. لا تكتب إجابات من عندها، وقد تخطئ في الاختيار.</t>
         </is>
       </c>
       <c r="L21" s="6" t="n"/>
@@ -2186,12 +2502,12 @@
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>ست-04</t>
+          <t>و-02</t>
         </is>
       </c>
       <c r="C22" s="6" t="inlineStr">
         <is>
-          <t>سؤال واسع</t>
+          <t>بعد كل جزء معروض</t>
         </is>
       </c>
       <c r="D22" s="6" t="n"/>
@@ -2203,7 +2519,7 @@
       <c r="J22" s="6" t="n"/>
       <c r="K22" s="6" t="inlineStr">
         <is>
-          <t>يمكننا أن نبدأ من أكثر من جهة، فبأيّها تبدأ؟</t>
+          <t>هل أجاب هذا عن سؤالك؟  [نعم] [جزئياً] [لا]</t>
         </is>
       </c>
       <c r="L22" s="6" t="n"/>
@@ -2234,12 +2550,12 @@
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>ام-01</t>
+          <t>و-03</t>
         </is>
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
-          <t>سؤال خارج القرآن</t>
+          <t>بعد «جزئياً»</t>
         </is>
       </c>
       <c r="D23" s="6" t="n"/>
@@ -2251,7 +2567,7 @@
       <c r="J23" s="6" t="n"/>
       <c r="K23" s="6" t="inlineStr">
         <is>
-          <t>يختص «دليل» حالياً بالتعرّف إلى القرآن الكريم، وسؤالك عن موضوع آخر. يمكنك الرجوع إلى الموسوعات العلمية في موقع الدرر السنية (dorar.net).</t>
+          <t>ما الذي بقي دون إجابة؟ اكتبه بكلماتك.</t>
         </is>
       </c>
       <c r="L23" s="6" t="n"/>
@@ -2265,7 +2581,7 @@
       <c r="P23" s="6" t="n"/>
       <c r="Q23" s="6" t="inlineStr">
         <is>
-          <t>مراجعة شرعية: نعم</t>
+          <t>مراجعة شرعية: لا</t>
         </is>
       </c>
       <c r="R23" s="6" t="n"/>
@@ -2282,12 +2598,12 @@
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>ام-02</t>
+          <t>و-04</t>
         </is>
       </c>
       <c r="C24" s="6" t="inlineStr">
         <is>
-          <t>فتوى أو حالة شخصية (المستوى د)</t>
+          <t>فوق كل مقطع (يُملأ من السجل)</t>
         </is>
       </c>
       <c r="D24" s="6" t="n"/>
@@ -2299,7 +2615,7 @@
       <c r="J24" s="6" t="n"/>
       <c r="K24" s="6" t="inlineStr">
         <is>
-          <t>سؤالك يحتاج إلى جواب يراعي حالتك بعينها، وهذا خارج ما يقدمه «دليل». ننصحك بسؤال عالم أو جهة إفتاء موثوقة في بلدك.</t>
+          <t>يجيب هذا المقطع عن: {يجيب_عن}</t>
         </is>
       </c>
       <c r="L24" s="6" t="n"/>
@@ -2313,7 +2629,7 @@
       <c r="P24" s="6" t="n"/>
       <c r="Q24" s="6" t="inlineStr">
         <is>
-          <t>مراجعة شرعية: نعم</t>
+          <t>مراجعة شرعية: لا</t>
         </is>
       </c>
       <c r="R24" s="6" t="n"/>
@@ -2330,12 +2646,12 @@
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>ام-03</t>
+          <t>و-05</t>
         </is>
       </c>
       <c r="C25" s="6" t="inlineStr">
         <is>
-          <t>القراءات وأوجه الأداء (قرار نطاق)</t>
+          <t>تحت وصف «يجيب عن»</t>
         </is>
       </c>
       <c r="D25" s="6" t="n"/>
@@ -2347,7 +2663,7 @@
       <c r="J25" s="6" t="n"/>
       <c r="K25" s="6" t="inlineStr">
         <is>
-          <t>تفاصيل القراءات علم متخصص لا يغطيه «دليل» في نسخته الحالية، ويُرجع فيه إلى أهل الاختصاص.</t>
+          <t>وصف مساعد كُتب بمساعدة الذكاء الاصطناعي وراجعه صاحب المشروع. النص المعتمد هو المقتبس.</t>
         </is>
       </c>
       <c r="L25" s="6" t="n"/>
@@ -2361,7 +2677,7 @@
       <c r="P25" s="6" t="n"/>
       <c r="Q25" s="6" t="inlineStr">
         <is>
-          <t>مراجعة شرعية: نعم</t>
+          <t>مراجعة شرعية: لا</t>
         </is>
       </c>
       <c r="R25" s="6" t="n"/>
@@ -2378,12 +2694,12 @@
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>ام-04</t>
+          <t>ست-01</t>
         </is>
       </c>
       <c r="C26" s="6" t="inlineStr">
         <is>
-          <t>«الإعجاز العلمي» (قرار نطاق)</t>
+          <t>التباس بين ح1 وح7</t>
         </is>
       </c>
       <c r="D26" s="6" t="n"/>
@@ -2395,7 +2711,7 @@
       <c r="J26" s="6" t="n"/>
       <c r="K26" s="6" t="inlineStr">
         <is>
-          <t>هذا الموضوع خارج ما تغطيه هذه النسخة من «دليل».</t>
+          <t>هل تريد تعريفاً بالقرآن ومكانته، أم الأسباب التي تجعل المسلمين يؤمنون أنه من عند الله؟</t>
         </is>
       </c>
       <c r="L26" s="6" t="n"/>
@@ -2426,12 +2742,12 @@
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>ام-05</t>
+          <t>ست-02</t>
         </is>
       </c>
       <c r="C27" s="6" t="inlineStr">
         <is>
-          <t>طلب حديث أو نص غير موجود في المواد</t>
+          <t>التباس بين ح2 وح7</t>
         </is>
       </c>
       <c r="D27" s="6" t="n"/>
@@ -2443,7 +2759,7 @@
       <c r="J27" s="6" t="n"/>
       <c r="K27" s="6" t="inlineStr">
         <is>
-          <t>لم نجد في مواد «دليل» المراجعة ما يطابق طلبك، ولا نعرض نصاً لم نتحقق منه. يمكنك البحث في الموسوعة الحديثية بموقع الدرر السنية، مع حكم كل حديث.</t>
+          <t>هل تقصد كيف كان الوحي يأتي النبي ﷺ، أم لماذا يؤمن المسلمون أن القرآن من عند الله؟</t>
         </is>
       </c>
       <c r="L27" s="6" t="n"/>
@@ -2474,12 +2790,12 @@
       </c>
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>ام-06</t>
+          <t>ست-03</t>
         </is>
       </c>
       <c r="C28" s="6" t="inlineStr">
         <is>
-          <t>آية لم تُعثر عليها في المصحف</t>
+          <t>سؤال عن «نسخ مختلفة» أو تغيّر القرآن</t>
         </is>
       </c>
       <c r="D28" s="6" t="n"/>
@@ -2491,7 +2807,7 @@
       <c r="J28" s="6" t="n"/>
       <c r="K28" s="6" t="inlineStr">
         <is>
-          <t>لم نجد آية تطابق النص الذي كتبته. يمكنك البحث عنها في مصحف موثوق مثل quranpedia.net.</t>
+          <t>هل تسأل: هل القرآن الذي بين أيدينا هو نفسه الذي نزل على النبي ﷺ؟</t>
         </is>
       </c>
       <c r="L28" s="6" t="n"/>
@@ -2505,7 +2821,7 @@
       <c r="P28" s="6" t="n"/>
       <c r="Q28" s="6" t="inlineStr">
         <is>
-          <t>مراجعة شرعية: لا</t>
+          <t>مراجعة شرعية: نعم</t>
         </is>
       </c>
       <c r="R28" s="6" t="n"/>
@@ -2522,12 +2838,12 @@
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>ام-07</t>
+          <t>ست-04</t>
         </is>
       </c>
       <c r="C29" s="6" t="inlineStr">
         <is>
-          <t>الحاجة داخل النطاق ولا جزء مناسب</t>
+          <t>سؤال واسع</t>
         </is>
       </c>
       <c r="D29" s="6" t="n"/>
@@ -2539,7 +2855,7 @@
       <c r="J29" s="6" t="n"/>
       <c r="K29" s="6" t="inlineStr">
         <is>
-          <t>لم نجد في مواد «دليل» المراجعة جزءاً يجيب عن هذا بدقة. نفضّل أن نخبرك بذلك على أن نعرض عليك ما لا يجيب. اختر من الأسئلة المتاحة أدناه.</t>
+          <t>يمكننا أن نبدأ من أكثر من جهة، فبأيّها تبدأ؟</t>
         </is>
       </c>
       <c r="L29" s="6" t="n"/>
@@ -2570,12 +2886,12 @@
       </c>
       <c r="B30" s="5" t="inlineStr">
         <is>
-          <t>ام-08</t>
+          <t>ام-01</t>
         </is>
       </c>
       <c r="C30" s="6" t="inlineStr">
         <is>
-          <t>سؤال بغير العربية</t>
+          <t>سؤال خارج القرآن</t>
         </is>
       </c>
       <c r="D30" s="6" t="n"/>
@@ -2587,7 +2903,7 @@
       <c r="J30" s="6" t="n"/>
       <c r="K30" s="6" t="inlineStr">
         <is>
-          <t>يعمل «دليل» حالياً باللغة العربية فقط. — Daleel currently works in Arabic only.</t>
+          <t>يختص «دليل» حالياً بالتعرّف إلى القرآن الكريم، وسؤالك عن موضوع آخر. يمكنك الرجوع إلى الموسوعات العلمية في موقع الدرر السنية (dorar.net).</t>
         </is>
       </c>
       <c r="L30" s="6" t="n"/>
@@ -2601,7 +2917,7 @@
       <c r="P30" s="6" t="n"/>
       <c r="Q30" s="6" t="inlineStr">
         <is>
-          <t>مراجعة شرعية: لا</t>
+          <t>مراجعة شرعية: نعم</t>
         </is>
       </c>
       <c r="R30" s="6" t="n"/>
@@ -2618,12 +2934,12 @@
       </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>ام-09</t>
+          <t>ام-02</t>
         </is>
       </c>
       <c r="C31" s="6" t="inlineStr">
         <is>
-          <t>تفسير آية بعينها (قرار نطاق)</t>
+          <t>فتوى أو حالة شخصية (المستوى د)</t>
         </is>
       </c>
       <c r="D31" s="6" t="n"/>
@@ -2635,7 +2951,7 @@
       <c r="J31" s="6" t="n"/>
       <c r="K31" s="6" t="inlineStr">
         <is>
-          <t>تفسير آيات بعينها خارج ما يغطيه «دليل» حالياً. يمكنك الرجوع إلى موسوعة التفسير بموقع الدرر السنية.</t>
+          <t>سؤالك يحتاج إلى جواب يراعي حالتك بعينها، وهذا خارج ما يقدمه «دليل». ننصحك بسؤال عالم أو جهة إفتاء موثوقة في بلدك.</t>
         </is>
       </c>
       <c r="L31" s="6" t="n"/>
@@ -2666,12 +2982,12 @@
       </c>
       <c r="B32" s="5" t="inlineStr">
         <is>
-          <t>ام-10</t>
+          <t>ام-03</t>
         </is>
       </c>
       <c r="C32" s="6" t="inlineStr">
         <is>
-          <t>تعطل خدمة الفهم</t>
+          <t>القراءات وأوجه الأداء (قرار نطاق)</t>
         </is>
       </c>
       <c r="D32" s="6" t="n"/>
@@ -2683,7 +2999,7 @@
       <c r="J32" s="6" t="n"/>
       <c r="K32" s="6" t="inlineStr">
         <is>
-          <t>خدمة فهم الأسئلة متوقفة مؤقتاً. اختر سؤالك من القائمة.</t>
+          <t>تفاصيل القراءات علم متخصص لا يغطيه «دليل» في نسخته الحالية، ويُرجع فيه إلى أهل الاختصاص.</t>
         </is>
       </c>
       <c r="L32" s="6" t="n"/>
@@ -2697,7 +3013,7 @@
       <c r="P32" s="6" t="n"/>
       <c r="Q32" s="6" t="inlineStr">
         <is>
-          <t>مراجعة شرعية: لا</t>
+          <t>مراجعة شرعية: نعم</t>
         </is>
       </c>
       <c r="R32" s="6" t="n"/>
@@ -2714,12 +3030,12 @@
       </c>
       <c r="B33" s="5" t="inlineStr">
         <is>
-          <t>و-06</t>
+          <t>ام-04</t>
         </is>
       </c>
       <c r="C33" s="6" t="inlineStr">
         <is>
-          <t>فوق نص المقطع (يُملأ من السجل)</t>
+          <t>«الإعجاز العلمي» (قرار نطاق)</t>
         </is>
       </c>
       <c r="D33" s="6" t="n"/>
@@ -2731,7 +3047,7 @@
       <c r="J33" s="6" t="n"/>
       <c r="K33" s="6" t="inlineStr">
         <is>
-          <t>من جواب «{المصدر}» عن سؤال: {عنوان_المسألة}</t>
+          <t>هذا الموضوع خارج ما تغطيه هذه النسخة من «دليل».</t>
         </is>
       </c>
       <c r="L33" s="6" t="n"/>
@@ -2745,7 +3061,7 @@
       <c r="P33" s="6" t="n"/>
       <c r="Q33" s="6" t="inlineStr">
         <is>
-          <t>مراجعة شرعية: لا</t>
+          <t>مراجعة شرعية: نعم</t>
         </is>
       </c>
       <c r="R33" s="6" t="n"/>
@@ -2762,12 +3078,12 @@
       </c>
       <c r="B34" s="5" t="inlineStr">
         <is>
-          <t>و-07</t>
+          <t>ام-05</t>
         </is>
       </c>
       <c r="C34" s="6" t="inlineStr">
         <is>
-          <t>شاشة البداية</t>
+          <t>طلب حديث أو نص غير موجود في المواد</t>
         </is>
       </c>
       <c r="D34" s="6" t="n"/>
@@ -2779,7 +3095,7 @@
       <c r="J34" s="6" t="n"/>
       <c r="K34" s="6" t="inlineStr">
         <is>
-          <t>اكتب سؤالك عن القرآن بكلماتك، مثل: كيف حُفظ القرآن؟ أو اختر من الأسئلة أدناه.</t>
+          <t>لم نجد في مواد «دليل» المراجعة ما يطابق طلبك، ولا نعرض نصاً لم نتحقق منه. يمكنك البحث في الموسوعة الحديثية بموقع الدرر السنية، مع حكم كل حديث.</t>
         </is>
       </c>
       <c r="L34" s="6" t="n"/>
@@ -2793,7 +3109,7 @@
       <c r="P34" s="6" t="n"/>
       <c r="Q34" s="6" t="inlineStr">
         <is>
-          <t>مراجعة شرعية: لا</t>
+          <t>مراجعة شرعية: نعم</t>
         </is>
       </c>
       <c r="R34" s="6" t="n"/>
@@ -2810,12 +3126,12 @@
       </c>
       <c r="B35" s="5" t="inlineStr">
         <is>
-          <t>و-08</t>
+          <t>ام-06</t>
         </is>
       </c>
       <c r="C35" s="6" t="inlineStr">
         <is>
-          <t>سطر الخصوصية</t>
+          <t>آية لم تُعثر عليها في المصحف</t>
         </is>
       </c>
       <c r="D35" s="6" t="n"/>
@@ -2827,7 +3143,7 @@
       <c r="J35" s="6" t="n"/>
       <c r="K35" s="6" t="inlineStr">
         <is>
-          <t>لا تكتب اسمك أو أي معلومات شخصية. لا نحفظ نص سؤالك، ونرسله إلى مزوّد النموذج اللغوي لفهمه فقط.</t>
+          <t>لم نجد آية تطابق النص الذي كتبته. يمكنك البحث عنها في مصحف موثوق مثل quranpedia.net.</t>
         </is>
       </c>
       <c r="L35" s="6" t="n"/>
@@ -2858,12 +3174,12 @@
       </c>
       <c r="B36" s="5" t="inlineStr">
         <is>
-          <t>و-09</t>
+          <t>ام-07</t>
         </is>
       </c>
       <c r="C36" s="6" t="inlineStr">
         <is>
-          <t>بعد «لا»</t>
+          <t>الحاجة داخل النطاق ولا جزء مناسب</t>
         </is>
       </c>
       <c r="D36" s="6" t="n"/>
@@ -2875,7 +3191,7 @@
       <c r="J36" s="6" t="n"/>
       <c r="K36" s="6" t="inlineStr">
         <is>
-          <t>شكراً لإخبارنا. يمكنك إعادة صياغة سؤالك، أو اختيار سؤال من القائمة.</t>
+          <t>لم نجد في مواد «دليل» المراجعة جزءاً يجيب عن هذا بدقة. نفضّل أن نخبرك بذلك على أن نعرض عليك ما لا يجيب. اختر من الأسئلة المتاحة أدناه.</t>
         </is>
       </c>
       <c r="L36" s="6" t="n"/>
@@ -2906,12 +3222,12 @@
       </c>
       <c r="B37" s="5" t="inlineStr">
         <is>
-          <t>و-10</t>
+          <t>ام-08</t>
         </is>
       </c>
       <c r="C37" s="6" t="inlineStr">
         <is>
-          <t>بعد «نعم»</t>
+          <t>سؤال بغير العربية</t>
         </is>
       </c>
       <c r="D37" s="6" t="n"/>
@@ -2923,7 +3239,7 @@
       <c r="J37" s="6" t="n"/>
       <c r="K37" s="6" t="inlineStr">
         <is>
-          <t>قد يهمك بعدها:</t>
+          <t>يعمل «دليل» حالياً باللغة العربية فقط. — Daleel currently works in Arabic only.</t>
         </is>
       </c>
       <c r="L37" s="6" t="n"/>
@@ -2954,12 +3270,12 @@
       </c>
       <c r="B38" s="5" t="inlineStr">
         <is>
-          <t>و-11</t>
+          <t>ام-09</t>
         </is>
       </c>
       <c r="C38" s="6" t="inlineStr">
         <is>
-          <t>إدخال فارغ أو غير مفهوم</t>
+          <t>تفسير آية بعينها (قرار نطاق)</t>
         </is>
       </c>
       <c r="D38" s="6" t="n"/>
@@ -2971,7 +3287,7 @@
       <c r="J38" s="6" t="n"/>
       <c r="K38" s="6" t="inlineStr">
         <is>
-          <t>لم نتمكن من قراءة سؤالك. اكتب سؤالاً قصيراً عن القرآن، أو اختر من القائمة.</t>
+          <t>تفسير آيات بعينها خارج ما يغطيه «دليل» حالياً. يمكنك الرجوع إلى موسوعة التفسير بموقع الدرر السنية.</t>
         </is>
       </c>
       <c r="L38" s="6" t="n"/>
@@ -2985,7 +3301,7 @@
       <c r="P38" s="6" t="n"/>
       <c r="Q38" s="6" t="inlineStr">
         <is>
-          <t>مراجعة شرعية: لا</t>
+          <t>مراجعة شرعية: نعم</t>
         </is>
       </c>
       <c r="R38" s="6" t="n"/>
@@ -3002,12 +3318,12 @@
       </c>
       <c r="B39" s="5" t="inlineStr">
         <is>
-          <t>و-12</t>
+          <t>ام-10</t>
         </is>
       </c>
       <c r="C39" s="6" t="inlineStr">
         <is>
-          <t>ما بقي غير مغطى</t>
+          <t>تعطل خدمة الفهم</t>
         </is>
       </c>
       <c r="D39" s="6" t="n"/>
@@ -3019,7 +3335,7 @@
       <c r="J39" s="6" t="n"/>
       <c r="K39" s="6" t="inlineStr">
         <is>
-          <t>لم نجد في مواد «دليل» جزءاً آخر يجيب عمّا بقي من سؤالك. نفضّل أن نخبرك بذلك على أن نعرض ما لا يجيب.</t>
+          <t>خدمة فهم الأسئلة متوقفة مؤقتاً. اختر سؤالك من القائمة.</t>
         </is>
       </c>
       <c r="L39" s="6" t="n"/>
@@ -3050,12 +3366,12 @@
       </c>
       <c r="B40" s="5" t="inlineStr">
         <is>
-          <t>و-13</t>
+          <t>و-06</t>
         </is>
       </c>
       <c r="C40" s="6" t="inlineStr">
         <is>
-          <t>آية مطابقة للمصحف</t>
+          <t>فوق نص المقطع (يُملأ من السجل)</t>
         </is>
       </c>
       <c r="D40" s="6" t="n"/>
@@ -3067,7 +3383,7 @@
       <c r="J40" s="6" t="n"/>
       <c r="K40" s="6" t="inlineStr">
         <is>
-          <t>هذا نص الآية كما في المصحف:</t>
+          <t>من جواب «{المصدر}» عن سؤال: {عنوان_المسألة}</t>
         </is>
       </c>
       <c r="L40" s="6" t="n"/>
@@ -3098,12 +3414,12 @@
       </c>
       <c r="B41" s="5" t="inlineStr">
         <is>
-          <t>و-14</t>
+          <t>و-07</t>
         </is>
       </c>
       <c r="C41" s="6" t="inlineStr">
         <is>
-          <t>آية مكتوبة بنص مختلف</t>
+          <t>شاشة البداية</t>
         </is>
       </c>
       <c r="D41" s="6" t="n"/>
@@ -3115,7 +3431,7 @@
       <c r="J41" s="6" t="n"/>
       <c r="K41" s="6" t="inlineStr">
         <is>
-          <t>النص الذي كتبته يختلف عن نص المصحف. هذا نص الآية كما في المصحف:</t>
+          <t>اكتب سؤالك عن القرآن بكلماتك، مثل: كيف حُفظ القرآن؟ أو اختر من الأسئلة أدناه.</t>
         </is>
       </c>
       <c r="L41" s="6" t="n"/>
@@ -3129,7 +3445,7 @@
       <c r="P41" s="6" t="n"/>
       <c r="Q41" s="6" t="inlineStr">
         <is>
-          <t>مراجعة شرعية: نعم</t>
+          <t>مراجعة شرعية: لا</t>
         </is>
       </c>
       <c r="R41" s="6" t="n"/>
@@ -3146,12 +3462,12 @@
       </c>
       <c r="B42" s="5" t="inlineStr">
         <is>
-          <t>و-15</t>
+          <t>و-08</t>
         </is>
       </c>
       <c r="C42" s="6" t="inlineStr">
         <is>
-          <t>أسفل كل مقطع</t>
+          <t>سطر الخصوصية</t>
         </is>
       </c>
       <c r="D42" s="6" t="n"/>
@@ -3163,7 +3479,7 @@
       <c r="J42" s="6" t="n"/>
       <c r="K42" s="6" t="inlineStr">
         <is>
-          <t>لا يتجاوز «دليل» هذا النص المقتبس، ولا يضيف إليه شرحاً من عنده.</t>
+          <t>لا تكتب اسمك أو أي معلومات شخصية. لا نحفظ نص سؤالك، ونرسله إلى مزوّد النموذج اللغوي لفهمه فقط.</t>
         </is>
       </c>
       <c r="L42" s="6" t="n"/>
@@ -3186,14 +3502,359 @@
       <c r="U42" s="8" t="n"/>
       <c r="V42" s="8" t="n"/>
     </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>قالب</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="inlineStr">
+        <is>
+          <t>و-09</t>
+        </is>
+      </c>
+      <c r="C43" s="6" t="inlineStr">
+        <is>
+          <t>بعد «لا»</t>
+        </is>
+      </c>
+      <c r="D43" s="6" t="n"/>
+      <c r="E43" s="6" t="n"/>
+      <c r="F43" s="6" t="n"/>
+      <c r="G43" s="6" t="n"/>
+      <c r="H43" s="6" t="n"/>
+      <c r="I43" s="6" t="n"/>
+      <c r="J43" s="6" t="n"/>
+      <c r="K43" s="6" t="inlineStr">
+        <is>
+          <t>شكراً لإخبارنا. يمكنك إعادة صياغة سؤالك، أو اختيار سؤال من القائمة.</t>
+        </is>
+      </c>
+      <c r="L43" s="6" t="n"/>
+      <c r="M43" s="6" t="n"/>
+      <c r="N43" s="6" t="n"/>
+      <c r="O43" s="6" t="inlineStr">
+        <is>
+          <t>لا</t>
+        </is>
+      </c>
+      <c r="P43" s="6" t="n"/>
+      <c r="Q43" s="6" t="inlineStr">
+        <is>
+          <t>مراجعة شرعية: لا</t>
+        </is>
+      </c>
+      <c r="R43" s="6" t="n"/>
+      <c r="S43" s="8" t="n"/>
+      <c r="T43" s="8" t="n"/>
+      <c r="U43" s="8" t="n"/>
+      <c r="V43" s="8" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>قالب</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="inlineStr">
+        <is>
+          <t>و-10</t>
+        </is>
+      </c>
+      <c r="C44" s="6" t="inlineStr">
+        <is>
+          <t>بعد «نعم»</t>
+        </is>
+      </c>
+      <c r="D44" s="6" t="n"/>
+      <c r="E44" s="6" t="n"/>
+      <c r="F44" s="6" t="n"/>
+      <c r="G44" s="6" t="n"/>
+      <c r="H44" s="6" t="n"/>
+      <c r="I44" s="6" t="n"/>
+      <c r="J44" s="6" t="n"/>
+      <c r="K44" s="6" t="inlineStr">
+        <is>
+          <t>قد يهمك بعدها:</t>
+        </is>
+      </c>
+      <c r="L44" s="6" t="n"/>
+      <c r="M44" s="6" t="n"/>
+      <c r="N44" s="6" t="n"/>
+      <c r="O44" s="6" t="inlineStr">
+        <is>
+          <t>لا</t>
+        </is>
+      </c>
+      <c r="P44" s="6" t="n"/>
+      <c r="Q44" s="6" t="inlineStr">
+        <is>
+          <t>مراجعة شرعية: لا</t>
+        </is>
+      </c>
+      <c r="R44" s="6" t="n"/>
+      <c r="S44" s="8" t="n"/>
+      <c r="T44" s="8" t="n"/>
+      <c r="U44" s="8" t="n"/>
+      <c r="V44" s="8" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>قالب</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="inlineStr">
+        <is>
+          <t>و-11</t>
+        </is>
+      </c>
+      <c r="C45" s="6" t="inlineStr">
+        <is>
+          <t>إدخال فارغ أو غير مفهوم</t>
+        </is>
+      </c>
+      <c r="D45" s="6" t="n"/>
+      <c r="E45" s="6" t="n"/>
+      <c r="F45" s="6" t="n"/>
+      <c r="G45" s="6" t="n"/>
+      <c r="H45" s="6" t="n"/>
+      <c r="I45" s="6" t="n"/>
+      <c r="J45" s="6" t="n"/>
+      <c r="K45" s="6" t="inlineStr">
+        <is>
+          <t>لم نتمكن من قراءة سؤالك. اكتب سؤالاً قصيراً عن القرآن، أو اختر من القائمة.</t>
+        </is>
+      </c>
+      <c r="L45" s="6" t="n"/>
+      <c r="M45" s="6" t="n"/>
+      <c r="N45" s="6" t="n"/>
+      <c r="O45" s="6" t="inlineStr">
+        <is>
+          <t>لا</t>
+        </is>
+      </c>
+      <c r="P45" s="6" t="n"/>
+      <c r="Q45" s="6" t="inlineStr">
+        <is>
+          <t>مراجعة شرعية: لا</t>
+        </is>
+      </c>
+      <c r="R45" s="6" t="n"/>
+      <c r="S45" s="8" t="n"/>
+      <c r="T45" s="8" t="n"/>
+      <c r="U45" s="8" t="n"/>
+      <c r="V45" s="8" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>قالب</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="inlineStr">
+        <is>
+          <t>و-12</t>
+        </is>
+      </c>
+      <c r="C46" s="6" t="inlineStr">
+        <is>
+          <t>ما بقي غير مغطى</t>
+        </is>
+      </c>
+      <c r="D46" s="6" t="n"/>
+      <c r="E46" s="6" t="n"/>
+      <c r="F46" s="6" t="n"/>
+      <c r="G46" s="6" t="n"/>
+      <c r="H46" s="6" t="n"/>
+      <c r="I46" s="6" t="n"/>
+      <c r="J46" s="6" t="n"/>
+      <c r="K46" s="6" t="inlineStr">
+        <is>
+          <t>لم نجد في مواد «دليل» جزءاً آخر يجيب عمّا بقي من سؤالك. نفضّل أن نخبرك بذلك على أن نعرض ما لا يجيب.</t>
+        </is>
+      </c>
+      <c r="L46" s="6" t="n"/>
+      <c r="M46" s="6" t="n"/>
+      <c r="N46" s="6" t="n"/>
+      <c r="O46" s="6" t="inlineStr">
+        <is>
+          <t>لا</t>
+        </is>
+      </c>
+      <c r="P46" s="6" t="n"/>
+      <c r="Q46" s="6" t="inlineStr">
+        <is>
+          <t>مراجعة شرعية: لا</t>
+        </is>
+      </c>
+      <c r="R46" s="6" t="n"/>
+      <c r="S46" s="8" t="n"/>
+      <c r="T46" s="8" t="n"/>
+      <c r="U46" s="8" t="n"/>
+      <c r="V46" s="8" t="n"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>قالب</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="inlineStr">
+        <is>
+          <t>و-13</t>
+        </is>
+      </c>
+      <c r="C47" s="6" t="inlineStr">
+        <is>
+          <t>آية مطابقة للمصحف</t>
+        </is>
+      </c>
+      <c r="D47" s="6" t="n"/>
+      <c r="E47" s="6" t="n"/>
+      <c r="F47" s="6" t="n"/>
+      <c r="G47" s="6" t="n"/>
+      <c r="H47" s="6" t="n"/>
+      <c r="I47" s="6" t="n"/>
+      <c r="J47" s="6" t="n"/>
+      <c r="K47" s="6" t="inlineStr">
+        <is>
+          <t>هذا نص الآية كما في المصحف:</t>
+        </is>
+      </c>
+      <c r="L47" s="6" t="n"/>
+      <c r="M47" s="6" t="n"/>
+      <c r="N47" s="6" t="n"/>
+      <c r="O47" s="6" t="inlineStr">
+        <is>
+          <t>لا</t>
+        </is>
+      </c>
+      <c r="P47" s="6" t="n"/>
+      <c r="Q47" s="6" t="inlineStr">
+        <is>
+          <t>مراجعة شرعية: لا</t>
+        </is>
+      </c>
+      <c r="R47" s="6" t="n"/>
+      <c r="S47" s="8" t="n"/>
+      <c r="T47" s="8" t="n"/>
+      <c r="U47" s="8" t="n"/>
+      <c r="V47" s="8" t="n"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>قالب</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="inlineStr">
+        <is>
+          <t>و-14</t>
+        </is>
+      </c>
+      <c r="C48" s="6" t="inlineStr">
+        <is>
+          <t>آية مكتوبة بنص مختلف</t>
+        </is>
+      </c>
+      <c r="D48" s="6" t="n"/>
+      <c r="E48" s="6" t="n"/>
+      <c r="F48" s="6" t="n"/>
+      <c r="G48" s="6" t="n"/>
+      <c r="H48" s="6" t="n"/>
+      <c r="I48" s="6" t="n"/>
+      <c r="J48" s="6" t="n"/>
+      <c r="K48" s="6" t="inlineStr">
+        <is>
+          <t>النص الذي كتبته يختلف عن نص المصحف. هذا نص الآية كما في المصحف:</t>
+        </is>
+      </c>
+      <c r="L48" s="6" t="n"/>
+      <c r="M48" s="6" t="n"/>
+      <c r="N48" s="6" t="n"/>
+      <c r="O48" s="6" t="inlineStr">
+        <is>
+          <t>لا</t>
+        </is>
+      </c>
+      <c r="P48" s="6" t="n"/>
+      <c r="Q48" s="6" t="inlineStr">
+        <is>
+          <t>مراجعة شرعية: نعم</t>
+        </is>
+      </c>
+      <c r="R48" s="6" t="n"/>
+      <c r="S48" s="8" t="n"/>
+      <c r="T48" s="8" t="n"/>
+      <c r="U48" s="8" t="n"/>
+      <c r="V48" s="8" t="n"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>قالب</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="inlineStr">
+        <is>
+          <t>و-15</t>
+        </is>
+      </c>
+      <c r="C49" s="6" t="inlineStr">
+        <is>
+          <t>أسفل كل مقطع</t>
+        </is>
+      </c>
+      <c r="D49" s="6" t="n"/>
+      <c r="E49" s="6" t="n"/>
+      <c r="F49" s="6" t="n"/>
+      <c r="G49" s="6" t="n"/>
+      <c r="H49" s="6" t="n"/>
+      <c r="I49" s="6" t="n"/>
+      <c r="J49" s="6" t="n"/>
+      <c r="K49" s="6" t="inlineStr">
+        <is>
+          <t>لا يتجاوز «دليل» هذا النص المقتبس، ولا يضيف إليه شرحاً من عنده.</t>
+        </is>
+      </c>
+      <c r="L49" s="6" t="n"/>
+      <c r="M49" s="6" t="n"/>
+      <c r="N49" s="6" t="n"/>
+      <c r="O49" s="6" t="inlineStr">
+        <is>
+          <t>لا</t>
+        </is>
+      </c>
+      <c r="P49" s="6" t="n"/>
+      <c r="Q49" s="6" t="inlineStr">
+        <is>
+          <t>مراجعة شرعية: لا</t>
+        </is>
+      </c>
+      <c r="R49" s="6" t="n"/>
+      <c r="S49" s="8" t="n"/>
+      <c r="T49" s="8" t="n"/>
+      <c r="U49" s="8" t="n"/>
+      <c r="V49" s="8" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:V42"/>
+  <autoFilter ref="A1:V49"/>
   <conditionalFormatting sqref="O2:O300">
     <cfRule type="expression" priority="1" dxfId="1">
       <formula>$O2="نعم"</formula>
     </cfRule>
+    <cfRule type="expression" priority="2" dxfId="1">
+      <formula>$O2="نعم"</formula>
+    </cfRule>
   </conditionalFormatting>
-  <dataValidations count="2">
+  <dataValidations count="4">
+    <dataValidation sqref="S2:S300" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"معتمد,معتمد بتعديل,مرفوض"</formula1>
+    </dataValidation>
+    <dataValidation sqref="V2:V300" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"موافق,موافق بتعديل,غير موافق"</formula1>
+    </dataValidation>
     <dataValidation sqref="S2:S300" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"معتمد,معتمد بتعديل,مرفوض"</formula1>
     </dataValidation>
@@ -4875,7 +5536,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F10"/>
+  <dimension ref="A1:F2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -4921,255 +5582,39 @@
     <row r="2" ht="34" customHeight="1">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>ق-05</t>
+          <t>ق-18</t>
         </is>
       </c>
       <c r="B2" s="5" t="inlineStr">
         <is>
-          <t>ح5</t>
+          <t>ح6</t>
         </is>
       </c>
       <c r="C2" s="6" t="inlineStr">
         <is>
-          <t>أساسي</t>
+          <t>إضافي</t>
         </is>
       </c>
       <c r="D2" s="6" t="inlineStr">
         <is>
-          <t>التوحيد وعبادة الله: الرسالة المحورية للقرآن</t>
+          <t>من أين يبدأ المبتدئ القراءة</t>
         </is>
       </c>
       <c r="E2" s="6" t="inlineStr">
         <is>
-          <t>كتاب في علوم القرآن (quranpedia) أو الدرر — يُحدد</t>
+          <t>لم يُعثر عليه في كتاب القطان؛ يُبحث في الدرر أو بينات</t>
         </is>
       </c>
       <c r="F2" s="6" t="n"/>
     </row>
-    <row r="3" ht="34" customHeight="1">
-      <c r="A3" s="5" t="inlineStr">
-        <is>
-          <t>ق-06</t>
-        </is>
-      </c>
-      <c r="B3" s="5" t="inlineStr">
-        <is>
-          <t>ح5</t>
-        </is>
-      </c>
-      <c r="C3" s="6" t="inlineStr">
-        <is>
-          <t>أساسي</t>
-        </is>
-      </c>
-      <c r="D3" s="6" t="inlineStr">
-        <is>
-          <t>الأنبياء وقصصهم في القرآن</t>
-        </is>
-      </c>
-      <c r="E3" s="6" t="inlineStr">
-        <is>
-          <t>كتاب في علوم القرآن (quranpedia) أو الدرر — يُحدد</t>
-        </is>
-      </c>
-      <c r="F3" s="6" t="n"/>
-    </row>
-    <row r="4" ht="34" customHeight="1">
-      <c r="A4" s="5" t="inlineStr">
-        <is>
-          <t>ق-07</t>
-        </is>
-      </c>
-      <c r="B4" s="5" t="inlineStr">
-        <is>
-          <t>ح5</t>
-        </is>
-      </c>
-      <c r="C4" s="6" t="inlineStr">
-        <is>
-          <t>أساسي</t>
-        </is>
-      </c>
-      <c r="D4" s="6" t="inlineStr">
-        <is>
-          <t>اليوم الآخر والقيم في القرآن إجمالاً</t>
-        </is>
-      </c>
-      <c r="E4" s="6" t="inlineStr">
-        <is>
-          <t>كتاب في علوم القرآن (quranpedia) أو الدرر — يُحدد</t>
-        </is>
-      </c>
-      <c r="F4" s="6" t="n"/>
-    </row>
-    <row r="5" ht="34" customHeight="1">
-      <c r="A5" s="5" t="inlineStr">
-        <is>
-          <t>ق-10</t>
-        </is>
-      </c>
-      <c r="B5" s="5" t="inlineStr">
-        <is>
-          <t>ح2</t>
-        </is>
-      </c>
-      <c r="C5" s="6" t="inlineStr">
-        <is>
-          <t>أساسي</t>
-        </is>
-      </c>
-      <c r="D5" s="6" t="inlineStr">
-        <is>
-          <t>المكي والمدني</t>
-        </is>
-      </c>
-      <c r="E5" s="6" t="inlineStr">
-        <is>
-          <t>كتاب في علوم القرآن (quranpedia) — يُحدد</t>
-        </is>
-      </c>
-      <c r="F5" s="6" t="n"/>
-    </row>
-    <row r="6" ht="34" customHeight="1">
-      <c r="A6" s="5" t="inlineStr">
-        <is>
-          <t>ق-15</t>
-        </is>
-      </c>
-      <c r="B6" s="5" t="inlineStr">
-        <is>
-          <t>ح4</t>
-        </is>
-      </c>
-      <c r="C6" s="6" t="inlineStr">
-        <is>
-          <t>أساسي</t>
-        </is>
-      </c>
-      <c r="D6" s="6" t="inlineStr">
-        <is>
-          <t>السورة والآية، وعدد سور القرآن</t>
-        </is>
-      </c>
-      <c r="E6" s="6" t="inlineStr">
-        <is>
-          <t>كتاب في علوم القرآن (quranpedia) — يُحدد</t>
-        </is>
-      </c>
-      <c r="F6" s="6" t="n"/>
-    </row>
-    <row r="7" ht="34" customHeight="1">
-      <c r="A7" s="5" t="inlineStr">
-        <is>
-          <t>ق-16</t>
-        </is>
-      </c>
-      <c r="B7" s="5" t="inlineStr">
-        <is>
-          <t>ح4</t>
-        </is>
-      </c>
-      <c r="C7" s="6" t="inlineStr">
-        <is>
-          <t>أساسي</t>
-        </is>
-      </c>
-      <c r="D7" s="6" t="inlineStr">
-        <is>
-          <t>كيف أصل إلى سورة وآية في المصحف</t>
-        </is>
-      </c>
-      <c r="E7" s="6" t="inlineStr">
-        <is>
-          <t>كتاب في علوم القرآن (quranpedia) — يُحدد</t>
-        </is>
-      </c>
-      <c r="F7" s="6" t="n"/>
-    </row>
-    <row r="8" ht="34" customHeight="1">
-      <c r="A8" s="5" t="inlineStr">
-        <is>
-          <t>ق-19</t>
-        </is>
-      </c>
-      <c r="B8" s="5" t="inlineStr">
-        <is>
-          <t>ح6</t>
-        </is>
-      </c>
-      <c r="C8" s="6" t="inlineStr">
-        <is>
-          <t>أساسي</t>
-        </is>
-      </c>
-      <c r="D8" s="6" t="inlineStr">
-        <is>
-          <t>فهم المعنى بتفسير مختصر موثوق</t>
-        </is>
-      </c>
-      <c r="E8" s="6" t="inlineStr">
-        <is>
-          <t>الدرر أو كتاب في علوم القرآن — يُحدد</t>
-        </is>
-      </c>
-      <c r="F8" s="6" t="n"/>
-    </row>
-    <row r="9" ht="34" customHeight="1">
-      <c r="A9" s="5" t="inlineStr">
-        <is>
-          <t>ق-20</t>
-        </is>
-      </c>
-      <c r="B9" s="5" t="inlineStr">
-        <is>
-          <t>ح6</t>
-        </is>
-      </c>
-      <c r="C9" s="6" t="inlineStr">
-        <is>
-          <t>أساسي</t>
-        </is>
-      </c>
-      <c r="D9" s="6" t="inlineStr">
-        <is>
-          <t>الفرق بين نص القرآن وتفسيره وترجمة معانيه</t>
-        </is>
-      </c>
-      <c r="E9" s="6" t="inlineStr">
-        <is>
-          <t>الدرر أو كتاب في علوم القرآن — يُحدد</t>
-        </is>
-      </c>
-      <c r="F9" s="6" t="n"/>
-    </row>
-    <row r="10" ht="34" customHeight="1">
-      <c r="A10" s="5" t="inlineStr">
-        <is>
-          <t>ق-18</t>
-        </is>
-      </c>
-      <c r="B10" s="5" t="inlineStr">
-        <is>
-          <t>ح6</t>
-        </is>
-      </c>
-      <c r="C10" s="6" t="inlineStr">
-        <is>
-          <t>إضافي</t>
-        </is>
-      </c>
-      <c r="D10" s="6" t="inlineStr">
-        <is>
-          <t>من أين يبدأ المبتدئ القراءة</t>
-        </is>
-      </c>
-      <c r="E10" s="6" t="inlineStr">
-        <is>
-          <t>الدرر أو كتاب في علوم القرآن — يُحدد</t>
-        </is>
-      </c>
-      <c r="F10" s="6" t="n"/>
-    </row>
+    <row r="3" ht="34" customHeight="1"/>
+    <row r="4" ht="34" customHeight="1"/>
+    <row r="5" ht="34" customHeight="1"/>
+    <row r="6" ht="34" customHeight="1"/>
+    <row r="7" ht="34" customHeight="1"/>
+    <row r="8" ht="34" customHeight="1"/>
+    <row r="9" ht="34" customHeight="1"/>
+    <row r="10" ht="34" customHeight="1"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -5241,7 +5686,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:G6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -5372,7 +5817,7 @@
       </c>
       <c r="B4" s="8" t="inlineStr">
         <is>
-          <t>[كتاب مختصر في علوم القرآن — يُحدد]</t>
+          <t>مباحث في علوم القرآن، مناع القطان</t>
         </is>
       </c>
       <c r="C4" s="6" t="inlineStr">
@@ -5382,7 +5827,7 @@
       </c>
       <c r="D4" s="8" t="inlineStr">
         <is>
-          <t>[الرابط]</t>
+          <t>https://quranpedia.net/book/23563</t>
         </is>
       </c>
       <c r="E4" s="6" t="inlineStr">
@@ -5390,65 +5835,73 @@
           <t>معروضة</t>
         </is>
       </c>
-      <c r="F4" s="8" t="n"/>
+      <c r="F4" s="8" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
       <c r="G4" s="6" t="inlineStr">
         <is>
-          <t>ح2 ح4</t>
+          <t>ح2 ح4 ح5 ح6</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
         <is>
-          <t>م-04</t>
+          <t>ت-01</t>
         </is>
       </c>
       <c r="B5" s="8" t="inlineStr">
         <is>
-          <t>[مادة للبدء بالقراءة والفهم — يُحدد]</t>
+          <t>مصحف مجمع الملك فهد (نص الآيات)</t>
         </is>
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>الدرر أو الجمهرة</t>
+          <t>مجمع الملك فهد</t>
         </is>
       </c>
       <c r="D5" s="8" t="inlineStr">
         <is>
-          <t>[الرابط]</t>
+          <t>https://quranpedia.net</t>
         </is>
       </c>
       <c r="E5" s="6" t="inlineStr">
         <is>
-          <t>معروضة</t>
-        </is>
-      </c>
-      <c r="F5" s="8" t="n"/>
+          <t>تحقق فقط</t>
+        </is>
+      </c>
+      <c r="F5" s="8" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
       <c r="G5" s="6" t="inlineStr">
         <is>
-          <t>ح5 ح6</t>
+          <t>كل الحاجات</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
         <is>
-          <t>ت-01</t>
+          <t>ت-02</t>
         </is>
       </c>
       <c r="B6" s="8" t="inlineStr">
         <is>
-          <t>مصحف مجمع الملك فهد (نص الآيات)</t>
+          <t>الموسوعة الحديثية</t>
         </is>
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>مجمع الملك فهد</t>
+          <t>الدرر السنية</t>
         </is>
       </c>
       <c r="D6" s="8" t="inlineStr">
         <is>
-          <t>https://quranpedia.net</t>
+          <t>https://dorar.net/hadith</t>
         </is>
       </c>
       <c r="E6" s="6" t="inlineStr">
@@ -5462,43 +5915,6 @@
         </is>
       </c>
       <c r="G6" s="6" t="inlineStr">
-        <is>
-          <t>كل الحاجات</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="6" t="inlineStr">
-        <is>
-          <t>ت-02</t>
-        </is>
-      </c>
-      <c r="B7" s="8" t="inlineStr">
-        <is>
-          <t>الموسوعة الحديثية</t>
-        </is>
-      </c>
-      <c r="C7" s="6" t="inlineStr">
-        <is>
-          <t>الدرر السنية</t>
-        </is>
-      </c>
-      <c r="D7" s="8" t="inlineStr">
-        <is>
-          <t>https://dorar.net/hadith</t>
-        </is>
-      </c>
-      <c r="E7" s="6" t="inlineStr">
-        <is>
-          <t>تحقق فقط</t>
-        </is>
-      </c>
-      <c r="F7" s="8" t="inlineStr">
-        <is>
-          <t>نعم</t>
-        </is>
-      </c>
-      <c r="G7" s="6" t="inlineStr">
         <is>
           <t>كل الحاجات</t>
         </is>

</xml_diff>

<commit_message>
Show only the sentences that answer the question (verbatim, with a full-text toggle) and link tafsir requests to al-Muyassar on quran.com
- app/units.py splits each approved passage into sentences that join back to the exact text
- app/focus.py: the model picks sentence numbers only; falls back to the full passage on any error, when >75% is selected, or for passages marked «لا يُجتزأ»
- tafsir abstentions and pasted verses get a link to al-Muyassar for that verse (new template ام-11 in review)
- evaluation reports how often answers are focused and how much of the text is shown

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RkXtRf8o9rcFbV2XzFoBFz
</commit_message>
<xml_diff>
--- a/data/register.xlsx
+++ b/data/register.xlsx
@@ -660,7 +660,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V49"/>
+  <dimension ref="A1:W50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -685,6 +685,7 @@
     <col width="36" customWidth="1" min="20" max="20"/>
     <col width="18" customWidth="1" min="21" max="21"/>
     <col width="14" customWidth="1" min="22" max="22"/>
+    <col width="10" customWidth="1" min="23" max="23"/>
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
@@ -796,6 +797,11 @@
       <c r="V1" s="4" t="inlineStr">
         <is>
           <t>رأي المختص الأعلم</t>
+        </is>
+      </c>
+      <c r="W1" s="4" t="inlineStr">
+        <is>
+          <t>لا يُجتزأ</t>
         </is>
       </c>
     </row>
@@ -2255,6 +2261,11 @@
       <c r="T18" s="8" t="n"/>
       <c r="U18" s="8" t="n"/>
       <c r="V18" s="8" t="n"/>
+      <c r="W18" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="150" customHeight="1">
       <c r="A19" s="5" t="inlineStr">
@@ -3837,6 +3848,51 @@
       <c r="T49" s="8" t="n"/>
       <c r="U49" s="8" t="n"/>
       <c r="V49" s="8" t="n"/>
+    </row>
+    <row r="50" ht="34" customHeight="1">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>قالب</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="inlineStr">
+        <is>
+          <t>ام-11</t>
+        </is>
+      </c>
+      <c r="C50" s="6" t="inlineStr">
+        <is>
+          <t>زر تحت الامتناع عن تفسير آية بعينها، أو تحت آية كتبها المستخدم</t>
+        </is>
+      </c>
+      <c r="D50" s="6" t="n"/>
+      <c r="E50" s="6" t="n"/>
+      <c r="F50" s="6" t="n"/>
+      <c r="G50" s="6" t="n"/>
+      <c r="H50" s="6" t="n"/>
+      <c r="I50" s="6" t="n"/>
+      <c r="J50" s="6" t="n"/>
+      <c r="K50" s="6" t="inlineStr">
+        <is>
+          <t>اقرأ معنى {الموضع} في «التفسير الميسر» (مجمع الملك فهد) على منصة القرآن الكريم</t>
+        </is>
+      </c>
+      <c r="L50" s="6" t="n"/>
+      <c r="M50" s="6" t="n"/>
+      <c r="N50" s="6" t="n"/>
+      <c r="O50" s="6" t="n"/>
+      <c r="P50" s="6" t="n"/>
+      <c r="Q50" s="6" t="inlineStr">
+        <is>
+          <t>يُحيل إلى صفحة التفسير الميسر للآية على quran.com ولا يعرض تفسيراً داخل «دليل». مراجعة شرعية: نعم (اختيار التفسير المُحال إليه).</t>
+        </is>
+      </c>
+      <c r="R50" s="6" t="n"/>
+      <c r="S50" s="6" t="n"/>
+      <c r="T50" s="6" t="n"/>
+      <c r="U50" s="6" t="n"/>
+      <c r="V50" s="6" t="n"/>
+      <c r="W50" s="6" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:V49"/>
@@ -3848,7 +3904,7 @@
       <formula>$O2="نعم"</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="4">
+  <dataValidations count="5">
     <dataValidation sqref="S2:S300" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"معتمد,معتمد بتعديل,مرفوض"</formula1>
     </dataValidation>
@@ -3861,6 +3917,9 @@
     <dataValidation sqref="V2:V300" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"موافق,موافق بتعديل,غير موافق"</formula1>
     </dataValidation>
+    <dataValidation sqref="W2:W300" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"نعم,لا"</formula1>
+    </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3872,7 +3931,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S16"/>
+  <dimension ref="A1:T16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -3894,6 +3953,7 @@
     <col width="14" customWidth="1" min="17" max="17"/>
     <col width="40" customWidth="1" min="18" max="18"/>
     <col width="16" customWidth="1" min="19" max="19"/>
+    <col width="10" customWidth="1" min="20" max="20"/>
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
@@ -3990,6 +4050,11 @@
       <c r="S1" s="4" t="inlineStr">
         <is>
           <t>صالح للنشر</t>
+        </is>
+      </c>
+      <c r="T1" s="4" t="inlineStr">
+        <is>
+          <t>لا يُجتزأ</t>
         </is>
       </c>
     </row>
@@ -5467,6 +5532,11 @@
       <formula>$N2="نعم"</formula>
     </cfRule>
   </conditionalFormatting>
+  <dataValidations count="1">
+    <dataValidation sqref="T2:T300" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"نعم,لا"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Fix wrong menu answers, separate unrelated questions, honest labels and safer requests
- menu buttons answer only with a core passage (or one named in «مقطع الزر»); needs without one show as «قيد المراجعة»
- gate: a passage from another need is not an answer unless fit is high; clarify never offers an uncovered need
- non-religious questions get their own message (ام-12, in review) instead of a referral to a sharia source
- page: shows which question the result belongs to, drops stale responses, offers retry, says «المتعلق بسؤالك», examples that pass the tests
- scripts/coverage.py writes eval/coverage.md; regression tests for all of the above; dev cases d36–d37

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RkXtRf8o9rcFbV2XzFoBFz
</commit_message>
<xml_diff>
--- a/data/register.xlsx
+++ b/data/register.xlsx
@@ -227,6 +227,21 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>دليل</author>
+  </authors>
+  <commentList>
+    <comment ref="J1" authorId="0" shapeId="0">
+      <text>
+        <t>اختياري: رقم المقطع (أو أكثر، مثل ق-01 ق-02) الذي يُعرض عند الضغط على زر هذه الحاجة. إن تُرك فارغاً يُعرض أول مقطع «أساسي» منشور، ويختفي الزر إن لم يوجد.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -660,7 +675,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W50"/>
+  <dimension ref="A1:W51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -3893,6 +3908,51 @@
       <c r="U50" s="6" t="n"/>
       <c r="V50" s="6" t="n"/>
       <c r="W50" s="6" t="n"/>
+    </row>
+    <row r="51" ht="34" customHeight="1">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>قالب</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="inlineStr">
+        <is>
+          <t>ام-12</t>
+        </is>
+      </c>
+      <c r="C51" s="6" t="inlineStr">
+        <is>
+          <t>سؤال لا علاقة له بالدين (طبخ، رياضة، معلومات عامة)</t>
+        </is>
+      </c>
+      <c r="D51" s="6" t="n"/>
+      <c r="E51" s="6" t="n"/>
+      <c r="F51" s="6" t="n"/>
+      <c r="G51" s="6" t="n"/>
+      <c r="H51" s="6" t="n"/>
+      <c r="I51" s="6" t="n"/>
+      <c r="J51" s="6" t="n"/>
+      <c r="K51" s="6" t="inlineStr">
+        <is>
+          <t>«دليل» مختص بالأسئلة عن القرآن الكريم، وسؤالك خارج هذا المجال. جرّب أن تسأل عن القرآن، أو اختر من الأسئلة أدناه.</t>
+        </is>
+      </c>
+      <c r="L51" s="6" t="n"/>
+      <c r="M51" s="6" t="n"/>
+      <c r="N51" s="6" t="n"/>
+      <c r="O51" s="6" t="n"/>
+      <c r="P51" s="6" t="n"/>
+      <c r="Q51" s="6" t="inlineStr">
+        <is>
+          <t>بديل عن ام-01 للأسئلة غير الدينية، حتى لا يُحال سؤال الطبخ إلى مرجع شرعي. مراجعة شرعية: لا.</t>
+        </is>
+      </c>
+      <c r="R51" s="6" t="n"/>
+      <c r="S51" s="6" t="n"/>
+      <c r="T51" s="6" t="n"/>
+      <c r="U51" s="6" t="n"/>
+      <c r="V51" s="6" t="n"/>
+      <c r="W51" s="6" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:V49"/>
@@ -6001,7 +6061,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I8"/>
+  <dimension ref="A1:J8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -6013,6 +6073,7 @@
     <col width="11" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -6061,6 +6122,11 @@
           <t>التغطية</t>
         </is>
       </c>
+      <c r="J1" s="4" t="inlineStr">
+        <is>
+          <t>مقطع الزر</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="6" t="inlineStr">
@@ -6105,6 +6171,7 @@
         <f>IF(H2=0,"لا تغطية",IF(H2&lt;G2,"جزئية","مكتملة"))</f>
         <v/>
       </c>
+      <c r="J2" s="7" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
@@ -6149,6 +6216,7 @@
         <f>IF(H3=0,"لا تغطية",IF(H3&lt;G3,"جزئية","مكتملة"))</f>
         <v/>
       </c>
+      <c r="J3" s="7" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
@@ -6193,6 +6261,7 @@
         <f>IF(H4=0,"لا تغطية",IF(H4&lt;G4,"جزئية","مكتملة"))</f>
         <v/>
       </c>
+      <c r="J4" s="7" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
@@ -6237,6 +6306,7 @@
         <f>IF(H5=0,"لا تغطية",IF(H5&lt;G5,"جزئية","مكتملة"))</f>
         <v/>
       </c>
+      <c r="J5" s="7" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
@@ -6281,6 +6351,7 @@
         <f>IF(H6=0,"لا تغطية",IF(H6&lt;G6,"جزئية","مكتملة"))</f>
         <v/>
       </c>
+      <c r="J6" s="7" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
@@ -6325,6 +6396,7 @@
         <f>IF(H7=0,"لا تغطية",IF(H7&lt;G7,"جزئية","مكتملة"))</f>
         <v/>
       </c>
+      <c r="J7" s="7" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
@@ -6369,9 +6441,11 @@
         <f>IF(H8=0,"لا تغطية",IF(H8&lt;G8,"جزئية","مكتملة"))</f>
         <v/>
       </c>
+      <c r="J8" s="7" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Matching method: near-miss questions per passage, a check of the passage text after routing, and tests built from the register
- register: «أسئلة قريبة لا يجيب عنها» per passage (drafts for all 34 passages); the router sees them
- after routing, the same call that selects sentences rates each passage answers / partial / none; none is dropped (abstain if nothing remains), partial is labelled «مقطع متعلق بسؤالك»; on error the router's choice stands
- eval set «register»: every phrasing must reach its passage, every near-miss must not; built at run time, so each new passage brings its own tests

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RkXtRf8o9rcFbV2XzFoBFz
</commit_message>
<xml_diff>
--- a/data/register.xlsx
+++ b/data/register.xlsx
@@ -230,6 +230,36 @@
 </file>
 
 <file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>دليل</author>
+  </authors>
+  <commentList>
+    <comment ref="X1" authorId="0" shapeId="0">
+      <text>
+        <t>أسئلة قريبة من موضوع المقطع لا يجيب عنها، تفصل بينها «|». يراها الموجِّه فلا يختار المقطع لها، وتُبنى منها حالات اختبار. مسودة بمساعدة الذكاء الاصطناعي.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments/comment2.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>دليل</author>
+  </authors>
+  <commentList>
+    <comment ref="U1" authorId="0" shapeId="0">
+      <text>
+        <t>أسئلة قريبة من موضوع المقطع لا يجيب عنها، تفصل بينها «|». يراها الموجِّه فلا يختار المقطع لها، وتُبنى منها حالات اختبار. مسودة بمساعدة الذكاء الاصطناعي.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments/comment3.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
     <author>دليل</author>
@@ -675,7 +705,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W51"/>
+  <dimension ref="A1:X51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -701,6 +731,7 @@
     <col width="18" customWidth="1" min="21" max="21"/>
     <col width="14" customWidth="1" min="22" max="22"/>
     <col width="10" customWidth="1" min="23" max="23"/>
+    <col width="34" customWidth="1" min="24" max="24"/>
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
@@ -817,6 +848,11 @@
       <c r="W1" s="4" t="inlineStr">
         <is>
           <t>لا يُجتزأ</t>
+        </is>
+      </c>
+      <c r="X1" s="4" t="inlineStr">
+        <is>
+          <t>أسئلة قريبة لا يجيب عنها</t>
         </is>
       </c>
     </row>
@@ -899,6 +935,11 @@
       <c r="T2" s="8" t="n"/>
       <c r="U2" s="8" t="n"/>
       <c r="V2" s="8" t="n"/>
+      <c r="X2" s="8" t="inlineStr">
+        <is>
+          <t>لماذا يعظّم المسلمون القرآن؟ | هل القرآن من تأليف محمد؟ | ما معنى كلمة قرآن في اللغة؟</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="150" customHeight="1">
       <c r="A3" s="5" t="inlineStr">
@@ -982,6 +1023,11 @@
       <c r="T3" s="8" t="n"/>
       <c r="U3" s="8" t="n"/>
       <c r="V3" s="8" t="n"/>
+      <c r="X3" s="8" t="inlineStr">
+        <is>
+          <t>ما تعريف القرآن؟ | ما فضل قراءة القرآن؟</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="150" customHeight="1">
       <c r="A4" s="5" t="inlineStr">
@@ -1071,6 +1117,11 @@
       <c r="T4" s="8" t="n"/>
       <c r="U4" s="8" t="n"/>
       <c r="V4" s="8" t="n"/>
+      <c r="X4" s="8" t="inlineStr">
+        <is>
+          <t>هل نقل محمد القرآن من التوراة؟ | ما الفرق بين القرآن والحديث؟</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="150" customHeight="1">
       <c r="A5" s="5" t="inlineStr">
@@ -1151,6 +1202,11 @@
       <c r="T5" s="8" t="n"/>
       <c r="U5" s="8" t="n"/>
       <c r="V5" s="8" t="n"/>
+      <c r="X5" s="8" t="inlineStr">
+        <is>
+          <t>ما تعريف القرآن اصطلاحاً؟ | ما أسماء القرآن الأخرى؟</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="150" customHeight="1">
       <c r="A6" s="5" t="inlineStr">
@@ -1234,6 +1290,11 @@
       <c r="T6" s="8" t="n"/>
       <c r="U6" s="8" t="n"/>
       <c r="V6" s="8" t="n"/>
+      <c r="X6" s="8" t="inlineStr">
+        <is>
+          <t>هل السنة حجة؟ | ما تعريف القرآن؟</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="150" customHeight="1">
       <c r="A7" s="5" t="inlineStr">
@@ -1316,6 +1377,11 @@
       <c r="T7" s="8" t="n"/>
       <c r="U7" s="8" t="n"/>
       <c r="V7" s="8" t="n"/>
+      <c r="X7" s="8" t="inlineStr">
+        <is>
+          <t>في أي شهر نزل القرآن؟ | لماذا لم ير الناس جبريل؟ | هل نزل القرآن مرة واحدة؟</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="150" customHeight="1">
       <c r="A8" s="5" t="inlineStr">
@@ -1398,6 +1464,11 @@
       <c r="T8" s="8" t="n"/>
       <c r="U8" s="8" t="n"/>
       <c r="V8" s="8" t="n"/>
+      <c r="X8" s="8" t="inlineStr">
+        <is>
+          <t>كيف كان الوحي يأتي النبي؟ | هل نزل القرآن مرة واحدة؟ | ما فضل شهر رمضان؟</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="150" customHeight="1">
       <c r="A9" s="5" t="inlineStr">
@@ -1478,6 +1549,11 @@
       <c r="T9" s="8" t="n"/>
       <c r="U9" s="8" t="n"/>
       <c r="V9" s="8" t="n"/>
+      <c r="X9" s="8" t="inlineStr">
+        <is>
+          <t>في أي شهر نزل القرآن؟ | كيف كان الوحي يأتي النبي؟</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="150" customHeight="1">
       <c r="A10" s="5" t="inlineStr">
@@ -1563,6 +1639,11 @@
       <c r="T10" s="8" t="n"/>
       <c r="U10" s="8" t="n"/>
       <c r="V10" s="8" t="n"/>
+      <c r="X10" s="8" t="inlineStr">
+        <is>
+          <t>كيف كان الوحي ينزل؟ | من رتّب سور القرآن؟</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="150" customHeight="1">
       <c r="A11" s="5" t="inlineStr">
@@ -1650,6 +1731,11 @@
       <c r="T11" s="8" t="n"/>
       <c r="U11" s="8" t="n"/>
       <c r="V11" s="8" t="n"/>
+      <c r="X11" s="8" t="inlineStr">
+        <is>
+          <t>لماذا جمع عثمان القرآن؟ | كم عدد حفّاظ القرآن اليوم؟</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="150" customHeight="1">
       <c r="A12" s="5" t="inlineStr">
@@ -1732,6 +1818,11 @@
       <c r="T12" s="8" t="n"/>
       <c r="U12" s="8" t="n"/>
       <c r="V12" s="8" t="n"/>
+      <c r="X12" s="8" t="inlineStr">
+        <is>
+          <t>كيف أبدأ قراءة القرآن؟ | ما حكم قراءة القرآن للحائض؟</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="150" customHeight="1">
       <c r="A13" s="5" t="inlineStr">
@@ -1814,6 +1905,11 @@
       <c r="T13" s="8" t="n"/>
       <c r="U13" s="8" t="n"/>
       <c r="V13" s="8" t="n"/>
+      <c r="X13" s="8" t="inlineStr">
+        <is>
+          <t>أين أتعلم القرآن؟ | ما أحكام التجويد؟</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="150" customHeight="1">
       <c r="A14" s="5" t="inlineStr">
@@ -1904,6 +2000,11 @@
       <c r="T14" s="8" t="n"/>
       <c r="U14" s="8" t="n"/>
       <c r="V14" s="8" t="n"/>
+      <c r="X14" s="8" t="inlineStr">
+        <is>
+          <t>ما الفرق بين أسلوب السور المكية والمدنية؟ | في أي شهر نزل القرآن؟</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="150" customHeight="1">
       <c r="A15" s="5" t="inlineStr">
@@ -1994,6 +2095,11 @@
       <c r="T15" s="8" t="n"/>
       <c r="U15" s="8" t="n"/>
       <c r="V15" s="8" t="n"/>
+      <c r="X15" s="8" t="inlineStr">
+        <is>
+          <t>ما قصة يوسف عليه السلام؟ | ما تفسير سورة الفاتحة؟</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="150" customHeight="1">
       <c r="A16" s="5" t="inlineStr">
@@ -2088,6 +2194,11 @@
       <c r="T16" s="8" t="n"/>
       <c r="U16" s="8" t="n"/>
       <c r="V16" s="8" t="n"/>
+      <c r="X16" s="8" t="inlineStr">
+        <is>
+          <t>ما قصة نوح بالتفصيل؟ | هل قصص القرآن منقولة من التوراة؟</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="150" customHeight="1">
       <c r="A17" s="5" t="inlineStr">
@@ -2181,6 +2292,11 @@
       <c r="T17" s="8" t="n"/>
       <c r="U17" s="8" t="n"/>
       <c r="V17" s="8" t="n"/>
+      <c r="X17" s="8" t="inlineStr">
+        <is>
+          <t>من رتّب سور القرآن؟ | كيف أجد آية في المصحف؟</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="150" customHeight="1">
       <c r="A18" s="5" t="inlineStr">
@@ -2281,6 +2397,11 @@
           <t>نعم</t>
         </is>
       </c>
+      <c r="X18" s="8" t="inlineStr">
+        <is>
+          <t>كم عدد سور القرآن؟ | لماذا تتنقل السورة بين موضوعات مختلفة؟</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="150" customHeight="1">
       <c r="A19" s="5" t="inlineStr">
@@ -2373,6 +2494,11 @@
       <c r="T19" s="8" t="n"/>
       <c r="U19" s="8" t="n"/>
       <c r="V19" s="8" t="n"/>
+      <c r="X19" s="8" t="inlineStr">
+        <is>
+          <t>ما تفسير آية الكرسي؟ | ما أفضل تفسير للمبتدئ؟</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="150" customHeight="1">
       <c r="A20" s="5" t="inlineStr">
@@ -2471,6 +2597,11 @@
       <c r="T20" s="8" t="n"/>
       <c r="U20" s="8" t="n"/>
       <c r="V20" s="8" t="n"/>
+      <c r="X20" s="8" t="inlineStr">
+        <is>
+          <t>هل تجوز الصلاة بترجمة القرآن؟ | ما أفضل ترجمة للقرآن؟</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="48" customHeight="1">
       <c r="A21" s="5" t="inlineStr">
@@ -3982,6 +4113,7 @@
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 
@@ -3991,7 +4123,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T16"/>
+  <dimension ref="A1:U16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -4014,6 +4146,7 @@
     <col width="40" customWidth="1" min="18" max="18"/>
     <col width="16" customWidth="1" min="19" max="19"/>
     <col width="10" customWidth="1" min="20" max="20"/>
+    <col width="34" customWidth="1" min="21" max="21"/>
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
@@ -4117,6 +4250,11 @@
           <t>لا يُجتزأ</t>
         </is>
       </c>
+      <c r="U1" s="4" t="inlineStr">
+        <is>
+          <t>أسئلة قريبة لا يجيب عنها</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="150" customHeight="1">
       <c r="A2" s="5" t="inlineStr">
@@ -4213,6 +4351,11 @@
         <f>IF(A2="","",IF(OR(M2="ج",M2="د"),"المستوى لا يُنشر",IF(IFERROR(INDEX(المصادر!$F$2:$F$30,MATCH(D2,المصادر!$A$2:$A$30,0)),"")&lt;&gt;"نعم","المصدر غير معتمد",IF(OR(B2="",E2="",J2="",K2="",P2=""),"بيانات ناقصة",IF(AND(N2="نعم",Q2&lt;&gt;"موافق"),"ينقصه رأي المختص","صالح للنشر")))))</f>
         <v/>
       </c>
+      <c r="U2" s="7" t="inlineStr">
+        <is>
+          <t>ما علاقة القرآن بالكتب السابقة؟ | ما تعريف القرآن؟ | ما مكانة القرآن عند المسلمين؟</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="150" customHeight="1">
       <c r="A3" s="5" t="inlineStr">
@@ -4304,6 +4447,11 @@
       <c r="S3" s="7">
         <f>IF(A3="","",IF(OR(M3="ج",M3="د"),"المستوى لا يُنشر",IF(IFERROR(INDEX(المصادر!$F$2:$F$30,MATCH(D3,المصادر!$A$2:$A$30,0)),"")&lt;&gt;"نعم","المصدر غير معتمد",IF(OR(B3="",E3="",J3="",K3="",P3=""),"بيانات ناقصة",IF(AND(N3="نعم",Q3&lt;&gt;"موافق"),"ينقصه رأي المختص","صالح للنشر")))))</f>
         <v/>
+      </c>
+      <c r="U3" s="7" t="inlineStr">
+        <is>
+          <t>كيف نزل القرآن؟ | في أي شهر نزل القرآن؟ | ما معنى سورة مكية؟</t>
+        </is>
       </c>
     </row>
     <row r="4" ht="150" customHeight="1">
@@ -4403,6 +4551,11 @@
       <c r="S4" s="7">
         <f>IF(A4="","",IF(OR(M4="ج",M4="د"),"المستوى لا يُنشر",IF(IFERROR(INDEX(المصادر!$F$2:$F$30,MATCH(D4,المصادر!$A$2:$A$30,0)),"")&lt;&gt;"نعم","المصدر غير معتمد",IF(OR(B4="",E4="",J4="",K4="",P4=""),"بيانات ناقصة",IF(AND(N4="نعم",Q4&lt;&gt;"موافق"),"ينقصه رأي المختص","صالح للنشر")))))</f>
         <v/>
+      </c>
+      <c r="U4" s="7" t="inlineStr">
+        <is>
+          <t>كيف كان الوحي يأتي النبي؟ | متى بدأ نزول الوحي؟</t>
+        </is>
       </c>
     </row>
     <row r="5" ht="150" customHeight="1">
@@ -4500,6 +4653,11 @@
       <c r="S5" s="7">
         <f>IF(A5="","",IF(OR(M5="ج",M5="د"),"المستوى لا يُنشر",IF(IFERROR(INDEX(المصادر!$F$2:$F$30,MATCH(D5,المصادر!$A$2:$A$30,0)),"")&lt;&gt;"نعم","المصدر غير معتمد",IF(OR(B5="",E5="",J5="",K5="",P5=""),"بيانات ناقصة",IF(AND(N5="نعم",Q5&lt;&gt;"موافق"),"ينقصه رأي المختص","صالح للنشر")))))</f>
         <v/>
+      </c>
+      <c r="U5" s="7" t="inlineStr">
+        <is>
+          <t>في أي شهر نزل القرآن؟ | هل نزل القرآن مفرقاً؟ | متى جُمع القرآن في مصحف واحد؟</t>
+        </is>
       </c>
     </row>
     <row r="6" ht="150" customHeight="1">
@@ -4598,6 +4756,11 @@
       <c r="S6" s="7">
         <f>IF(A6="","",IF(OR(M6="ج",M6="د"),"المستوى لا يُنشر",IF(IFERROR(INDEX(المصادر!$F$2:$F$30,MATCH(D6,المصادر!$A$2:$A$30,0)),"")&lt;&gt;"نعم","المصدر غير معتمد",IF(OR(B6="",E6="",J6="",K6="",P6=""),"بيانات ناقصة",IF(AND(N6="نعم",Q6&lt;&gt;"موافق"),"ينقصه رأي المختص","صالح للنشر")))))</f>
         <v/>
+      </c>
+      <c r="U6" s="7" t="inlineStr">
+        <is>
+          <t>كيف كان الوحي ينزل على النبي؟ | كم عدد الحفاظ من الصحابة؟</t>
+        </is>
       </c>
     </row>
     <row r="7" ht="150" customHeight="1">
@@ -4703,6 +4866,11 @@
         <f>IF(A7="","",IF(OR(M7="ج",M7="د"),"المستوى لا يُنشر",IF(IFERROR(INDEX(المصادر!$F$2:$F$30,MATCH(D7,المصادر!$A$2:$A$30,0)),"")&lt;&gt;"نعم","المصدر غير معتمد",IF(OR(B7="",E7="",J7="",K7="",P7=""),"بيانات ناقصة",IF(AND(N7="نعم",Q7&lt;&gt;"موافق"),"ينقصه رأي المختص","صالح للنشر")))))</f>
         <v/>
       </c>
+      <c r="U7" s="7" t="inlineStr">
+        <is>
+          <t>كيف كُتب القرآن زمن النبي؟ | ما القراءات؟</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="150" customHeight="1">
       <c r="A8" s="5" t="inlineStr">
@@ -4801,6 +4969,11 @@
       <c r="S8" s="7">
         <f>IF(A8="","",IF(OR(M8="ج",M8="د"),"المستوى لا يُنشر",IF(IFERROR(INDEX(المصادر!$F$2:$F$30,MATCH(D8,المصادر!$A$2:$A$30,0)),"")&lt;&gt;"نعم","المصدر غير معتمد",IF(OR(B8="",E8="",J8="",K8="",P8=""),"بيانات ناقصة",IF(AND(N8="نعم",Q8&lt;&gt;"موافق"),"ينقصه رأي المختص","صالح للنشر")))))</f>
         <v/>
+      </c>
+      <c r="U8" s="7" t="inlineStr">
+        <is>
+          <t>كيف جمع عثمان القرآن؟ | كيف أحفظ القرآن؟</t>
+        </is>
       </c>
     </row>
     <row r="9" ht="150" customHeight="1">
@@ -4902,6 +5075,11 @@
         <f>IF(A9="","",IF(OR(M9="ج",M9="د"),"المستوى لا يُنشر",IF(IFERROR(INDEX(المصادر!$F$2:$F$30,MATCH(D9,المصادر!$A$2:$A$30,0)),"")&lt;&gt;"نعم","المصدر غير معتمد",IF(OR(B9="",E9="",J9="",K9="",P9=""),"بيانات ناقصة",IF(AND(N9="نعم",Q9&lt;&gt;"موافق"),"ينقصه رأي المختص","صالح للنشر")))))</f>
         <v/>
       </c>
+      <c r="U9" s="7" t="inlineStr">
+        <is>
+          <t>كم عدد سور القرآن؟ | لماذا تتنقل السورة بين موضوعات مختلفة؟</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="150" customHeight="1">
       <c r="A10" s="5" t="inlineStr">
@@ -4995,6 +5173,11 @@
       <c r="S10" s="7">
         <f>IF(A10="","",IF(OR(M10="ج",M10="د"),"المستوى لا يُنشر",IF(IFERROR(INDEX(المصادر!$F$2:$F$30,MATCH(D10,المصادر!$A$2:$A$30,0)),"")&lt;&gt;"نعم","المصدر غير معتمد",IF(OR(B10="",E10="",J10="",K10="",P10=""),"بيانات ناقصة",IF(AND(N10="نعم",Q10&lt;&gt;"موافق"),"ينقصه رأي المختص","صالح للنشر")))))</f>
         <v/>
+      </c>
+      <c r="U10" s="7" t="inlineStr">
+        <is>
+          <t>من رتّب سور القرآن؟ | ما أبرز موضوعات القرآن؟</t>
+        </is>
       </c>
     </row>
     <row r="11" ht="150" customHeight="1">
@@ -5091,6 +5274,11 @@
         <f>IF(A11="","",IF(OR(M11="ج",M11="د"),"المستوى لا يُنشر",IF(IFERROR(INDEX(المصادر!$F$2:$F$30,MATCH(D11,المصادر!$A$2:$A$30,0)),"")&lt;&gt;"نعم","المصدر غير معتمد",IF(OR(B11="",E11="",J11="",K11="",P11=""),"بيانات ناقصة",IF(AND(N11="نعم",Q11&lt;&gt;"موافق"),"ينقصه رأي المختص","صالح للنشر")))))</f>
         <v/>
       </c>
+      <c r="U11" s="7" t="inlineStr">
+        <is>
+          <t>ما أفضل ترجمة للقرآن؟ | ما هو التفسير؟ | هل تجوز الصلاة بترجمة القرآن؟</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="150" customHeight="1">
       <c r="A12" s="5" t="inlineStr">
@@ -5188,6 +5376,11 @@
       <c r="S12" s="7">
         <f>IF(A12="","",IF(OR(M12="ج",M12="د"),"المستوى لا يُنشر",IF(IFERROR(INDEX(المصادر!$F$2:$F$30,MATCH(D12,المصادر!$A$2:$A$30,0)),"")&lt;&gt;"نعم","المصدر غير معتمد",IF(OR(B12="",E12="",J12="",K12="",P12=""),"بيانات ناقصة",IF(AND(N12="نعم",Q12&lt;&gt;"موافق"),"ينقصه رأي المختص","صالح للنشر")))))</f>
         <v/>
+      </c>
+      <c r="U12" s="7" t="inlineStr">
+        <is>
+          <t>ما تعريف القرآن؟ | لماذا يعظّم المسلمون القرآن؟ | ما أمثلة الإعجاز العلمي؟</t>
+        </is>
       </c>
     </row>
     <row r="13" ht="150" customHeight="1">
@@ -5288,6 +5481,11 @@
         <f>IF(A13="","",IF(OR(M13="ج",M13="د"),"المستوى لا يُنشر",IF(IFERROR(INDEX(المصادر!$F$2:$F$30,MATCH(D13,المصادر!$A$2:$A$30,0)),"")&lt;&gt;"نعم","المصدر غير معتمد",IF(OR(B13="",E13="",J13="",K13="",P13=""),"بيانات ناقصة",IF(AND(N13="نعم",Q13&lt;&gt;"موافق"),"ينقصه رأي المختص","صالح للنشر")))))</f>
         <v/>
       </c>
+      <c r="U13" s="7" t="inlineStr">
+        <is>
+          <t>ما هو القرآن؟ | ما مكانة القرآن؟ | كيف كان الوحي ينزل؟</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="150" customHeight="1">
       <c r="A14" s="5" t="inlineStr">
@@ -5385,6 +5583,11 @@
         <f>IF(A14="","",IF(OR(M14="ج",M14="د"),"المستوى لا يُنشر",IF(IFERROR(INDEX(المصادر!$F$2:$F$30,MATCH(D14,المصادر!$A$2:$A$30,0)),"")&lt;&gt;"نعم","المصدر غير معتمد",IF(OR(B14="",E14="",J14="",K14="",P14=""),"بيانات ناقصة",IF(AND(N14="نعم",Q14&lt;&gt;"موافق"),"ينقصه رأي المختص","صالح للنشر")))))</f>
         <v/>
       </c>
+      <c r="U14" s="7" t="inlineStr">
+        <is>
+          <t>ما معنى أن القرآن مهيمن على الكتب السابقة؟ | ما قصص الأنبياء في القرآن؟</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="150" customHeight="1">
       <c r="A15" s="5" t="inlineStr">
@@ -5481,6 +5684,11 @@
         <f>IF(A15="","",IF(OR(M15="ج",M15="د"),"المستوى لا يُنشر",IF(IFERROR(INDEX(المصادر!$F$2:$F$30,MATCH(D15,المصادر!$A$2:$A$30,0)),"")&lt;&gt;"نعم","المصدر غير معتمد",IF(OR(B15="",E15="",J15="",K15="",P15=""),"بيانات ناقصة",IF(AND(N15="نعم",Q15&lt;&gt;"موافق"),"ينقصه رأي المختص","صالح للنشر")))))</f>
         <v/>
       </c>
+      <c r="U15" s="7" t="inlineStr">
+        <is>
+          <t>كيف جُمع القرآن؟ | ما أسباب نزول آية بعينها؟</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="150" customHeight="1">
       <c r="A16" s="5" t="inlineStr">
@@ -5578,6 +5786,11 @@
       <c r="S16" s="7">
         <f>IF(A16="","",IF(OR(M16="ج",M16="د"),"المستوى لا يُنشر",IF(IFERROR(INDEX(المصادر!$F$2:$F$30,MATCH(D16,المصادر!$A$2:$A$30,0)),"")&lt;&gt;"نعم","المصدر غير معتمد",IF(OR(B16="",E16="",J16="",K16="",P16=""),"بيانات ناقصة",IF(AND(N16="نعم",Q16&lt;&gt;"موافق"),"ينقصه رأي المختص","صالح للنشر")))))</f>
         <v/>
+      </c>
+      <c r="U16" s="7" t="inlineStr">
+        <is>
+          <t>ما أمثلة الإعجاز العلمي؟ | ما مكانة القرآن؟</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -5598,6 +5811,7 @@
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Phase 2: show a verse from the Mushaf when the user names it (البقرة 255، آية الكرسي) with its al-Muyassar link; fixed clarification for «من كتب القرآن؟» (template ست-05 in review)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RkXtRf8o9rcFbV2XzFoBFz
</commit_message>
<xml_diff>
--- a/data/register.xlsx
+++ b/data/register.xlsx
@@ -705,7 +705,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X52"/>
+  <dimension ref="A1:X53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -4142,6 +4142,52 @@
       <c r="V52" s="6" t="n"/>
       <c r="W52" s="6" t="n"/>
       <c r="X52" s="6" t="n"/>
+    </row>
+    <row r="53" ht="34" customHeight="1">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t>قالب</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="inlineStr">
+        <is>
+          <t>ست-05</t>
+        </is>
+      </c>
+      <c r="C53" s="6" t="inlineStr">
+        <is>
+          <t>سؤال «من كتب القرآن؟»: المصدر أم كتّاب الوحي</t>
+        </is>
+      </c>
+      <c r="D53" s="6" t="n"/>
+      <c r="E53" s="6" t="n"/>
+      <c r="F53" s="6" t="n"/>
+      <c r="G53" s="6" t="n"/>
+      <c r="H53" s="6" t="n"/>
+      <c r="I53" s="6" t="n"/>
+      <c r="J53" s="6" t="n"/>
+      <c r="K53" s="6" t="inlineStr">
+        <is>
+          <t>هل تسأل من أين جاء القرآن ولماذا يؤمن المسلمون أنه كلام الله، أم من كان يكتبه ويحفظه في عهد النبي ﷺ؟</t>
+        </is>
+      </c>
+      <c r="L53" s="6" t="n"/>
+      <c r="M53" s="6" t="n"/>
+      <c r="N53" s="6" t="n"/>
+      <c r="O53" s="6" t="n"/>
+      <c r="P53" s="6" t="n"/>
+      <c r="Q53" s="6" t="inlineStr">
+        <is>
+          <t>استيضاح ثابت بين ح7 وح3 (ملاحظة المراجعة الحية). مراجعة شرعية: نعم.</t>
+        </is>
+      </c>
+      <c r="R53" s="6" t="n"/>
+      <c r="S53" s="6" t="n"/>
+      <c r="T53" s="6" t="n"/>
+      <c r="U53" s="6" t="n"/>
+      <c r="V53" s="6" t="n"/>
+      <c r="W53" s="6" t="n"/>
+      <c r="X53" s="6" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:V49"/>

</xml_diff>

<commit_message>
Acceptance cases from the methodology pack, partial-limit line (template و-16), follow-up choices after «لا/جزئياً», and two stale dev labels fixed
- Six dev cases (d38–d43): practical start, who wrote, evidence, verse location, comparison follow-up, «إذا قرأت ولم أفهم».
- d09 accepts ق-16 and d15 accepts ق-20: both were unpublished when the labels were written (fixed after seeing the run; disclosed).
- Template و-16 (draft) under a partial passage; after «لا» or «جزئياً» the user can ask for the rest, the detail, the source, a new question or the menu.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RkXtRf8o9rcFbV2XzFoBFz
</commit_message>
<xml_diff>
--- a/data/register.xlsx
+++ b/data/register.xlsx
@@ -778,7 +778,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z1"/>
+  <dimension ref="A1:Z2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -940,7 +940,54 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="150" customHeight="1"/>
+    <row r="2" ht="150" customHeight="1">
+      <c r="A2" s="10" t="inlineStr">
+        <is>
+          <t>قالب</t>
+        </is>
+      </c>
+      <c r="B2" s="10" t="inlineStr">
+        <is>
+          <t>و-16</t>
+        </is>
+      </c>
+      <c r="C2" s="11" t="inlineStr">
+        <is>
+          <t>تحت المقطع الذي حكم الفحص بأنه يجيب عن جزء من السؤال فقط (عنوانه «مقطع متعلق بسؤالك»)</t>
+        </is>
+      </c>
+      <c r="D2" s="11" t="n"/>
+      <c r="E2" s="11" t="n"/>
+      <c r="F2" s="11" t="n"/>
+      <c r="G2" s="11" t="n"/>
+      <c r="H2" s="11" t="n"/>
+      <c r="I2" s="11" t="n"/>
+      <c r="J2" s="11" t="n"/>
+      <c r="K2" s="11" t="inlineStr">
+        <is>
+          <t>قد لا يجيب هذا النص عن سؤالك كله. إن بقي منه شيء فاختر «جزئياً» واكتب ما بقي.</t>
+        </is>
+      </c>
+      <c r="L2" s="11" t="n"/>
+      <c r="M2" s="11" t="n"/>
+      <c r="N2" s="11" t="n"/>
+      <c r="O2" s="11" t="n"/>
+      <c r="P2" s="11" t="n"/>
+      <c r="Q2" s="11" t="inlineStr">
+        <is>
+          <t>نص واجهة، لا يحتاج مراجعة شرعية. يطابق ما تطلبه المنهجية: الجواب الجزئي يصرّح بحدوده.</t>
+        </is>
+      </c>
+      <c r="R2" s="11" t="n"/>
+      <c r="S2" s="11" t="n"/>
+      <c r="T2" s="11" t="n"/>
+      <c r="U2" s="11" t="n"/>
+      <c r="V2" s="11" t="n"/>
+      <c r="W2" s="11" t="n"/>
+      <c r="X2" s="11" t="n"/>
+      <c r="Y2" s="11" t="n"/>
+      <c r="Z2" s="11" t="n"/>
+    </row>
     <row r="3" ht="150" customHeight="1"/>
     <row r="4" ht="150" customHeight="1"/>
     <row r="5" ht="150" customHeight="1"/>
@@ -998,8 +1045,11 @@
     <cfRule type="expression" priority="3" dxfId="4">
       <formula>$O2="نعم"</formula>
     </cfRule>
+    <cfRule type="expression" priority="4" dxfId="4">
+      <formula>$O2="نعم"</formula>
+    </cfRule>
   </conditionalFormatting>
-  <dataValidations count="5">
+  <dataValidations count="7">
     <dataValidation sqref="S2:S300" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"معتمد,معتمد بتعديل,مرفوض"</formula1>
     </dataValidation>
@@ -1008,6 +1058,12 @@
     </dataValidation>
     <dataValidation sqref="W2:W300" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"نعم,لا"</formula1>
+    </dataValidation>
+    <dataValidation sqref="S2:S300" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"معتمد,معتمد بتعديل,مرفوض"</formula1>
+    </dataValidation>
+    <dataValidation sqref="V2:V300" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"موافق,موافق بتعديل,غير موافق"</formula1>
     </dataValidation>
     <dataValidation sqref="S2:S300" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"معتمد,معتمد بتعديل,مرفوض"</formula1>

</xml_diff>

<commit_message>
Template و-16 approved by the reviewer
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RkXtRf8o9rcFbV2XzFoBFz
</commit_message>
<xml_diff>
--- a/data/register.xlsx
+++ b/data/register.xlsx
@@ -778,7 +778,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z2"/>
+  <dimension ref="A1:Z1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -940,54 +940,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="150" customHeight="1">
-      <c r="A2" s="10" t="inlineStr">
-        <is>
-          <t>قالب</t>
-        </is>
-      </c>
-      <c r="B2" s="10" t="inlineStr">
-        <is>
-          <t>و-16</t>
-        </is>
-      </c>
-      <c r="C2" s="11" t="inlineStr">
-        <is>
-          <t>تحت المقطع الذي حكم الفحص بأنه يجيب عن جزء من السؤال فقط (عنوانه «مقطع متعلق بسؤالك»)</t>
-        </is>
-      </c>
-      <c r="D2" s="11" t="n"/>
-      <c r="E2" s="11" t="n"/>
-      <c r="F2" s="11" t="n"/>
-      <c r="G2" s="11" t="n"/>
-      <c r="H2" s="11" t="n"/>
-      <c r="I2" s="11" t="n"/>
-      <c r="J2" s="11" t="n"/>
-      <c r="K2" s="11" t="inlineStr">
-        <is>
-          <t>قد لا يجيب هذا النص عن سؤالك كله. إن بقي منه شيء فاختر «جزئياً» واكتب ما بقي.</t>
-        </is>
-      </c>
-      <c r="L2" s="11" t="n"/>
-      <c r="M2" s="11" t="n"/>
-      <c r="N2" s="11" t="n"/>
-      <c r="O2" s="11" t="n"/>
-      <c r="P2" s="11" t="n"/>
-      <c r="Q2" s="11" t="inlineStr">
-        <is>
-          <t>نص واجهة، لا يحتاج مراجعة شرعية. يطابق ما تطلبه المنهجية: الجواب الجزئي يصرّح بحدوده.</t>
-        </is>
-      </c>
-      <c r="R2" s="11" t="n"/>
-      <c r="S2" s="11" t="n"/>
-      <c r="T2" s="11" t="n"/>
-      <c r="U2" s="11" t="n"/>
-      <c r="V2" s="11" t="n"/>
-      <c r="W2" s="11" t="n"/>
-      <c r="X2" s="11" t="n"/>
-      <c r="Y2" s="11" t="n"/>
-      <c r="Z2" s="11" t="n"/>
-    </row>
+    <row r="2" ht="150" customHeight="1"/>
     <row r="3" ht="150" customHeight="1"/>
     <row r="4" ht="150" customHeight="1"/>
     <row r="5" ht="150" customHeight="1"/>
@@ -1048,8 +1001,11 @@
     <cfRule type="expression" priority="4" dxfId="4">
       <formula>$O2="نعم"</formula>
     </cfRule>
+    <cfRule type="expression" priority="5" dxfId="4">
+      <formula>$O2="نعم"</formula>
+    </cfRule>
   </conditionalFormatting>
-  <dataValidations count="7">
+  <dataValidations count="9">
     <dataValidation sqref="S2:S300" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"معتمد,معتمد بتعديل,مرفوض"</formula1>
     </dataValidation>
@@ -1058,6 +1014,12 @@
     </dataValidation>
     <dataValidation sqref="W2:W300" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"نعم,لا"</formula1>
+    </dataValidation>
+    <dataValidation sqref="S2:S300" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"معتمد,معتمد بتعديل,مرفوض"</formula1>
+    </dataValidation>
+    <dataValidation sqref="V2:V300" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"موافق,موافق بتعديل,غير موافق"</formula1>
     </dataValidation>
     <dataValidation sqref="S2:S300" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"معتمد,معتمد بتعديل,مرفوض"</formula1>
@@ -4651,12 +4613,18 @@
     <cfRule type="expression" priority="3" dxfId="5">
       <formula>$S2="صالح للنشر"</formula>
     </cfRule>
+    <cfRule type="expression" priority="5" dxfId="5">
+      <formula>$S2="صالح للنشر"</formula>
+    </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="N2:N200">
     <cfRule type="expression" priority="2" dxfId="0">
       <formula>$N2="نعم"</formula>
     </cfRule>
     <cfRule type="expression" priority="4" dxfId="4">
+      <formula>$N2="نعم"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="6" dxfId="4">
       <formula>$N2="نعم"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -4676,7 +4644,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F34"/>
+  <dimension ref="A1:F35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -5770,6 +5738,38 @@
         </is>
       </c>
       <c r="F34" s="11" t="inlineStr">
+        <is>
+          <t>اعتُمد دون ملاحظات.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="34" customHeight="1">
+      <c r="A35" s="10" t="inlineStr">
+        <is>
+          <t>و-16</t>
+        </is>
+      </c>
+      <c r="B35" s="10" t="inlineStr">
+        <is>
+          <t>تحت المقطع الذي حكم الفحص بأنه يجيب عن جزء من السؤال فقط (عنوانه «مقطع متعلق بسؤالك»)</t>
+        </is>
+      </c>
+      <c r="C35" s="11" t="inlineStr">
+        <is>
+          <t>قد لا يجيب هذا النص عن سؤالك كله. إن بقي منه شيء فاختر «جزئياً» واكتب ما بقي.</t>
+        </is>
+      </c>
+      <c r="D35" s="11" t="inlineStr">
+        <is>
+          <t>لا</t>
+        </is>
+      </c>
+      <c r="E35" s="11" t="inlineStr">
+        <is>
+          <t>محمد — 5 أكتوبر 2026</t>
+        </is>
+      </c>
+      <c r="F35" s="11" t="inlineStr">
         <is>
           <t>اعتُمد دون ملاحظات.</t>
         </is>

</xml_diff>

<commit_message>
Register: move three phrasings to the passage that answers them and drop one the text does not answer (after the register run, reviewer-approved)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RkXtRf8o9rcFbV2XzFoBFz
</commit_message>
<xml_diff>
--- a/data/register.xlsx
+++ b/data/register.xlsx
@@ -1801,7 +1801,7 @@
       </c>
       <c r="R7" s="6" t="inlineStr">
         <is>
-          <t>مراجعة النقل: مطابق دون ملاحظات. مقطع حساس: وافق المختص الأعلم دون تعديل (2026-10-04). [5 أكتوبر] عُدّلت بيانات التوجيه بعد مراجعة اللجنة الخارجية؛ النص المعتمد لم يتغير. «لا يُجتزأ»: مقطع حجاجي يُعرض كاملاً حتى لا تُقتطع نتيجة دون حجتها (ملاحظة اللجنة).</t>
+          <t>مراجعة النقل: مطابق دون ملاحظات. مقطع حساس: وافق المختص الأعلم دون تعديل (2026-10-04). [5 أكتوبر] عُدّلت بيانات التوجيه بعد مراجعة اللجنة الخارجية؛ النص المعتمد لم يتغير. «لا يُجتزأ»: مقطع حجاجي يُعرض كاملاً حتى لا تُقتطع نتيجة دون حجتها (ملاحظة اللجنة). [5 أكتوبر] أُضيفت صياغة «لماذا جمع عثمان القرآن؟» من ق-33 (موافقة محمد).</t>
         </is>
       </c>
       <c r="S7" s="7">
@@ -1880,7 +1880,7 @@
       </c>
       <c r="L8" s="6" t="inlineStr">
         <is>
-          <t>كم عدد الصحابة الذين حفظوا القرآن؟ | هل نُقل القرآن عن عدد قليل؟ | كيف وصل القرآن إلينا؟</t>
+          <t>كم عدد الصحابة الذين حفظوا القرآن؟ | هل نُقل القرآن عن عدد قليل؟</t>
         </is>
       </c>
       <c r="M8" s="6" t="inlineStr">
@@ -1910,7 +1910,7 @@
       </c>
       <c r="R8" s="6" t="inlineStr">
         <is>
-          <t>مراجعة النقل: مطابق دون ملاحظات. مقطع حساس: وافق المختص الأعلم دون تعديل (2026-10-04). «لا يُجتزأ»: مقطع حجاجي يُعرض كاملاً حتى لا تُقتطع نتيجة دون حجتها (ملاحظة اللجنة).</t>
+          <t>مراجعة النقل: مطابق دون ملاحظات. مقطع حساس: وافق المختص الأعلم دون تعديل (2026-10-04). «لا يُجتزأ»: مقطع حجاجي يُعرض كاملاً حتى لا تُقتطع نتيجة دون حجتها (ملاحظة اللجنة). [5 أكتوبر] نُقلت صياغة «كيف وصل القرآن إلينا؟» إلى ق-33 بعد قياس السجل (موافقة محمد).</t>
         </is>
       </c>
       <c r="S8" s="7">
@@ -2912,7 +2912,7 @@
       </c>
       <c r="L18" s="11" t="inlineStr">
         <is>
-          <t>ما مكانة القرآن عند المسلمين؟ | لماذا يعظّم المسلمون القرآن؟ | ما فائدة القرآن للإنسان؟ | لماذا يقرأ المسلمون القرآن كثيراً؟</t>
+          <t>ما مكانة القرآن عند المسلمين؟ | لماذا يعظّم المسلمون القرآن؟ | ما فائدة القرآن للإنسان؟</t>
         </is>
       </c>
       <c r="M18" s="11" t="inlineStr">
@@ -2938,7 +2938,7 @@
       <c r="Q18" s="11" t="n"/>
       <c r="R18" s="11" t="inlineStr">
         <is>
-          <t>اعتُمد دون ملاحظات.</t>
+          <t>اعتُمد دون ملاحظات. [5 أكتوبر] نُقلت صياغة «لماذا يقرأ المسلمون القرآن كثيراً؟» إلى ق-36 بعد قياس السجل (موافقة محمد).</t>
         </is>
       </c>
       <c r="S18" s="12">
@@ -3572,7 +3572,7 @@
       </c>
       <c r="L25" s="11" t="inlineStr">
         <is>
-          <t>كيف جُمع القرآن؟ | متى صار القرآن كتاباً واحداً؟ | لماذا جمع أبو بكر القرآن؟ | لماذا جمع عثمان القرآن؟ | هل تغيّر القرآن منذ زمن الصحابة؟</t>
+          <t>كيف جُمع القرآن؟ | متى صار القرآن كتاباً واحداً؟ | لماذا جمع أبو بكر القرآن؟ | هل تغيّر القرآن منذ زمن الصحابة؟ | كيف وصل القرآن إلينا؟</t>
         </is>
       </c>
       <c r="M25" s="11" t="inlineStr">
@@ -3598,7 +3598,7 @@
       <c r="Q25" s="11" t="n"/>
       <c r="R25" s="11" t="inlineStr">
         <is>
-          <t>اعتُمد دون ملاحظات.</t>
+          <t>اعتُمد دون ملاحظات. [5 أكتوبر] أُضيفت صياغة «كيف وصل القرآن إلينا؟» من ق-14 (موافقة محمد). [5 أكتوبر] نُقلت صياغة «لماذا جمع عثمان القرآن؟» إلى ق-13 بعد قياس السجل (موافقة محمد).</t>
         </is>
       </c>
       <c r="S25" s="12">
@@ -3757,7 +3757,7 @@
       </c>
       <c r="L27" s="11" t="inlineStr">
         <is>
-          <t>ما فضل قراءة القرآن؟ | لماذا أقرأ القرآن؟ | هل في قراءة القرآن أجر؟ | ما فائدة الاجتماع على القرآن؟</t>
+          <t>ما فضل قراءة القرآن؟ | لماذا أقرأ القرآن؟ | هل في قراءة القرآن أجر؟ | ما فائدة الاجتماع على القرآن؟ | لماذا يقرأ المسلمون القرآن كثيراً؟</t>
         </is>
       </c>
       <c r="M27" s="11" t="inlineStr">
@@ -3783,7 +3783,7 @@
       <c r="Q27" s="11" t="n"/>
       <c r="R27" s="11" t="inlineStr">
         <is>
-          <t>اعتُمد دون ملاحظات.</t>
+          <t>اعتُمد دون ملاحظات. [5 أكتوبر] أُضيفت صياغة «لماذا يقرأ المسلمون القرآن كثيراً؟» من ق-02 (موافقة محمد).</t>
         </is>
       </c>
       <c r="S27" s="12">
@@ -4350,7 +4350,7 @@
       </c>
       <c r="L33" s="11" t="inlineStr">
         <is>
-          <t>ليش السور مو مرتبة حسب نزولها؟ | من رتب سور القرآن؟ | هل ترتيب الآيات من النبي؟ | ليش البقرة أول القرآن مع إنها مدنية؟</t>
+          <t>ليش السور مو مرتبة حسب نزولها؟ | من رتب سور القرآن؟ | هل ترتيب الآيات من النبي؟</t>
         </is>
       </c>
       <c r="M33" s="11" t="inlineStr">
@@ -4376,7 +4376,7 @@
       <c r="Q33" s="11" t="n"/>
       <c r="R33" s="11" t="inlineStr">
         <is>
-          <t>نُفّذ: جملة المراجع تظهر سطراً مستقلاً بعنوان «تنبيه المراجع» لا داخل الاقتباس.</t>
+          <t>نُفّذ: جملة المراجع تظهر سطراً مستقلاً بعنوان «تنبيه المراجع» لا داخل الاقتباس. [5 أكتوبر] حُذفت صياغة «ليش البقرة أول القرآن مع إنها مدنية؟» لأن النص لا يذكر البقرة (موافقة محمد).</t>
         </is>
       </c>
       <c r="S33" s="12">

</xml_diff>

<commit_message>
Follow-up v1 completed: «المعنى غير واضح» uses the passage's detail, then registered related content, then an honest approved message (ام-15); every follow-up is logged by kind; navigation buttons separated; docs corrected (G3 partial, review wording, model role, results tied to v21)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RkXtRf8o9rcFbV2XzFoBFz
</commit_message>
<xml_diff>
--- a/data/register.xlsx
+++ b/data/register.xlsx
@@ -818,7 +818,7 @@
       </c>
       <c r="B10" s="33" t="inlineStr">
         <is>
-          <t>34 مقطعاً · 7 احتياجات · 5 مصادر/مراجع · 39 قالب محادثة (منها ست-06 بخياراتها الثلاثة، وام-14، وو-16)</t>
+          <t>34 مقطعاً · 7 احتياجات · 5 مصادر/مراجع · 40 قالب محادثة (منها ست-06 بخياراتها الثلاثة، وام-14، وام-15، وو-16)</t>
         </is>
       </c>
       <c r="C10" s="33" t="str"/>
@@ -7277,8 +7277,8 @@
   </sheetData>
   <mergeCells count="6">
     <mergeCell ref="A2:AH2"/>
+    <mergeCell ref="N3:AA3"/>
     <mergeCell ref="A3:D3"/>
-    <mergeCell ref="N3:AA3"/>
     <mergeCell ref="AB3:AH3"/>
     <mergeCell ref="A1:AH1"/>
     <mergeCell ref="E3:M3"/>
@@ -8299,7 +8299,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H43"/>
+  <dimension ref="A1:H44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -10016,6 +10016,48 @@
         </is>
       </c>
       <c r="H43" s="37" t="inlineStr">
+        <is>
+          <t>اعتمده محمد نصاً في المحادثة (5 أكتوبر 2026).</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="58" customHeight="1">
+      <c r="A44" s="37" t="inlineStr">
+        <is>
+          <t>ام-15</t>
+        </is>
+      </c>
+      <c r="B44" s="37" t="inlineStr">
+        <is>
+          <t>NOT_COVERED</t>
+        </is>
+      </c>
+      <c r="C44" s="37" t="inlineStr">
+        <is>
+          <t>«المعنى غير واضح» بلا تفصيل ولا محتوى مرتبط</t>
+        </is>
+      </c>
+      <c r="D44" s="37" t="inlineStr">
+        <is>
+          <t>بعد «لا» أو «جزئياً» حين يختار المستخدم «المعنى غير واضح»، وليس للمقطع تفصيل لم يُعرض ولا محتوى مرتبط مسجّل</t>
+        </is>
+      </c>
+      <c r="E44" s="37" t="inlineStr">
+        <is>
+          <t>لا تحتوي مكتبة «دليل» حاليًا شرحًا أبسط لهذه النقطة. يمكنك الرجوع إلى مصدر موثوق يشرحها بمزيد من التبسيط، أو سؤال معلّم أو مختص.</t>
+        </is>
+      </c>
+      <c r="F44" s="37" t="inlineStr">
+        <is>
+          <t>لا</t>
+        </is>
+      </c>
+      <c r="G44" s="37" t="inlineStr">
+        <is>
+          <t>محمد — 5 أكتوبر 2026</t>
+        </is>
+      </c>
+      <c r="H44" s="37" t="inlineStr">
         <is>
           <t>اعتمده محمد نصاً في المحادثة (5 أكتوبر 2026).</t>
         </is>

</xml_diff>

<commit_message>
Library v23 final candidate (not pushed): v22 + negative/partial/clarify decisions (ق-14 partial, ق-25 explicit negative, ق-06 evidence-only negative), reference clarification templates ست-07/ست-08 (inactive), new gaps, governance note, changelog; 0 reference-text changes
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RkXtRf8o9rcFbV2XzFoBFz
</commit_message>
<xml_diff>
--- a/data/register.xlsx
+++ b/data/register.xlsx
@@ -4,16 +4,17 @@
   <workbookPr/>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="المحتوى المهيكل" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="الاحتياجات" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="المصادر" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="منطق المحادثة" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="للمراجعة" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="المرفوض" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="الناقص" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="التغطية والفجوات" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="قاموس المنهجية" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="تدقيق 34" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="سجل التغييرات" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="المحتوى المهيكل" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="الاحتياجات" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="المصادر" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="منطق المحادثة" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="للمراجعة" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="المرفوض" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="الناقص" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="التغطية والفجوات" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="قاموس المنهجية" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="تدقيق 34" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
 </workbook>
@@ -866,7 +867,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F13"/>
+  <dimension ref="A1:F15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" style="49" min="1" max="1"/>
@@ -901,7 +902,6 @@
       <c r="E2" s="1" t="n"/>
       <c r="F2" s="1" t="n"/>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="63" t="inlineStr">
         <is>
@@ -1051,6 +1051,30 @@
       <c r="B13" t="inlineStr">
         <is>
           <t>v22 (5 أكتوبر 2026): تدقيق المقاطع الـ34 (ورقة «تدقيق 34»): 12 مقطعاً عُدّلت بياناتها الوصفية فقط، ولم يتغير أي نص مرجعي. دُمج القالب ام-15، وحُذف «هل القرآن مثل الإنجيل عند المسيحيين؟» من صياغات ح1 النشطة ونُقل إلى الفجوات. أرقام v21 لا تنتقل إلى هذه النسخة إلا بقياس جديد.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>الحوكمة</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>جميع مصادر المحتوى في هذه النسخة معتمدة. المراجعة المسجلة لبعض المقاطع تتعلق بسلامة النقل والتجزئة والسياق وحدود استخدام المقتطف، ولا تعني بالضرورة مراجعة شرعية مستقلة لمضمون المصدر من الصفر.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>النسخة v23</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>v23 (المرشحة النهائية، 5 أكتوبر 2026): v22 + قرارات المنع والاستيضاح الأخيرة (ق-14، ق-25، ق-06)، وقالبا استيضاح مرجعيان غير مفعّلين (ست-07، ست-08)، وفجوات جديدة، و«سجل التغييرات». صفر تغييرات في النص المرجعي. القاعدة: المنع لما لا يصلح للسؤال أصلاً؛ PARTIAL لما يفيد دون أن يكمل؛ CLARIFY لما يحتمل معنى يجيب عنه المقطع ومعنى لا يجيب عنه.</t>
         </is>
       </c>
     </row>
@@ -1064,6 +1088,1106 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K33"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" style="49" min="1" max="1"/>
+    <col width="38" customWidth="1" style="49" min="2" max="2"/>
+    <col width="25" customWidth="1" style="49" min="3" max="3"/>
+    <col width="12" customWidth="1" style="49" min="4" max="4"/>
+    <col width="55" customWidth="1" style="49" min="5" max="5"/>
+    <col width="18" customWidth="1" style="49" min="6" max="6"/>
+    <col width="45" customWidth="1" style="49" min="7" max="7"/>
+    <col width="14" customWidth="1" style="49" min="8" max="8"/>
+    <col width="14" customWidth="1" style="49" min="9" max="9"/>
+    <col width="14" customWidth="1" style="49" min="10" max="10"/>
+    <col width="48" customWidth="1" style="49" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="9" t="inlineStr">
+        <is>
+          <t>Coverage Map — مصفوفة التغطية وفجوات النسخة الحالية</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="n"/>
+      <c r="C1" s="1" t="n"/>
+      <c r="D1" s="1" t="n"/>
+      <c r="E1" s="1" t="n"/>
+      <c r="F1" s="1" t="n"/>
+      <c r="G1" s="1" t="n"/>
+      <c r="H1" s="1" t="n"/>
+      <c r="I1" s="1" t="n"/>
+      <c r="J1" s="1" t="n"/>
+      <c r="K1" s="1" t="n"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="19" t="inlineStr">
+        <is>
+          <t>العدد لا يعني جودة التغطية وحده؛ الفجوات أدناه مبنية على مقارنة صياغات الاحتياجات بما تجيب عنه المقاطع وما تستبعده صراحة.</t>
+        </is>
+      </c>
+      <c r="B2" s="1" t="n"/>
+      <c r="C2" s="1" t="n"/>
+      <c r="D2" s="1" t="n"/>
+      <c r="E2" s="1" t="n"/>
+      <c r="F2" s="1" t="n"/>
+      <c r="G2" s="1" t="n"/>
+      <c r="H2" s="1" t="n"/>
+      <c r="I2" s="1" t="n"/>
+      <c r="J2" s="1" t="n"/>
+      <c r="K2" s="1" t="n"/>
+    </row>
+    <row r="3"/>
+    <row r="4">
+      <c r="A4" s="63" t="inlineStr">
+        <is>
+          <t>الحاجة</t>
+        </is>
+      </c>
+      <c r="B4" s="63" t="inlineStr">
+        <is>
+          <t>عدد المقاطع</t>
+        </is>
+      </c>
+      <c r="C4" s="63" t="inlineStr">
+        <is>
+          <t>تعريف</t>
+        </is>
+      </c>
+      <c r="D4" s="63" t="inlineStr">
+        <is>
+          <t>شرح</t>
+        </is>
+      </c>
+      <c r="E4" s="63" t="inlineStr">
+        <is>
+          <t>تعليم</t>
+        </is>
+      </c>
+      <c r="F4" s="63" t="inlineStr">
+        <is>
+          <t>استدلال</t>
+        </is>
+      </c>
+      <c r="G4" s="63" t="inlineStr">
+        <is>
+          <t>معالجة اعتراض</t>
+        </is>
+      </c>
+      <c r="H4" s="63" t="inlineStr">
+        <is>
+          <t>مقارنة</t>
+        </is>
+      </c>
+      <c r="I4" s="63" t="inlineStr">
+        <is>
+          <t>بحث أو تحقيق</t>
+        </is>
+      </c>
+      <c r="J4" s="63" t="inlineStr">
+        <is>
+          <t>توجيه عملي</t>
+        </is>
+      </c>
+      <c r="K4" s="63" t="inlineStr">
+        <is>
+          <t>الحكم</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="67" t="inlineStr">
+        <is>
+          <t>ح1</t>
+        </is>
+      </c>
+      <c r="B5" s="67" t="n">
+        <v>6</v>
+      </c>
+      <c r="C5" s="67" t="n">
+        <v>4</v>
+      </c>
+      <c r="D5" s="67" t="n">
+        <v>6</v>
+      </c>
+      <c r="E5" s="67" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" s="67" t="n">
+        <v>1</v>
+      </c>
+      <c r="G5" s="67" t="n">
+        <v>1</v>
+      </c>
+      <c r="H5" s="67" t="n">
+        <v>2</v>
+      </c>
+      <c r="I5" s="67" t="n">
+        <v>0</v>
+      </c>
+      <c r="J5" s="67" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" s="67" t="inlineStr">
+        <is>
+          <t>جيد؛ بقيت فجوتان: مقارنة مباشرة بين القرآن والحديث النبوي، والمقارنة العامة بين دور القرآن والإنجيل.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="67" t="inlineStr">
+        <is>
+          <t>ح5</t>
+        </is>
+      </c>
+      <c r="B6" s="67" t="n">
+        <v>2</v>
+      </c>
+      <c r="C6" s="67" t="n">
+        <v>2</v>
+      </c>
+      <c r="D6" s="67" t="n">
+        <v>2</v>
+      </c>
+      <c r="E6" s="67" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" s="67" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" s="67" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" s="67" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" s="67" t="n">
+        <v>0</v>
+      </c>
+      <c r="J6" s="67" t="n">
+        <v>0</v>
+      </c>
+      <c r="K6" s="67" t="inlineStr">
+        <is>
+          <t>جيد في عرض الموضوعات والقصص؛ لا يغطي استدلالاً مستقلاً على تاريخية القصص.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="67" t="inlineStr">
+        <is>
+          <t>ح2</t>
+        </is>
+      </c>
+      <c r="B7" s="67" t="n">
+        <v>6</v>
+      </c>
+      <c r="C7" s="67" t="n">
+        <v>2</v>
+      </c>
+      <c r="D7" s="67" t="n">
+        <v>6</v>
+      </c>
+      <c r="E7" s="67" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" s="67" t="n">
+        <v>1</v>
+      </c>
+      <c r="G7" s="67" t="n">
+        <v>2</v>
+      </c>
+      <c r="H7" s="67" t="n">
+        <v>1</v>
+      </c>
+      <c r="I7" s="67" t="n">
+        <v>1</v>
+      </c>
+      <c r="J7" s="67" t="n">
+        <v>0</v>
+      </c>
+      <c r="K7" s="67" t="inlineStr">
+        <is>
+          <t>جيد؛ بقيت فجوات في تعريف الوحي المباشر، ومدة النزول، وأول ما نزل.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="67" t="inlineStr">
+        <is>
+          <t>ح3</t>
+        </is>
+      </c>
+      <c r="B8" s="67" t="n">
+        <v>6</v>
+      </c>
+      <c r="C8" s="67" t="n">
+        <v>0</v>
+      </c>
+      <c r="D8" s="67" t="n">
+        <v>5</v>
+      </c>
+      <c r="E8" s="67" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" s="67" t="n">
+        <v>1</v>
+      </c>
+      <c r="G8" s="67" t="n">
+        <v>2</v>
+      </c>
+      <c r="H8" s="67" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" s="67" t="n">
+        <v>6</v>
+      </c>
+      <c r="J8" s="67" t="n">
+        <v>0</v>
+      </c>
+      <c r="K8" s="67" t="inlineStr">
+        <is>
+          <t>جيد؛ المقارنة المباشرة بين جمع أبي بكر وجمع عثمان تغطيتها جزئية.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="67" t="inlineStr">
+        <is>
+          <t>ح4</t>
+        </is>
+      </c>
+      <c r="B9" s="67" t="n">
+        <v>4</v>
+      </c>
+      <c r="C9" s="67" t="n">
+        <v>1</v>
+      </c>
+      <c r="D9" s="67" t="n">
+        <v>4</v>
+      </c>
+      <c r="E9" s="67" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" s="67" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" s="67" t="n">
+        <v>2</v>
+      </c>
+      <c r="H9" s="67" t="n">
+        <v>0</v>
+      </c>
+      <c r="I9" s="67" t="n">
+        <v>2</v>
+      </c>
+      <c r="J9" s="67" t="n">
+        <v>0</v>
+      </c>
+      <c r="K9" s="67" t="inlineStr">
+        <is>
+          <t>غير مكتمل عملياً؛ تعريف البنية موجود لكن الوصول إلى آية/جزء محدد غير مغطى.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="67" t="inlineStr">
+        <is>
+          <t>ح6</t>
+        </is>
+      </c>
+      <c r="B10" s="67" t="n">
+        <v>5</v>
+      </c>
+      <c r="C10" s="67" t="n">
+        <v>0</v>
+      </c>
+      <c r="D10" s="67" t="n">
+        <v>5</v>
+      </c>
+      <c r="E10" s="67" t="n">
+        <v>1</v>
+      </c>
+      <c r="F10" s="67" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" s="67" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" s="67" t="n">
+        <v>2</v>
+      </c>
+      <c r="I10" s="67" t="n">
+        <v>0</v>
+      </c>
+      <c r="J10" s="67" t="n">
+        <v>3</v>
+      </c>
+      <c r="K10" s="67" t="inlineStr">
+        <is>
+          <t>غير مكتمل عملياً؛ توجد مواد للفهم والفضل والترجمة، لكن نقطة البداية واختيار تفسير للمبتدئ غير مغطاتين.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="67" t="inlineStr">
+        <is>
+          <t>ح7</t>
+        </is>
+      </c>
+      <c r="B11" s="67" t="n">
+        <v>5</v>
+      </c>
+      <c r="C11" s="67" t="n">
+        <v>0</v>
+      </c>
+      <c r="D11" s="67" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" s="67" t="n">
+        <v>0</v>
+      </c>
+      <c r="F11" s="67" t="n">
+        <v>5</v>
+      </c>
+      <c r="G11" s="67" t="n">
+        <v>5</v>
+      </c>
+      <c r="H11" s="67" t="n">
+        <v>1</v>
+      </c>
+      <c r="I11" s="67" t="n">
+        <v>1</v>
+      </c>
+      <c r="J11" s="67" t="n">
+        <v>0</v>
+      </c>
+      <c r="K11" s="67" t="inlineStr">
+        <is>
+          <t>جيد في الاستدلال والاعتراضات؛ بقيت فجوة فرعية في سؤال معرفة النبي ﷺ بالقراءة والكتابة.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12"/>
+    <row r="13"/>
+    <row r="14"/>
+    <row r="15">
+      <c r="A15" s="45" t="inlineStr">
+        <is>
+          <t>فجوات واضحة تحتاج محتوى أو معالجة صريحة</t>
+        </is>
+      </c>
+      <c r="B15" s="1" t="n"/>
+      <c r="C15" s="1" t="n"/>
+      <c r="D15" s="1" t="n"/>
+      <c r="E15" s="1" t="n"/>
+      <c r="F15" s="1" t="n"/>
+      <c r="G15" s="1" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="63" t="inlineStr">
+        <is>
+          <t>الحاجة</t>
+        </is>
+      </c>
+      <c r="B16" s="63" t="inlineStr">
+        <is>
+          <t>السؤال/الفجوة</t>
+        </is>
+      </c>
+      <c r="C16" s="63" t="inlineStr">
+        <is>
+          <t>نوع الفجوة</t>
+        </is>
+      </c>
+      <c r="D16" s="63" t="inlineStr">
+        <is>
+          <t>الأولوية</t>
+        </is>
+      </c>
+      <c r="E16" s="63" t="inlineStr">
+        <is>
+          <t>الدليل من السجل</t>
+        </is>
+      </c>
+      <c r="F16" s="63" t="inlineStr">
+        <is>
+          <t>الحالة</t>
+        </is>
+      </c>
+      <c r="G16" s="63" t="inlineStr">
+        <is>
+          <t>الإجراء الهيكلي</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="60" customHeight="1" s="49">
+      <c r="A17" s="67" t="inlineStr">
+        <is>
+          <t>ح1</t>
+        </is>
+      </c>
+      <c r="B17" s="67" t="inlineStr">
+        <is>
+          <t>ما الفرق بين القرآن والحديث؟</t>
+        </is>
+      </c>
+      <c r="C17" s="67" t="inlineStr">
+        <is>
+          <t>تغطية مباشرة مفقودة</t>
+        </is>
+      </c>
+      <c r="D17" s="67" t="inlineStr">
+        <is>
+          <t>متوسطة</t>
+        </is>
+      </c>
+      <c r="E17" s="67" t="inlineStr">
+        <is>
+          <t>ق-35 يستبعد الفرق الشامل بين القرآن والحديث النبوي؛ ق-32 يعالج حجية السنة.</t>
+        </is>
+      </c>
+      <c r="F17" s="67" t="inlineStr">
+        <is>
+          <t>غير مغطى مباشرة</t>
+        </is>
+      </c>
+      <c r="G17" s="67" t="inlineStr">
+        <is>
+          <t>إضافة مقطع مقارنة مباشر أو إعلان عدم التغطية.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="60" customHeight="1" s="49">
+      <c r="A18" s="67" t="inlineStr">
+        <is>
+          <t>ح2</t>
+        </is>
+      </c>
+      <c r="B18" s="67" t="inlineStr">
+        <is>
+          <t>كم سنة استمر نزول القرآن؟</t>
+        </is>
+      </c>
+      <c r="C18" s="67" t="inlineStr">
+        <is>
+          <t>معلومة تأسيسية مفقودة</t>
+        </is>
+      </c>
+      <c r="D18" s="67" t="inlineStr">
+        <is>
+          <t>متوسطة</t>
+        </is>
+      </c>
+      <c r="E18" s="67" t="inlineStr">
+        <is>
+          <t>مذكور ضمن صياغات الحاجة ح2 ولا يوجد مقطع يجيب عنها مباشرة.</t>
+        </is>
+      </c>
+      <c r="F18" s="67" t="inlineStr">
+        <is>
+          <t>غير مغطى</t>
+        </is>
+      </c>
+      <c r="G18" s="67" t="inlineStr">
+        <is>
+          <t>إضافة مقتطف موثق مباشر.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="60" customHeight="1" s="49">
+      <c r="A19" s="67" t="inlineStr">
+        <is>
+          <t>ح2</t>
+        </is>
+      </c>
+      <c r="B19" s="67" t="inlineStr">
+        <is>
+          <t>ما أول آية نزلت؟</t>
+        </is>
+      </c>
+      <c r="C19" s="67" t="inlineStr">
+        <is>
+          <t>معلومة تأسيسية مفقودة</t>
+        </is>
+      </c>
+      <c r="D19" s="67" t="inlineStr">
+        <is>
+          <t>متوسطة</t>
+        </is>
+      </c>
+      <c r="E19" s="67" t="inlineStr">
+        <is>
+          <t>مذكور ضمن صياغات الحاجة ح2 ولا يوجد مقطع يجيب عنها مباشرة.</t>
+        </is>
+      </c>
+      <c r="F19" s="67" t="inlineStr">
+        <is>
+          <t>غير مغطى</t>
+        </is>
+      </c>
+      <c r="G19" s="67" t="inlineStr">
+        <is>
+          <t>إضافة مقتطف موثق مباشر.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="60" customHeight="1" s="49">
+      <c r="A20" s="67" t="inlineStr">
+        <is>
+          <t>ح3</t>
+        </is>
+      </c>
+      <c r="B20" s="67" t="inlineStr">
+        <is>
+          <t>ما الفرق بين جمع أبي بكر وجمع عثمان؟</t>
+        </is>
+      </c>
+      <c r="C20" s="67" t="inlineStr">
+        <is>
+          <t>مقارنة جزئية</t>
+        </is>
+      </c>
+      <c r="D20" s="67" t="inlineStr">
+        <is>
+          <t>متوسطة</t>
+        </is>
+      </c>
+      <c r="E20" s="67" t="inlineStr">
+        <is>
+          <t>ق-13 يذكر صراحة أنه لا يجيب عن المقارنة؛ ق-33 يعرض المراحل دون مقارنة مركزة.</t>
+        </is>
+      </c>
+      <c r="F20" s="67" t="inlineStr">
+        <is>
+          <t>جزئي</t>
+        </is>
+      </c>
+      <c r="G20" s="67" t="inlineStr">
+        <is>
+          <t>إضافة مقارنة قصيرة أو PARTIAL بحدود واضحة.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="60" customHeight="1" s="49">
+      <c r="A21" s="67" t="inlineStr">
+        <is>
+          <t>ح4</t>
+        </is>
+      </c>
+      <c r="B21" s="67" t="inlineStr">
+        <is>
+          <t>كيف أجد آية في المصحف؟</t>
+        </is>
+      </c>
+      <c r="C21" s="67" t="inlineStr">
+        <is>
+          <t>تعليم عملي مفقود</t>
+        </is>
+      </c>
+      <c r="D21" s="67" t="inlineStr">
+        <is>
+          <t>عالية</t>
+        </is>
+      </c>
+      <c r="E21" s="67" t="inlineStr">
+        <is>
+          <t>ق-15 يسجلها ضمن الأسئلة القريبة التي لا يجيب عنها.</t>
+        </is>
+      </c>
+      <c r="F21" s="67" t="inlineStr">
+        <is>
+          <t>غير مغطى</t>
+        </is>
+      </c>
+      <c r="G21" s="67" t="inlineStr">
+        <is>
+          <t>إضافة مقطع/إرشاد عملي مستقل.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="60" customHeight="1" s="49">
+      <c r="A22" s="67" t="inlineStr">
+        <is>
+          <t>ح4</t>
+        </is>
+      </c>
+      <c r="B22" s="67" t="inlineStr">
+        <is>
+          <t>ما معنى جزء عمّ؟</t>
+        </is>
+      </c>
+      <c r="C22" s="67" t="inlineStr">
+        <is>
+          <t>تعريف عملي مفقود</t>
+        </is>
+      </c>
+      <c r="D22" s="67" t="inlineStr">
+        <is>
+          <t>متوسطة</t>
+        </is>
+      </c>
+      <c r="E22" s="67" t="inlineStr">
+        <is>
+          <t>مذكور ضمن صياغات الحاجة ح4 ولا يوجد مقطع مباشر.</t>
+        </is>
+      </c>
+      <c r="F22" s="67" t="inlineStr">
+        <is>
+          <t>غير مغطى</t>
+        </is>
+      </c>
+      <c r="G22" s="67" t="inlineStr">
+        <is>
+          <t>إضافة مقتطف تعريفي مباشر.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="60" customHeight="1" s="49">
+      <c r="A23" s="67" t="inlineStr">
+        <is>
+          <t>ح4</t>
+        </is>
+      </c>
+      <c r="B23" s="67" t="inlineStr">
+        <is>
+          <t>كيف أعرف رقم الآية؟</t>
+        </is>
+      </c>
+      <c r="C23" s="67" t="inlineStr">
+        <is>
+          <t>تعليم عملي مفقود</t>
+        </is>
+      </c>
+      <c r="D23" s="67" t="inlineStr">
+        <is>
+          <t>عالية</t>
+        </is>
+      </c>
+      <c r="E23" s="67" t="inlineStr">
+        <is>
+          <t>مذكور ضمن صياغات الحاجة ح4 ولا يوجد مقطع مباشر.</t>
+        </is>
+      </c>
+      <c r="F23" s="67" t="inlineStr">
+        <is>
+          <t>غير مغطى</t>
+        </is>
+      </c>
+      <c r="G23" s="67" t="inlineStr">
+        <is>
+          <t>إضافة مقطع/إرشاد عملي مستقل.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="60" customHeight="1" s="49">
+      <c r="A24" s="67" t="inlineStr">
+        <is>
+          <t>ح6</t>
+        </is>
+      </c>
+      <c r="B24" s="67" t="inlineStr">
+        <is>
+          <t>من أين أبدأ قراءة القرآن؟</t>
+        </is>
+      </c>
+      <c r="C24" s="67" t="inlineStr">
+        <is>
+          <t>توجيه عملي مفقود</t>
+        </is>
+      </c>
+      <c r="D24" s="67" t="inlineStr">
+        <is>
+          <t>عالية</t>
+        </is>
+      </c>
+      <c r="E24" s="67" t="inlineStr">
+        <is>
+          <t>ق-18 في ورقة «الناقص» الأصلية: من أين يبدأ المبتدئ القراءة.</t>
+        </is>
+      </c>
+      <c r="F24" s="67" t="inlineStr">
+        <is>
+          <t>غير مغطى</t>
+        </is>
+      </c>
+      <c r="G24" s="67" t="inlineStr">
+        <is>
+          <t>إضافة مادة بداية عملية قبل التجميد.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="60" customHeight="1" s="49">
+      <c r="A25" s="67" t="inlineStr">
+        <is>
+          <t>ح6</t>
+        </is>
+      </c>
+      <c r="B25" s="67" t="inlineStr">
+        <is>
+          <t>ما أفضل تفسير للمبتدئ؟</t>
+        </is>
+      </c>
+      <c r="C25" s="67" t="inlineStr">
+        <is>
+          <t>توجيه مصدر مفقود</t>
+        </is>
+      </c>
+      <c r="D25" s="67" t="inlineStr">
+        <is>
+          <t>عالية</t>
+        </is>
+      </c>
+      <c r="E25" s="67" t="inlineStr">
+        <is>
+          <t>ق-19 يسجل السؤال ضمن الأسئلة القريبة التي لا يجيب عنها.</t>
+        </is>
+      </c>
+      <c r="F25" s="67" t="inlineStr">
+        <is>
+          <t>غير مغطى</t>
+        </is>
+      </c>
+      <c r="G25" s="67" t="inlineStr">
+        <is>
+          <t>إضافة توصية مصدر مراجعة وفق سياسة المرجعية أو إحالة مضبوطة.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="60" customHeight="1" s="49">
+      <c r="A26" s="67" t="inlineStr">
+        <is>
+          <t>ح7</t>
+        </is>
+      </c>
+      <c r="B26" s="67" t="inlineStr">
+        <is>
+          <t>هل كان النبي يعرف القراءة والكتابة؟</t>
+        </is>
+      </c>
+      <c r="C26" s="67" t="inlineStr">
+        <is>
+          <t>استدلال فرعي مفقود</t>
+        </is>
+      </c>
+      <c r="D26" s="67" t="inlineStr">
+        <is>
+          <t>متوسطة</t>
+        </is>
+      </c>
+      <c r="E26" s="67" t="inlineStr">
+        <is>
+          <t>مذكور ضمن صياغات الحاجة ح7 ولا يوجد مقطع يجيب عنه مباشرة.</t>
+        </is>
+      </c>
+      <c r="F26" s="67" t="inlineStr">
+        <is>
+          <t>غير مغطى</t>
+        </is>
+      </c>
+      <c r="G26" s="67" t="inlineStr">
+        <is>
+          <t>إضافة مقتطف موثق إذا سيبقى السؤال ضمن الوعود النشطة.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="42" customHeight="1" s="49">
+      <c r="A27" s="94" t="inlineStr">
+        <is>
+          <t>ح1</t>
+        </is>
+      </c>
+      <c r="B27" s="94" t="inlineStr">
+        <is>
+          <t>هل القرآن مثل الإنجيل عند المسيحيين؟</t>
+        </is>
+      </c>
+      <c r="C27" s="94" t="inlineStr">
+        <is>
+          <t>مقارنة عامة ملتبسة وغير مغطاة مباشرة</t>
+        </is>
+      </c>
+      <c r="D27" s="94" t="inlineStr">
+        <is>
+          <t>متوسطة</t>
+        </is>
+      </c>
+      <c r="E27" s="94" t="inlineStr">
+        <is>
+          <t>ق-03 يشرح علاقة القرآن بالكتب السابقة، لا المقارنة بين دور القرآن عند المسلمين ودور الإنجيل عند المسيحيين.</t>
+        </is>
+      </c>
+      <c r="F27" s="94" t="inlineStr">
+        <is>
+          <t>غير مغطى مباشرة</t>
+        </is>
+      </c>
+      <c r="G27" s="94" t="inlineStr">
+        <is>
+          <t>CLARIFY حسب المقصود، أو NOT_COVERED إذا كان المقصود مقارنة الدور الديني العامة.</t>
+        </is>
+      </c>
+      <c r="H27" s="94" t="n"/>
+      <c r="I27" s="94" t="n"/>
+      <c r="J27" s="94" t="n"/>
+      <c r="K27" s="94" t="n"/>
+    </row>
+    <row r="28" ht="42" customHeight="1" s="49">
+      <c r="A28" s="93" t="inlineStr">
+        <is>
+          <t>ح2</t>
+        </is>
+      </c>
+      <c r="B28" s="93" t="inlineStr">
+        <is>
+          <t>ما هو الوحي؟</t>
+        </is>
+      </c>
+      <c r="C28" s="93" t="inlineStr">
+        <is>
+          <t>تعريف تأسيسي غير مباشر</t>
+        </is>
+      </c>
+      <c r="D28" s="93" t="inlineStr">
+        <is>
+          <t>عالية</t>
+        </is>
+      </c>
+      <c r="E28" s="93" t="inlineStr">
+        <is>
+          <t>ق-08 يشرح صور مجيء الوحي للنبي ﷺ، لكنه لا يقدم تعريفاً تمهيدياً مستقلاً لمفهوم الوحي.</t>
+        </is>
+      </c>
+      <c r="F28" s="93" t="inlineStr">
+        <is>
+          <t>جزئي</t>
+        </is>
+      </c>
+      <c r="G28" s="93" t="inlineStr">
+        <is>
+          <t>PARTIAL أو إضافة تعريف مباشر قبل توسيع الوعد.</t>
+        </is>
+      </c>
+      <c r="H28" s="93" t="n"/>
+      <c r="I28" s="93" t="n"/>
+      <c r="J28" s="93" t="n"/>
+      <c r="K28" s="93" t="n"/>
+    </row>
+    <row r="29" ht="42" customHeight="1" s="49">
+      <c r="A29" s="94" t="inlineStr">
+        <is>
+          <t>ح5</t>
+        </is>
+      </c>
+      <c r="B29" s="94" t="inlineStr">
+        <is>
+          <t>كيف نعرف أن قصص القرآن حقيقية؟</t>
+        </is>
+      </c>
+      <c r="C29" s="94" t="inlineStr">
+        <is>
+          <t>استدلال/اعتراض غير مغطى</t>
+        </is>
+      </c>
+      <c r="D29" s="94" t="inlineStr">
+        <is>
+          <t>متوسطة</t>
+        </is>
+      </c>
+      <c r="E29" s="94" t="inlineStr">
+        <is>
+          <t>ق-06 يعرّف القصص وأنواعها وغاياتها، لكنه لا يقدم دليلاً مستقلاً لمن يطلب إثبات تاريخيتها.</t>
+        </is>
+      </c>
+      <c r="F29" s="94" t="inlineStr">
+        <is>
+          <t>غير مغطى</t>
+        </is>
+      </c>
+      <c r="G29" s="94" t="inlineStr">
+        <is>
+          <t>NOT_COVERED ضمن النسخة الحالية ما لم تضاف مادة استدلالية مستقلة.</t>
+        </is>
+      </c>
+      <c r="H29" s="94" t="n"/>
+      <c r="I29" s="94" t="n"/>
+      <c r="J29" s="94" t="n"/>
+      <c r="K29" s="94" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="95" t="inlineStr">
+        <is>
+          <t>ح1</t>
+        </is>
+      </c>
+      <c r="B30" s="95" t="inlineStr">
+        <is>
+          <t>هل القرآن مثل الإنجيل عند المسيحيين؟</t>
+        </is>
+      </c>
+      <c r="C30" s="95" t="inlineStr">
+        <is>
+          <t>مقارنة غير مغطاة</t>
+        </is>
+      </c>
+      <c r="D30" s="95" t="inlineStr">
+        <is>
+          <t>متوسطة</t>
+        </is>
+      </c>
+      <c r="E30" s="95" t="inlineStr">
+        <is>
+          <t>v22: ق-03 يستبعدها صراحة؛ يجيب عن صلة القرآن بالكتب السابقة لا عن مقارنة دوره بدور الإنجيل.</t>
+        </is>
+      </c>
+      <c r="F30" s="95" t="inlineStr">
+        <is>
+          <t>غير مغطى</t>
+        </is>
+      </c>
+      <c r="G30" s="95" t="inlineStr">
+        <is>
+          <t>حُذفت من صياغات ح1 النشطة؛ تُضاف مادة مقارنة مباشرة أو يبقى الامتناع.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="95" t="inlineStr">
+        <is>
+          <t>ح2</t>
+        </is>
+      </c>
+      <c r="B31" s="95" t="inlineStr">
+        <is>
+          <t>ما هو الوحي؟ (تعريف تمهيدي مباشر)</t>
+        </is>
+      </c>
+      <c r="C31" s="95" t="inlineStr">
+        <is>
+          <t>تعريف مفقود</t>
+        </is>
+      </c>
+      <c r="D31" s="95" t="inlineStr">
+        <is>
+          <t>متوسطة</t>
+        </is>
+      </c>
+      <c r="E31" s="95" t="inlineStr">
+        <is>
+          <t>v22: حُذفت من صياغات ق-08؛ ق-08 يشرح صور الوحي لا تعريفه.</t>
+        </is>
+      </c>
+      <c r="F31" s="95" t="inlineStr">
+        <is>
+          <t>غير مغطى</t>
+        </is>
+      </c>
+      <c r="G31" s="95" t="inlineStr">
+        <is>
+          <t>إضافة مقتطف تعريفي أو الامتناع.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="95" t="inlineStr">
+        <is>
+          <t>ح5</t>
+        </is>
+      </c>
+      <c r="B32" s="95" t="inlineStr">
+        <is>
+          <t>كيف نعرف أن قصص القرآن حقيقية؟ (إثبات تاريخيتها)</t>
+        </is>
+      </c>
+      <c r="C32" s="95" t="inlineStr">
+        <is>
+          <t>استدلال مفقود</t>
+        </is>
+      </c>
+      <c r="D32" s="95" t="inlineStr">
+        <is>
+          <t>متوسطة</t>
+        </is>
+      </c>
+      <c r="E32" s="95" t="inlineStr">
+        <is>
+          <t>ق-06 يعامل القصص وقائع ولا يقدم دليلاً مستقلاً؛ السؤال الأبسط PARTIAL بـ ق-06.</t>
+        </is>
+      </c>
+      <c r="F32" s="95" t="inlineStr">
+        <is>
+          <t>غير مغطى</t>
+        </is>
+      </c>
+      <c r="G32" s="95" t="inlineStr">
+        <is>
+          <t>إضافة مادة استدلالية أو الامتناع.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="95" t="inlineStr">
+        <is>
+          <t>ح7</t>
+        </is>
+      </c>
+      <c r="B33" s="95" t="inlineStr">
+        <is>
+          <t>لماذا تتشابه قصص القرآن مع الكتب السابقة؟</t>
+        </is>
+      </c>
+      <c r="C33" s="95" t="inlineStr">
+        <is>
+          <t>شرح مفقود</t>
+        </is>
+      </c>
+      <c r="D33" s="95" t="inlineStr">
+        <is>
+          <t>متوسطة</t>
+        </is>
+      </c>
+      <c r="E33" s="95" t="inlineStr">
+        <is>
+          <t>ق-25 يرد على دعوى الاقتباس ولا يشرح سبب التشابه (منع صريح في v23).</t>
+        </is>
+      </c>
+      <c r="F33" s="95" t="inlineStr">
+        <is>
+          <t>غير مغطى</t>
+        </is>
+      </c>
+      <c r="G33" s="95" t="inlineStr">
+        <is>
+          <t>إضافة مادة أو الامتناع.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A2:K2"/>
+    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="A15:G15"/>
+  </mergeCells>
+  <conditionalFormatting sqref="D17:D26">
+    <cfRule type="expression" priority="1" dxfId="0">
+      <formula>D17="عالية"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="2">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1594,7 +2718,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4256,6 +5380,999 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E36"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" style="49" min="1" max="1"/>
+    <col width="8" customWidth="1" style="49" min="2" max="2"/>
+    <col width="22" customWidth="1" style="49" min="3" max="3"/>
+    <col width="60" customWidth="1" style="49" min="4" max="4"/>
+    <col width="60" customWidth="1" style="49" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>النسخة</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>المقطع</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>الحقل</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>التغيير</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>السبب</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>v22</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>النص المرجعي</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>0 تغييرات في المقاطع الـ34</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>تدقيق «تدقيق 34»</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>v22</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>ق-03</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>صياغات المستخدم</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>قبل: هل القرآن مثل الإنجيل عند المسيحيين؟ | ما علاقة القرآن بالتوراة والإنجيل؟ | ما معنى أن القرآن مهيمن؟ ← بعد: ما علاقة القرآن بالتوراة والإنجيل؟ | ما معنى أن القرآن مهيمن؟</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>تدقيق v22</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>v22</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>ق-03</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>EVIDENCE_LIMITS</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>قبل: يشرح صلة القرآن بالكتب السابقة إجمالاً، ولا يعالج وحده دعوى الاقتباس أو الفرق بين القرآن والحديث. ← بعد: يشرح صلة القرآن بالكتب السابقة إجمالاً، ولا يعالج وحده دعوى الاقتباس أو الفرق بين القرآن والحديث. ولا يقارن دور القرآن عند المسلمين بدور الإنجيل عند ا</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>تدقيق v22</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>v22</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>ق-03</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>أسئلة قريبة لا يجيب عنها</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>قبل: هل نقل محمد القرآن من التوراة؟ | ما الفرق بين القرآن والحديث؟ ← بعد: هل نقل محمد القرآن من التوراة؟ | ما الفرق بين القرآن والحديث؟ | هل القرآن مثل الإنجيل عند المسيحيين؟</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>تدقيق v22</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>v22</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>ق-06</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>صياغات المستخدم</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>قبل: هل القرآن فيه قصص؟ | هل يذكر القرآن موسى وعيسى؟ | ليش القرآن يحكي قصص الأنبياء؟ | هل قصص القرآن حقيقية؟ ← بعد: هل القرآن فيه قصص؟ | هل يذكر القرآن موسى وعيسى؟ | ليش القرآن يحكي قصص الأنبياء؟</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>تدقيق v22</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>v22</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>ق-06</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>EVIDENCE_LIMITS</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>قبل: يبين وجود القصص في القرآن وغايتها إجمالاً، ولا يسرد قصة نبي بالتفصيل أو يناقش مصدر القصص. ← بعد: يبين وجود القصص في القرآن وغايتها إجمالاً، ولا يسرد قصة نبي بالتفصيل أو يناقش مصدر القصص. ولا يقدم استدلالاً مستقلاً على تاريخية القصص لمن يطلب إثباته</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>تدقيق v22</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>v22</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>ق-06</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>أسئلة قريبة لا يجيب عنها</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>قبل: ما قصة نوح بالتفصيل؟ | هل قصص القرآن منقولة من التوراة؟ ← بعد: ما قصة نوح بالتفصيل؟ | هل قصص القرآن منقولة من التوراة؟ | كيف نعرف أن قصص القرآن حقيقية؟</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>تدقيق v22</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>v22</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>ق-08</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>صياغات المستخدم</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">قبل: كيف كان الوحي يأتي النبي؟ | ما هو الوحي؟ | كيف وصل القرآن لمحمد؟ | كيف كان جبريل ينزل بالقرآن؟ | ما طرق نزول الوحي على النبي؟ | هل كان جبريل يأتي النب ← بعد: كيف كان الوحي يأتي النبي؟ | كيف وصل القرآن لمحمد؟ | كيف كان جبريل ينزل بالقرآن؟ | ما طرق نزول الوحي على النبي؟ | هل كان جبريل يأتي النبي في صورة رجل؟ </t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>تدقيق v22</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>v22</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>ق-08</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>EVIDENCE_LIMITS</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>قبل: يشرح صور مجيء الوحي للنبي ﷺ، ولا يحدد زمن النزول أو يجيب عن حكمة خفاء الوحي. ← بعد: يشرح صور مجيء الوحي للنبي ﷺ، ولا يحدد زمن النزول أو يجيب عن حكمة خفاء الوحي. ولا يقدم تعريفاً تمهيدياً مستقلاً لمفهوم الوحي.</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>تدقيق v22</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>v22</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>ق-09</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>صياغات المستخدم</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>قبل: متى نزل القرآن؟ | في أي شهر نزل القرآن؟ | ما علاقة القرآن برمضان؟ ← بعد: في أي شهر نزل القرآن؟ | ما علاقة القرآن برمضان؟</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>تدقيق v22</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>v22</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>ق-09</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>PRIMARY_TASK</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>قبل: تعريف ← بعد: شرح</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>تدقيق v22</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>v22</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>ق-09</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>TASK_TYPES</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>قبل: شرح ← بعد: —</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>تدقيق v22</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>v22</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>ق-09</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>EVIDENCE_LIMITS</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">قبل: يثبت ارتباط نزول القرآن برمضان، ولا يشرح صور الوحي أو كيفية النزول المفرق. ← بعد: يثبت ارتباط نزول القرآن برمضان، ولا يشرح صور الوحي أو كيفية النزول المفرق. والسؤال العام «متى نزل القرآن؟» يحتاج تحديد المقصود: الشهر أو بداية النزول </t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>تدقيق v22</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>v22</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>ق-14</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>صياغات المستخدم</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>قبل: كم عدد الصحابة الذين حفظوا القرآن؟ | هل نُقل القرآن عن عدد قليل؟ ← بعد: هل نُقل القرآن عن عدد قليل؟</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>تدقيق v22</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>v22</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>ق-14</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>أسئلة قريبة لا يجيب عنها</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>قبل: كيف جمع عثمان القرآن؟ | كيف أحفظ القرآن؟ ← بعد: كيف جمع عثمان القرآن؟ | كيف أحفظ القرآن؟ | كم كان عدد حفظة القرآن من الصحابة تحديداً؟</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>تدقيق v22</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>v22</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>ق-20</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>صياغات المستخدم</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>قبل: هل الترجمة تعتبر قرآناً؟ | أقدر أقرأ القرآن بالإنجليزي؟ | ما الفرق بين القرآن وترجمة معانيه؟ | ليش يقولون ترجمة معاني القرآن؟ ← بعد: هل الترجمة تعتبر قرآناً؟ | ما الفرق بين القرآن وترجمة معانيه؟ | ليش يقولون ترجمة معاني القرآن؟</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>تدقيق v22</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>v22</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>ق-20</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>EVIDENCE_LIMITS</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>قبل: يبين الفرق بين القرآن وترجمة معانيه وحكم الترجمة الحرفية في النص، ولا يحدد أفضل ترجمة أو يفتي في الصلاة بالترجمة. ← بعد: يبين الفرق بين القرآن وترجمة معانيه وحكم الترجمة الحرفية في النص، ولا يحدد أفضل ترجمة أو يفتي في الصلاة بالترجمة. وصيغة «القراءة بالإنجليزية» ملتبسة ب</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>تدقيق v22</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>v22</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>ق-24</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>أسئلة قريبة لا يجيب عنها</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>قبل: ما هو القرآن؟ | ما مكانة القرآن؟ | كيف كان الوحي ينزل؟ ← بعد: ما هو القرآن؟ | ما مكانة القرآن؟ | كيف كان الوحي ينزل؟ | ما أمثلة الإعجاز العلمي؟</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>تدقيق v22</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>v22</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>ق-25</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>صياغات المستخدم</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>قبل: هل نقل محمد القرآن من التوراة والإنجيل؟ | لماذا تتشابه قصص القرآن مع الكتب السابقة؟ | هل القرآن مقتبس؟ ← بعد: هل نقل محمد القرآن من التوراة والإنجيل؟ | هل القرآن مقتبس؟</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>تدقيق v22</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>v22</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>ق-25</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>EVIDENCE_LIMITS</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>قبل: يعالج دعوى الاقتباس من الكتب السابقة إجمالاً، ولا يشرح كل أوجه التشابه أو تاريخ النصوص السابقة. ← بعد: يعالج دعوى الاقتباس من الكتب السابقة إجمالاً، ولا يشرح كل أوجه التشابه أو تاريخ النصوص السابقة. ولا يشرح سبب وجود أوجه تشابه بين بعض القصص؛ بل يعالج د</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>تدقيق v22</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>v22</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>ق-25</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>أسئلة قريبة لا يجيب عنها</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>قبل: ما معنى أن القرآن مهيمن على الكتب السابقة؟ | ما قصص الأنبياء في القرآن؟ ← بعد: ما معنى أن القرآن مهيمن على الكتب السابقة؟ | ما قصص الأنبياء في القرآن؟ | ما سبب تشابه بعض قصص القرآن مع الكتب السابقة؟</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>تدقيق v22</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>v22</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>ق-26</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>أسئلة قريبة لا يجيب عنها</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>قبل: كيف جُمع القرآن؟ | ما أسباب نزول آية بعينها؟ ← بعد: كيف جُمع القرآن؟ | ما أسباب نزول آية بعينها؟ | ما أمثلة الإعجاز العلمي؟</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>تدقيق v22</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>v22</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>ق-29</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>EVIDENCE_LIMITS</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>قبل: يعالج دعوى أن اختلاف اللين والشدة سببه تأثر بشري بالبيئة، ولا يشرح تعريف المكي والمدني ولا تاريخ النزول. ← بعد: يعالج دعوى أن اختلاف اللين والشدة سببه تأثر بشري بالبيئة، ولا يشرح تعريف المكي والمدني ولا تاريخ النزول. ولا يقدم مقارنة شاملة لجميع خصائص الأسلوب الم</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>تدقيق v22</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>v22</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>ق-29</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>أسئلة قريبة لا يجيب عنها</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>قبل: كيف نزل القرآن؟ | في أي شهر نزل القرآن؟ | ما معنى سورة مكية؟ | ما الفرق بين أسلوب السور المكية والمدنية؟ ← بعد: كيف نزل القرآن؟ | في أي شهر نزل القرآن؟ | ما معنى سورة مكية؟</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>تدقيق v22</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>v22</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>ق-32</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>EVIDENCE_LIMITS</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>قبل: يثبت حاجة الدين إلى السنة وحجيتها بوصفها مبيِّنة للقرآن، ولا يقدّم تفصيلاً في علوم الحديث أو حجية كل نوع من أنواع السنة. ← بعد: يثبت حاجة الدين إلى السنة وحجيتها بوصفها مبيِّنة للقرآن، ولا يقدّم تفصيلاً في علوم الحديث أو حجية كل نوع من أنواع السنة. وقد يفيد جزئياً في سؤال علاقة</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>تدقيق v22</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>v22</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>ق-32</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>أسئلة قريبة لا يجيب عنها</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>قبل: ما علاقة القرآن بالكتب السابقة؟ | ما تعريف القرآن؟ | ما مكانة القرآن عند المسلمين؟ | ما علاقة الحديث بالقرآن؟ | ما الفرق بين القرآن والحديث؟ ← بعد: ما علاقة القرآن بالكتب السابقة؟ | ما تعريف القرآن؟ | ما مكانة القرآن عند المسلمين؟ | ما الفرق بين القرآن والحديث؟</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>تدقيق v22</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>v22</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>ق-37</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>صياغات المستخدم</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>قبل: هل نزل القرآن مرة واحدة؟ | لماذا نزل القرآن مفرّقاً؟ | كم مرة نزل القرآن؟ ← بعد: هل نزل القرآن مرة واحدة؟ | لماذا نزل القرآن مفرّقاً؟</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>تدقيق v22</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>v22</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>ق-37</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>EVIDENCE_LIMITS</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>قبل: يشرح أن القرآن نزل مفرقاً بحسب الوقائع، ولا يحدد شهر النزول أو صور مجيء الوحي. ← بعد: يشرح أن القرآن نزل مفرقاً بحسب الوقائع، ولا يحدد شهر النزول أو صور مجيء الوحي. ولا يحدد عدداً معيناً لمرات النزول.</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>تدقيق v22</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>v22</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>ق-37</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>أسئلة قريبة لا يجيب عنها</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>قبل: في أي شهر نزل القرآن؟ | كيف كان الوحي يأتي النبي؟ ← بعد: في أي شهر نزل القرآن؟ | كيف كان الوحي يأتي النبي؟ | كم مرة تحديداً نزل القرآن؟</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>تدقيق v22</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>v23</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>ق-06</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>أسئلة قريبة لا يجيب عنها</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>أُضيف «ما الدليل على أن قصص القرآن حقيقية؟»</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>طلب الدليل NOT_COVERED؛ والسؤال الأبسط «هل قصص القرآن حقيقية؟» PARTIAL بلا منع</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>v23</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>ق-14</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>أسئلة قريبة لا يجيب عنها</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>حُذف «كم كان عدد حفظة القرآن من الصحابة تحديداً؟»</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>السؤال عن العدد PARTIAL بـ ق-14 لا منع؛ والقيد في الحدود</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>v23</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>ق-25</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>أسئلة قريبة لا يجيب عنها</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>أُضيف «لماذا تتشابه قصص القرآن مع الكتب السابقة؟»</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>NOT_COVERED: يرد على دعوى الاقتباس ولا يشرح سبب التشابه</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>v23</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>ح1</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>صياغات المستخدم</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>أُعيد «هل القرآن مثل الإنجيل عند المسيحيين؟» موسوماً [فجوة]</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>حاجة حقيقية غير مغطاة؛ لا تُصدَّر للموجّه</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>v23</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>منطق المحادثة</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>ست-07 وست-08 بخياراتهما (مرجعية، غير مفعّلة)</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>الحقيقة المرجعية CLARIFY لـ«متى نزل القرآن؟» و«أقدر أقرأ بالإنجليزي؟»</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>v23</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>النص المرجعي</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>0 تغييرات</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5826,7 +7943,7 @@
       </c>
       <c r="Y12" s="67" t="inlineStr">
         <is>
-          <t>ما قصة نوح بالتفصيل؟ | هل قصص القرآن منقولة من التوراة؟ | كيف نعرف أن قصص القرآن حقيقية؟</t>
+          <t>ما قصة نوح بالتفصيل؟ | هل قصص القرآن منقولة من التوراة؟ | كيف نعرف أن قصص القرآن حقيقية؟ | ما الدليل على أن قصص القرآن حقيقية؟</t>
         </is>
       </c>
       <c r="Z12" s="67" t="inlineStr">
@@ -7604,17 +9721,17 @@
       </c>
       <c r="W23" s="67" t="inlineStr">
         <is>
-          <t>يرد على دعوى قلة ناقلي القرآن ويبين كثرة الحفاظ، ولا يقدم إحصاءً حصرياً أو شرحاً كاملاً لعلم التواتر.</t>
+          <t>يرد على دعوى قلة ناقلي القرآن ويبين كثرة الحفاظ، ولا يقدم إحصاءً حصرياً أو شرحاً كاملاً لعلم التواتر. لا يقدم عددًا حصريًا محددًا لحفاظ القرآن من الصحابة.</t>
         </is>
       </c>
       <c r="X23" s="67" t="inlineStr">
         <is>
-          <t>لا يشرح جمع عثمان ولا كيفية حفظ القرآن عملياً.</t>
+          <t>لا يشرح جمع عثمان ولا كيفية حفظ القرآن عملياً. لا يقدم عددًا حصريًا محددًا لحفاظ القرآن من الصحابة.</t>
         </is>
       </c>
       <c r="Y23" s="67" t="inlineStr">
         <is>
-          <t>كيف جمع عثمان القرآن؟ | كيف أحفظ القرآن؟ | كم كان عدد حفظة القرآن من الصحابة تحديداً؟</t>
+          <t>كيف جمع عثمان القرآن؟ | كيف أحفظ القرآن؟</t>
         </is>
       </c>
       <c r="Z23" s="67" t="inlineStr">
@@ -9736,12 +11853,12 @@
       </c>
       <c r="X36" s="67" t="inlineStr">
         <is>
-          <t>لا يشرح معنى هيمنة القرآن على الكتب السابقة ولا يسرد قصص الأنبياء.</t>
+          <t>لا يشرح معنى هيمنة القرآن على الكتب السابقة ولا يسرد قصص الأنبياء. لا يشرح سبب أوجه التشابه بين بعض قصص القرآن والكتب السابقة.</t>
         </is>
       </c>
       <c r="Y36" s="67" t="inlineStr">
         <is>
-          <t>ما معنى أن القرآن مهيمن على الكتب السابقة؟ | ما قصص الأنبياء في القرآن؟ | ما سبب تشابه بعض قصص القرآن مع الكتب السابقة؟</t>
+          <t>ما معنى أن القرآن مهيمن على الكتب السابقة؟ | ما قصص الأنبياء في القرآن؟ | ما سبب تشابه بعض قصص القرآن مع الكتب السابقة؟ | لماذا تتشابه قصص القرآن مع الكتب السابقة؟</t>
         </is>
       </c>
       <c r="Z36" s="67" t="inlineStr">
@@ -10138,9 +12255,9 @@
   </sheetData>
   <mergeCells count="6">
     <mergeCell ref="A2:AH2"/>
-    <mergeCell ref="N3:AA3"/>
     <mergeCell ref="A3:D3"/>
     <mergeCell ref="AB3:AH3"/>
+    <mergeCell ref="N3:AA3"/>
     <mergeCell ref="A1:AH1"/>
     <mergeCell ref="E3:M3"/>
   </mergeCells>
@@ -10161,7 +12278,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -10335,7 +12452,7 @@
       </c>
       <c r="F5" s="67" t="inlineStr">
         <is>
-          <t>«ما هو القرآن؟» · «إيش يعني القرآن؟» · «ليش المسلمين يقدّسون القرآن؟» · «ما الفرق بين القرآن والحديث؟» · «لماذا يقرأ المسلمون القرآن كثيراً؟»</t>
+          <t>«ما هو القرآن؟» · «إيش يعني القرآن؟» · «ليش المسلمين يقدّسون القرآن؟» · «ما الفرق بين القرآن والحديث؟» · «لماذا يقرأ المسلمون القرآن كثيراً؟» · «هل القرآن مثل الإنجيل عند المسيحيين؟» [فجوة]</t>
         </is>
       </c>
       <c r="G5" s="67" t="inlineStr">
@@ -10844,7 +12961,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -11155,13 +13272,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H44"/>
+  <dimension ref="A1:H52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" style="49" min="1" max="1"/>
@@ -12925,6 +15042,342 @@
         </is>
       </c>
     </row>
+    <row r="45" ht="58" customHeight="1" s="49">
+      <c r="A45" s="37" t="inlineStr">
+        <is>
+          <t>ست-07</t>
+        </is>
+      </c>
+      <c r="B45" s="37" t="inlineStr">
+        <is>
+          <t>CLARIFY (مرجعي)</t>
+        </is>
+      </c>
+      <c r="C45" s="37" t="inlineStr">
+        <is>
+          <t>CLARIFY: الشهر أو بداية النزول أو مدته</t>
+        </is>
+      </c>
+      <c r="D45" s="37" t="inlineStr">
+        <is>
+          <t>سؤال «متى نزل القرآن؟» العام</t>
+        </is>
+      </c>
+      <c r="E45" s="37" t="inlineStr">
+        <is>
+          <t>ماذا تقصد بـ«متى نزل القرآن»؟</t>
+        </is>
+      </c>
+      <c r="F45" s="37" t="inlineStr">
+        <is>
+          <t>لا</t>
+        </is>
+      </c>
+      <c r="G45" s="37" t="inlineStr">
+        <is>
+          <t>محمد — 5 أكتوبر 2026</t>
+        </is>
+      </c>
+      <c r="H45" s="37" t="inlineStr">
+        <is>
+          <t>مرجعي — غير مفعّل برمجياً في v1.0؛ يحدد الحقيقة المرجعية (CLARIFY) ويُفعَّل في إصدار لاحق بعد قياس.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="58" customHeight="1" s="49">
+      <c r="A46" s="37" t="inlineStr">
+        <is>
+          <t>ست-07-1</t>
+        </is>
+      </c>
+      <c r="B46" s="37" t="inlineStr">
+        <is>
+          <t>CLARIFY (مرجعي)</t>
+        </is>
+      </c>
+      <c r="C46" s="37" t="inlineStr">
+        <is>
+          <t>خيار ← ق-09</t>
+        </is>
+      </c>
+      <c r="D46" s="37" t="inlineStr">
+        <is>
+          <t>الخيار الأول في ست-07 ← ق-09</t>
+        </is>
+      </c>
+      <c r="E46" s="37" t="inlineStr">
+        <is>
+          <t>في أي شهر نزل القرآن؟</t>
+        </is>
+      </c>
+      <c r="F46" s="37" t="inlineStr">
+        <is>
+          <t>لا</t>
+        </is>
+      </c>
+      <c r="G46" s="37" t="inlineStr">
+        <is>
+          <t>محمد — 5 أكتوبر 2026</t>
+        </is>
+      </c>
+      <c r="H46" s="37" t="inlineStr">
+        <is>
+          <t>مرجعي — غير مفعّل برمجياً في v1.0؛ يحدد الحقيقة المرجعية (CLARIFY) ويُفعَّل في إصدار لاحق بعد قياس.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="58" customHeight="1" s="49">
+      <c r="A47" s="37" t="inlineStr">
+        <is>
+          <t>ست-07-2</t>
+        </is>
+      </c>
+      <c r="B47" s="37" t="inlineStr">
+        <is>
+          <t>CLARIFY (مرجعي)</t>
+        </is>
+      </c>
+      <c r="C47" s="37" t="inlineStr">
+        <is>
+          <t>خيار ← غير مغطى</t>
+        </is>
+      </c>
+      <c r="D47" s="37" t="inlineStr">
+        <is>
+          <t>الخيار الثاني في ست-07 ← NOT_COVERED حالياً</t>
+        </is>
+      </c>
+      <c r="E47" s="37" t="inlineStr">
+        <is>
+          <t>متى بدأ نزول القرآن أول مرة؟</t>
+        </is>
+      </c>
+      <c r="F47" s="37" t="inlineStr">
+        <is>
+          <t>لا</t>
+        </is>
+      </c>
+      <c r="G47" s="37" t="inlineStr">
+        <is>
+          <t>محمد — 5 أكتوبر 2026</t>
+        </is>
+      </c>
+      <c r="H47" s="37" t="inlineStr">
+        <is>
+          <t>مرجعي — غير مفعّل برمجياً في v1.0؛ يحدد الحقيقة المرجعية (CLARIFY) ويُفعَّل في إصدار لاحق بعد قياس.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="58" customHeight="1" s="49">
+      <c r="A48" s="37" t="inlineStr">
+        <is>
+          <t>ست-07-3</t>
+        </is>
+      </c>
+      <c r="B48" s="37" t="inlineStr">
+        <is>
+          <t>CLARIFY (مرجعي)</t>
+        </is>
+      </c>
+      <c r="C48" s="37" t="inlineStr">
+        <is>
+          <t>خيار ← غير مغطى</t>
+        </is>
+      </c>
+      <c r="D48" s="37" t="inlineStr">
+        <is>
+          <t>الخيار الثالث في ست-07 ← NOT_COVERED حالياً</t>
+        </is>
+      </c>
+      <c r="E48" s="37" t="inlineStr">
+        <is>
+          <t>كم سنة استمر نزول القرآن؟</t>
+        </is>
+      </c>
+      <c r="F48" s="37" t="inlineStr">
+        <is>
+          <t>لا</t>
+        </is>
+      </c>
+      <c r="G48" s="37" t="inlineStr">
+        <is>
+          <t>محمد — 5 أكتوبر 2026</t>
+        </is>
+      </c>
+      <c r="H48" s="37" t="inlineStr">
+        <is>
+          <t>مرجعي — غير مفعّل برمجياً في v1.0؛ يحدد الحقيقة المرجعية (CLARIFY) ويُفعَّل في إصدار لاحق بعد قياس.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="58" customHeight="1" s="49">
+      <c r="A49" s="37" t="inlineStr">
+        <is>
+          <t>ست-08</t>
+        </is>
+      </c>
+      <c r="B49" s="37" t="inlineStr">
+        <is>
+          <t>CLARIFY (مرجعي)</t>
+        </is>
+      </c>
+      <c r="C49" s="37" t="inlineStr">
+        <is>
+          <t>CLARIFY: الفهم أو حكم الترجمة أو العبادة</t>
+        </is>
+      </c>
+      <c r="D49" s="37" t="inlineStr">
+        <is>
+          <t>سؤال «أقدر أقرأ القرآن بالإنجليزي؟» وما في معناه</t>
+        </is>
+      </c>
+      <c r="E49" s="37" t="inlineStr">
+        <is>
+          <t>ماذا تقصد بالقراءة بالإنجليزية؟</t>
+        </is>
+      </c>
+      <c r="F49" s="37" t="inlineStr">
+        <is>
+          <t>لا</t>
+        </is>
+      </c>
+      <c r="G49" s="37" t="inlineStr">
+        <is>
+          <t>محمد — 5 أكتوبر 2026</t>
+        </is>
+      </c>
+      <c r="H49" s="37" t="inlineStr">
+        <is>
+          <t>مرجعي — غير مفعّل برمجياً في v1.0؛ يحدد الحقيقة المرجعية (CLARIFY) ويُفعَّل في إصدار لاحق بعد قياس.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="58" customHeight="1" s="49">
+      <c r="A50" s="37" t="inlineStr">
+        <is>
+          <t>ست-08-1</t>
+        </is>
+      </c>
+      <c r="B50" s="37" t="inlineStr">
+        <is>
+          <t>CLARIFY (مرجعي)</t>
+        </is>
+      </c>
+      <c r="C50" s="37" t="inlineStr">
+        <is>
+          <t>خيار ← ق-20</t>
+        </is>
+      </c>
+      <c r="D50" s="37" t="inlineStr">
+        <is>
+          <t>الخيار الأول في ست-08 ← ق-20</t>
+        </is>
+      </c>
+      <c r="E50" s="37" t="inlineStr">
+        <is>
+          <t>قراءة ترجمة معاني القرآن للفهم؟</t>
+        </is>
+      </c>
+      <c r="F50" s="37" t="inlineStr">
+        <is>
+          <t>لا</t>
+        </is>
+      </c>
+      <c r="G50" s="37" t="inlineStr">
+        <is>
+          <t>محمد — 5 أكتوبر 2026</t>
+        </is>
+      </c>
+      <c r="H50" s="37" t="inlineStr">
+        <is>
+          <t>مرجعي — غير مفعّل برمجياً في v1.0؛ يحدد الحقيقة المرجعية (CLARIFY) ويُفعَّل في إصدار لاحق بعد قياس.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="58" customHeight="1" s="49">
+      <c r="A51" s="37" t="inlineStr">
+        <is>
+          <t>ست-08-2</t>
+        </is>
+      </c>
+      <c r="B51" s="37" t="inlineStr">
+        <is>
+          <t>CLARIFY (مرجعي)</t>
+        </is>
+      </c>
+      <c r="C51" s="37" t="inlineStr">
+        <is>
+          <t>خيار ← ق-20</t>
+        </is>
+      </c>
+      <c r="D51" s="37" t="inlineStr">
+        <is>
+          <t>الخيار الثاني في ست-08 ← ق-20</t>
+        </is>
+      </c>
+      <c r="E51" s="37" t="inlineStr">
+        <is>
+          <t>هل الترجمة الإنجليزية نفسها تُعد قرآنًا؟</t>
+        </is>
+      </c>
+      <c r="F51" s="37" t="inlineStr">
+        <is>
+          <t>لا</t>
+        </is>
+      </c>
+      <c r="G51" s="37" t="inlineStr">
+        <is>
+          <t>محمد — 5 أكتوبر 2026</t>
+        </is>
+      </c>
+      <c r="H51" s="37" t="inlineStr">
+        <is>
+          <t>مرجعي — غير مفعّل برمجياً في v1.0؛ يحدد الحقيقة المرجعية (CLARIFY) ويُفعَّل في إصدار لاحق بعد قياس.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="58" customHeight="1" s="49">
+      <c r="A52" s="37" t="inlineStr">
+        <is>
+          <t>ست-08-3</t>
+        </is>
+      </c>
+      <c r="B52" s="37" t="inlineStr">
+        <is>
+          <t>CLARIFY (مرجعي)</t>
+        </is>
+      </c>
+      <c r="C52" s="37" t="inlineStr">
+        <is>
+          <t>خيار ← إحالة (ام-02)</t>
+        </is>
+      </c>
+      <c r="D52" s="37" t="inlineStr">
+        <is>
+          <t>الخيار الثالث في ست-08 ← REFER</t>
+        </is>
+      </c>
+      <c r="E52" s="37" t="inlineStr">
+        <is>
+          <t>القراءة بالإنجليزية في الصلاة أو العبادة؟</t>
+        </is>
+      </c>
+      <c r="F52" s="37" t="inlineStr">
+        <is>
+          <t>لا</t>
+        </is>
+      </c>
+      <c r="G52" s="37" t="inlineStr">
+        <is>
+          <t>محمد — 5 أكتوبر 2026</t>
+        </is>
+      </c>
+      <c r="H52" s="37" t="inlineStr">
+        <is>
+          <t>مرجعي — غير مفعّل برمجياً في v1.0؛ يحدد الحقيقة المرجعية (CLARIFY) ويُفعَّل في إصدار لاحق بعد قياس.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A2:H2"/>
@@ -12937,7 +15390,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -13124,7 +15577,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -13184,7 +15637,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -13264,993 +15717,4 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:K30"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="10" customWidth="1" style="49" min="1" max="1"/>
-    <col width="38" customWidth="1" style="49" min="2" max="2"/>
-    <col width="25" customWidth="1" style="49" min="3" max="3"/>
-    <col width="12" customWidth="1" style="49" min="4" max="4"/>
-    <col width="55" customWidth="1" style="49" min="5" max="5"/>
-    <col width="18" customWidth="1" style="49" min="6" max="6"/>
-    <col width="45" customWidth="1" style="49" min="7" max="7"/>
-    <col width="14" customWidth="1" style="49" min="8" max="8"/>
-    <col width="14" customWidth="1" style="49" min="9" max="9"/>
-    <col width="14" customWidth="1" style="49" min="10" max="10"/>
-    <col width="48" customWidth="1" style="49" min="11" max="11"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="9" t="inlineStr">
-        <is>
-          <t>Coverage Map — مصفوفة التغطية وفجوات النسخة الحالية</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="n"/>
-      <c r="C1" s="1" t="n"/>
-      <c r="D1" s="1" t="n"/>
-      <c r="E1" s="1" t="n"/>
-      <c r="F1" s="1" t="n"/>
-      <c r="G1" s="1" t="n"/>
-      <c r="H1" s="1" t="n"/>
-      <c r="I1" s="1" t="n"/>
-      <c r="J1" s="1" t="n"/>
-      <c r="K1" s="1" t="n"/>
-    </row>
-    <row r="2">
-      <c r="A2" s="19" t="inlineStr">
-        <is>
-          <t>العدد لا يعني جودة التغطية وحده؛ الفجوات أدناه مبنية على مقارنة صياغات الاحتياجات بما تجيب عنه المقاطع وما تستبعده صراحة.</t>
-        </is>
-      </c>
-      <c r="B2" s="1" t="n"/>
-      <c r="C2" s="1" t="n"/>
-      <c r="D2" s="1" t="n"/>
-      <c r="E2" s="1" t="n"/>
-      <c r="F2" s="1" t="n"/>
-      <c r="G2" s="1" t="n"/>
-      <c r="H2" s="1" t="n"/>
-      <c r="I2" s="1" t="n"/>
-      <c r="J2" s="1" t="n"/>
-      <c r="K2" s="1" t="n"/>
-    </row>
-    <row r="3"/>
-    <row r="4">
-      <c r="A4" s="63" t="inlineStr">
-        <is>
-          <t>الحاجة</t>
-        </is>
-      </c>
-      <c r="B4" s="63" t="inlineStr">
-        <is>
-          <t>عدد المقاطع</t>
-        </is>
-      </c>
-      <c r="C4" s="63" t="inlineStr">
-        <is>
-          <t>تعريف</t>
-        </is>
-      </c>
-      <c r="D4" s="63" t="inlineStr">
-        <is>
-          <t>شرح</t>
-        </is>
-      </c>
-      <c r="E4" s="63" t="inlineStr">
-        <is>
-          <t>تعليم</t>
-        </is>
-      </c>
-      <c r="F4" s="63" t="inlineStr">
-        <is>
-          <t>استدلال</t>
-        </is>
-      </c>
-      <c r="G4" s="63" t="inlineStr">
-        <is>
-          <t>معالجة اعتراض</t>
-        </is>
-      </c>
-      <c r="H4" s="63" t="inlineStr">
-        <is>
-          <t>مقارنة</t>
-        </is>
-      </c>
-      <c r="I4" s="63" t="inlineStr">
-        <is>
-          <t>بحث أو تحقيق</t>
-        </is>
-      </c>
-      <c r="J4" s="63" t="inlineStr">
-        <is>
-          <t>توجيه عملي</t>
-        </is>
-      </c>
-      <c r="K4" s="63" t="inlineStr">
-        <is>
-          <t>الحكم</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="67" t="inlineStr">
-        <is>
-          <t>ح1</t>
-        </is>
-      </c>
-      <c r="B5" s="67" t="n">
-        <v>6</v>
-      </c>
-      <c r="C5" s="67" t="n">
-        <v>4</v>
-      </c>
-      <c r="D5" s="67" t="n">
-        <v>6</v>
-      </c>
-      <c r="E5" s="67" t="n">
-        <v>0</v>
-      </c>
-      <c r="F5" s="67" t="n">
-        <v>1</v>
-      </c>
-      <c r="G5" s="67" t="n">
-        <v>1</v>
-      </c>
-      <c r="H5" s="67" t="n">
-        <v>2</v>
-      </c>
-      <c r="I5" s="67" t="n">
-        <v>0</v>
-      </c>
-      <c r="J5" s="67" t="n">
-        <v>0</v>
-      </c>
-      <c r="K5" s="67" t="inlineStr">
-        <is>
-          <t>جيد؛ بقيت فجوتان: مقارنة مباشرة بين القرآن والحديث النبوي، والمقارنة العامة بين دور القرآن والإنجيل.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="67" t="inlineStr">
-        <is>
-          <t>ح5</t>
-        </is>
-      </c>
-      <c r="B6" s="67" t="n">
-        <v>2</v>
-      </c>
-      <c r="C6" s="67" t="n">
-        <v>2</v>
-      </c>
-      <c r="D6" s="67" t="n">
-        <v>2</v>
-      </c>
-      <c r="E6" s="67" t="n">
-        <v>0</v>
-      </c>
-      <c r="F6" s="67" t="n">
-        <v>0</v>
-      </c>
-      <c r="G6" s="67" t="n">
-        <v>0</v>
-      </c>
-      <c r="H6" s="67" t="n">
-        <v>0</v>
-      </c>
-      <c r="I6" s="67" t="n">
-        <v>0</v>
-      </c>
-      <c r="J6" s="67" t="n">
-        <v>0</v>
-      </c>
-      <c r="K6" s="67" t="inlineStr">
-        <is>
-          <t>جيد في عرض الموضوعات والقصص؛ لا يغطي استدلالاً مستقلاً على تاريخية القصص.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="67" t="inlineStr">
-        <is>
-          <t>ح2</t>
-        </is>
-      </c>
-      <c r="B7" s="67" t="n">
-        <v>6</v>
-      </c>
-      <c r="C7" s="67" t="n">
-        <v>2</v>
-      </c>
-      <c r="D7" s="67" t="n">
-        <v>6</v>
-      </c>
-      <c r="E7" s="67" t="n">
-        <v>0</v>
-      </c>
-      <c r="F7" s="67" t="n">
-        <v>1</v>
-      </c>
-      <c r="G7" s="67" t="n">
-        <v>2</v>
-      </c>
-      <c r="H7" s="67" t="n">
-        <v>1</v>
-      </c>
-      <c r="I7" s="67" t="n">
-        <v>1</v>
-      </c>
-      <c r="J7" s="67" t="n">
-        <v>0</v>
-      </c>
-      <c r="K7" s="67" t="inlineStr">
-        <is>
-          <t>جيد؛ بقيت فجوات في تعريف الوحي المباشر، ومدة النزول، وأول ما نزل.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="67" t="inlineStr">
-        <is>
-          <t>ح3</t>
-        </is>
-      </c>
-      <c r="B8" s="67" t="n">
-        <v>6</v>
-      </c>
-      <c r="C8" s="67" t="n">
-        <v>0</v>
-      </c>
-      <c r="D8" s="67" t="n">
-        <v>5</v>
-      </c>
-      <c r="E8" s="67" t="n">
-        <v>0</v>
-      </c>
-      <c r="F8" s="67" t="n">
-        <v>1</v>
-      </c>
-      <c r="G8" s="67" t="n">
-        <v>2</v>
-      </c>
-      <c r="H8" s="67" t="n">
-        <v>0</v>
-      </c>
-      <c r="I8" s="67" t="n">
-        <v>6</v>
-      </c>
-      <c r="J8" s="67" t="n">
-        <v>0</v>
-      </c>
-      <c r="K8" s="67" t="inlineStr">
-        <is>
-          <t>جيد؛ المقارنة المباشرة بين جمع أبي بكر وجمع عثمان تغطيتها جزئية.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="67" t="inlineStr">
-        <is>
-          <t>ح4</t>
-        </is>
-      </c>
-      <c r="B9" s="67" t="n">
-        <v>4</v>
-      </c>
-      <c r="C9" s="67" t="n">
-        <v>1</v>
-      </c>
-      <c r="D9" s="67" t="n">
-        <v>4</v>
-      </c>
-      <c r="E9" s="67" t="n">
-        <v>0</v>
-      </c>
-      <c r="F9" s="67" t="n">
-        <v>0</v>
-      </c>
-      <c r="G9" s="67" t="n">
-        <v>2</v>
-      </c>
-      <c r="H9" s="67" t="n">
-        <v>0</v>
-      </c>
-      <c r="I9" s="67" t="n">
-        <v>2</v>
-      </c>
-      <c r="J9" s="67" t="n">
-        <v>0</v>
-      </c>
-      <c r="K9" s="67" t="inlineStr">
-        <is>
-          <t>غير مكتمل عملياً؛ تعريف البنية موجود لكن الوصول إلى آية/جزء محدد غير مغطى.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="67" t="inlineStr">
-        <is>
-          <t>ح6</t>
-        </is>
-      </c>
-      <c r="B10" s="67" t="n">
-        <v>5</v>
-      </c>
-      <c r="C10" s="67" t="n">
-        <v>0</v>
-      </c>
-      <c r="D10" s="67" t="n">
-        <v>5</v>
-      </c>
-      <c r="E10" s="67" t="n">
-        <v>1</v>
-      </c>
-      <c r="F10" s="67" t="n">
-        <v>0</v>
-      </c>
-      <c r="G10" s="67" t="n">
-        <v>0</v>
-      </c>
-      <c r="H10" s="67" t="n">
-        <v>2</v>
-      </c>
-      <c r="I10" s="67" t="n">
-        <v>0</v>
-      </c>
-      <c r="J10" s="67" t="n">
-        <v>3</v>
-      </c>
-      <c r="K10" s="67" t="inlineStr">
-        <is>
-          <t>غير مكتمل عملياً؛ توجد مواد للفهم والفضل والترجمة، لكن نقطة البداية واختيار تفسير للمبتدئ غير مغطاتين.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="67" t="inlineStr">
-        <is>
-          <t>ح7</t>
-        </is>
-      </c>
-      <c r="B11" s="67" t="n">
-        <v>5</v>
-      </c>
-      <c r="C11" s="67" t="n">
-        <v>0</v>
-      </c>
-      <c r="D11" s="67" t="n">
-        <v>0</v>
-      </c>
-      <c r="E11" s="67" t="n">
-        <v>0</v>
-      </c>
-      <c r="F11" s="67" t="n">
-        <v>5</v>
-      </c>
-      <c r="G11" s="67" t="n">
-        <v>5</v>
-      </c>
-      <c r="H11" s="67" t="n">
-        <v>1</v>
-      </c>
-      <c r="I11" s="67" t="n">
-        <v>1</v>
-      </c>
-      <c r="J11" s="67" t="n">
-        <v>0</v>
-      </c>
-      <c r="K11" s="67" t="inlineStr">
-        <is>
-          <t>جيد في الاستدلال والاعتراضات؛ بقيت فجوة فرعية في سؤال معرفة النبي ﷺ بالقراءة والكتابة.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12"/>
-    <row r="13"/>
-    <row r="14"/>
-    <row r="15">
-      <c r="A15" s="45" t="inlineStr">
-        <is>
-          <t>فجوات واضحة تحتاج محتوى أو معالجة صريحة</t>
-        </is>
-      </c>
-      <c r="B15" s="1" t="n"/>
-      <c r="C15" s="1" t="n"/>
-      <c r="D15" s="1" t="n"/>
-      <c r="E15" s="1" t="n"/>
-      <c r="F15" s="1" t="n"/>
-      <c r="G15" s="1" t="n"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="63" t="inlineStr">
-        <is>
-          <t>الحاجة</t>
-        </is>
-      </c>
-      <c r="B16" s="63" t="inlineStr">
-        <is>
-          <t>السؤال/الفجوة</t>
-        </is>
-      </c>
-      <c r="C16" s="63" t="inlineStr">
-        <is>
-          <t>نوع الفجوة</t>
-        </is>
-      </c>
-      <c r="D16" s="63" t="inlineStr">
-        <is>
-          <t>الأولوية</t>
-        </is>
-      </c>
-      <c r="E16" s="63" t="inlineStr">
-        <is>
-          <t>الدليل من السجل</t>
-        </is>
-      </c>
-      <c r="F16" s="63" t="inlineStr">
-        <is>
-          <t>الحالة</t>
-        </is>
-      </c>
-      <c r="G16" s="63" t="inlineStr">
-        <is>
-          <t>الإجراء الهيكلي</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="60" customHeight="1" s="49">
-      <c r="A17" s="67" t="inlineStr">
-        <is>
-          <t>ح1</t>
-        </is>
-      </c>
-      <c r="B17" s="67" t="inlineStr">
-        <is>
-          <t>ما الفرق بين القرآن والحديث؟</t>
-        </is>
-      </c>
-      <c r="C17" s="67" t="inlineStr">
-        <is>
-          <t>تغطية مباشرة مفقودة</t>
-        </is>
-      </c>
-      <c r="D17" s="67" t="inlineStr">
-        <is>
-          <t>متوسطة</t>
-        </is>
-      </c>
-      <c r="E17" s="67" t="inlineStr">
-        <is>
-          <t>ق-35 يستبعد الفرق الشامل بين القرآن والحديث النبوي؛ ق-32 يعالج حجية السنة.</t>
-        </is>
-      </c>
-      <c r="F17" s="67" t="inlineStr">
-        <is>
-          <t>غير مغطى مباشرة</t>
-        </is>
-      </c>
-      <c r="G17" s="67" t="inlineStr">
-        <is>
-          <t>إضافة مقطع مقارنة مباشر أو إعلان عدم التغطية.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="60" customHeight="1" s="49">
-      <c r="A18" s="67" t="inlineStr">
-        <is>
-          <t>ح2</t>
-        </is>
-      </c>
-      <c r="B18" s="67" t="inlineStr">
-        <is>
-          <t>كم سنة استمر نزول القرآن؟</t>
-        </is>
-      </c>
-      <c r="C18" s="67" t="inlineStr">
-        <is>
-          <t>معلومة تأسيسية مفقودة</t>
-        </is>
-      </c>
-      <c r="D18" s="67" t="inlineStr">
-        <is>
-          <t>متوسطة</t>
-        </is>
-      </c>
-      <c r="E18" s="67" t="inlineStr">
-        <is>
-          <t>مذكور ضمن صياغات الحاجة ح2 ولا يوجد مقطع يجيب عنها مباشرة.</t>
-        </is>
-      </c>
-      <c r="F18" s="67" t="inlineStr">
-        <is>
-          <t>غير مغطى</t>
-        </is>
-      </c>
-      <c r="G18" s="67" t="inlineStr">
-        <is>
-          <t>إضافة مقتطف موثق مباشر.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="60" customHeight="1" s="49">
-      <c r="A19" s="67" t="inlineStr">
-        <is>
-          <t>ح2</t>
-        </is>
-      </c>
-      <c r="B19" s="67" t="inlineStr">
-        <is>
-          <t>ما أول آية نزلت؟</t>
-        </is>
-      </c>
-      <c r="C19" s="67" t="inlineStr">
-        <is>
-          <t>معلومة تأسيسية مفقودة</t>
-        </is>
-      </c>
-      <c r="D19" s="67" t="inlineStr">
-        <is>
-          <t>متوسطة</t>
-        </is>
-      </c>
-      <c r="E19" s="67" t="inlineStr">
-        <is>
-          <t>مذكور ضمن صياغات الحاجة ح2 ولا يوجد مقطع يجيب عنها مباشرة.</t>
-        </is>
-      </c>
-      <c r="F19" s="67" t="inlineStr">
-        <is>
-          <t>غير مغطى</t>
-        </is>
-      </c>
-      <c r="G19" s="67" t="inlineStr">
-        <is>
-          <t>إضافة مقتطف موثق مباشر.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="60" customHeight="1" s="49">
-      <c r="A20" s="67" t="inlineStr">
-        <is>
-          <t>ح3</t>
-        </is>
-      </c>
-      <c r="B20" s="67" t="inlineStr">
-        <is>
-          <t>ما الفرق بين جمع أبي بكر وجمع عثمان؟</t>
-        </is>
-      </c>
-      <c r="C20" s="67" t="inlineStr">
-        <is>
-          <t>مقارنة جزئية</t>
-        </is>
-      </c>
-      <c r="D20" s="67" t="inlineStr">
-        <is>
-          <t>متوسطة</t>
-        </is>
-      </c>
-      <c r="E20" s="67" t="inlineStr">
-        <is>
-          <t>ق-13 يذكر صراحة أنه لا يجيب عن المقارنة؛ ق-33 يعرض المراحل دون مقارنة مركزة.</t>
-        </is>
-      </c>
-      <c r="F20" s="67" t="inlineStr">
-        <is>
-          <t>جزئي</t>
-        </is>
-      </c>
-      <c r="G20" s="67" t="inlineStr">
-        <is>
-          <t>إضافة مقارنة قصيرة أو PARTIAL بحدود واضحة.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="60" customHeight="1" s="49">
-      <c r="A21" s="67" t="inlineStr">
-        <is>
-          <t>ح4</t>
-        </is>
-      </c>
-      <c r="B21" s="67" t="inlineStr">
-        <is>
-          <t>كيف أجد آية في المصحف؟</t>
-        </is>
-      </c>
-      <c r="C21" s="67" t="inlineStr">
-        <is>
-          <t>تعليم عملي مفقود</t>
-        </is>
-      </c>
-      <c r="D21" s="67" t="inlineStr">
-        <is>
-          <t>عالية</t>
-        </is>
-      </c>
-      <c r="E21" s="67" t="inlineStr">
-        <is>
-          <t>ق-15 يسجلها ضمن الأسئلة القريبة التي لا يجيب عنها.</t>
-        </is>
-      </c>
-      <c r="F21" s="67" t="inlineStr">
-        <is>
-          <t>غير مغطى</t>
-        </is>
-      </c>
-      <c r="G21" s="67" t="inlineStr">
-        <is>
-          <t>إضافة مقطع/إرشاد عملي مستقل.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="60" customHeight="1" s="49">
-      <c r="A22" s="67" t="inlineStr">
-        <is>
-          <t>ح4</t>
-        </is>
-      </c>
-      <c r="B22" s="67" t="inlineStr">
-        <is>
-          <t>ما معنى جزء عمّ؟</t>
-        </is>
-      </c>
-      <c r="C22" s="67" t="inlineStr">
-        <is>
-          <t>تعريف عملي مفقود</t>
-        </is>
-      </c>
-      <c r="D22" s="67" t="inlineStr">
-        <is>
-          <t>متوسطة</t>
-        </is>
-      </c>
-      <c r="E22" s="67" t="inlineStr">
-        <is>
-          <t>مذكور ضمن صياغات الحاجة ح4 ولا يوجد مقطع مباشر.</t>
-        </is>
-      </c>
-      <c r="F22" s="67" t="inlineStr">
-        <is>
-          <t>غير مغطى</t>
-        </is>
-      </c>
-      <c r="G22" s="67" t="inlineStr">
-        <is>
-          <t>إضافة مقتطف تعريفي مباشر.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="60" customHeight="1" s="49">
-      <c r="A23" s="67" t="inlineStr">
-        <is>
-          <t>ح4</t>
-        </is>
-      </c>
-      <c r="B23" s="67" t="inlineStr">
-        <is>
-          <t>كيف أعرف رقم الآية؟</t>
-        </is>
-      </c>
-      <c r="C23" s="67" t="inlineStr">
-        <is>
-          <t>تعليم عملي مفقود</t>
-        </is>
-      </c>
-      <c r="D23" s="67" t="inlineStr">
-        <is>
-          <t>عالية</t>
-        </is>
-      </c>
-      <c r="E23" s="67" t="inlineStr">
-        <is>
-          <t>مذكور ضمن صياغات الحاجة ح4 ولا يوجد مقطع مباشر.</t>
-        </is>
-      </c>
-      <c r="F23" s="67" t="inlineStr">
-        <is>
-          <t>غير مغطى</t>
-        </is>
-      </c>
-      <c r="G23" s="67" t="inlineStr">
-        <is>
-          <t>إضافة مقطع/إرشاد عملي مستقل.</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="60" customHeight="1" s="49">
-      <c r="A24" s="67" t="inlineStr">
-        <is>
-          <t>ح6</t>
-        </is>
-      </c>
-      <c r="B24" s="67" t="inlineStr">
-        <is>
-          <t>من أين أبدأ قراءة القرآن؟</t>
-        </is>
-      </c>
-      <c r="C24" s="67" t="inlineStr">
-        <is>
-          <t>توجيه عملي مفقود</t>
-        </is>
-      </c>
-      <c r="D24" s="67" t="inlineStr">
-        <is>
-          <t>عالية</t>
-        </is>
-      </c>
-      <c r="E24" s="67" t="inlineStr">
-        <is>
-          <t>ق-18 في ورقة «الناقص» الأصلية: من أين يبدأ المبتدئ القراءة.</t>
-        </is>
-      </c>
-      <c r="F24" s="67" t="inlineStr">
-        <is>
-          <t>غير مغطى</t>
-        </is>
-      </c>
-      <c r="G24" s="67" t="inlineStr">
-        <is>
-          <t>إضافة مادة بداية عملية قبل التجميد.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="60" customHeight="1" s="49">
-      <c r="A25" s="67" t="inlineStr">
-        <is>
-          <t>ح6</t>
-        </is>
-      </c>
-      <c r="B25" s="67" t="inlineStr">
-        <is>
-          <t>ما أفضل تفسير للمبتدئ؟</t>
-        </is>
-      </c>
-      <c r="C25" s="67" t="inlineStr">
-        <is>
-          <t>توجيه مصدر مفقود</t>
-        </is>
-      </c>
-      <c r="D25" s="67" t="inlineStr">
-        <is>
-          <t>عالية</t>
-        </is>
-      </c>
-      <c r="E25" s="67" t="inlineStr">
-        <is>
-          <t>ق-19 يسجل السؤال ضمن الأسئلة القريبة التي لا يجيب عنها.</t>
-        </is>
-      </c>
-      <c r="F25" s="67" t="inlineStr">
-        <is>
-          <t>غير مغطى</t>
-        </is>
-      </c>
-      <c r="G25" s="67" t="inlineStr">
-        <is>
-          <t>إضافة توصية مصدر مراجعة وفق سياسة المرجعية أو إحالة مضبوطة.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="60" customHeight="1" s="49">
-      <c r="A26" s="67" t="inlineStr">
-        <is>
-          <t>ح7</t>
-        </is>
-      </c>
-      <c r="B26" s="67" t="inlineStr">
-        <is>
-          <t>هل كان النبي يعرف القراءة والكتابة؟</t>
-        </is>
-      </c>
-      <c r="C26" s="67" t="inlineStr">
-        <is>
-          <t>استدلال فرعي مفقود</t>
-        </is>
-      </c>
-      <c r="D26" s="67" t="inlineStr">
-        <is>
-          <t>متوسطة</t>
-        </is>
-      </c>
-      <c r="E26" s="67" t="inlineStr">
-        <is>
-          <t>مذكور ضمن صياغات الحاجة ح7 ولا يوجد مقطع يجيب عنه مباشرة.</t>
-        </is>
-      </c>
-      <c r="F26" s="67" t="inlineStr">
-        <is>
-          <t>غير مغطى</t>
-        </is>
-      </c>
-      <c r="G26" s="67" t="inlineStr">
-        <is>
-          <t>إضافة مقتطف موثق إذا سيبقى السؤال ضمن الوعود النشطة.</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="42" customHeight="1" s="49">
-      <c r="A27" s="94" t="inlineStr">
-        <is>
-          <t>ح1</t>
-        </is>
-      </c>
-      <c r="B27" s="94" t="inlineStr">
-        <is>
-          <t>هل القرآن مثل الإنجيل عند المسيحيين؟</t>
-        </is>
-      </c>
-      <c r="C27" s="94" t="inlineStr">
-        <is>
-          <t>مقارنة عامة ملتبسة وغير مغطاة مباشرة</t>
-        </is>
-      </c>
-      <c r="D27" s="94" t="inlineStr">
-        <is>
-          <t>متوسطة</t>
-        </is>
-      </c>
-      <c r="E27" s="94" t="inlineStr">
-        <is>
-          <t>ق-03 يشرح علاقة القرآن بالكتب السابقة، لا المقارنة بين دور القرآن عند المسلمين ودور الإنجيل عند المسيحيين.</t>
-        </is>
-      </c>
-      <c r="F27" s="94" t="inlineStr">
-        <is>
-          <t>غير مغطى مباشرة</t>
-        </is>
-      </c>
-      <c r="G27" s="94" t="inlineStr">
-        <is>
-          <t>CLARIFY حسب المقصود، أو NOT_COVERED إذا كان المقصود مقارنة الدور الديني العامة.</t>
-        </is>
-      </c>
-      <c r="H27" s="94" t="n"/>
-      <c r="I27" s="94" t="n"/>
-      <c r="J27" s="94" t="n"/>
-      <c r="K27" s="94" t="n"/>
-    </row>
-    <row r="28" ht="42" customHeight="1" s="49">
-      <c r="A28" s="93" t="inlineStr">
-        <is>
-          <t>ح2</t>
-        </is>
-      </c>
-      <c r="B28" s="93" t="inlineStr">
-        <is>
-          <t>ما هو الوحي؟</t>
-        </is>
-      </c>
-      <c r="C28" s="93" t="inlineStr">
-        <is>
-          <t>تعريف تأسيسي غير مباشر</t>
-        </is>
-      </c>
-      <c r="D28" s="93" t="inlineStr">
-        <is>
-          <t>عالية</t>
-        </is>
-      </c>
-      <c r="E28" s="93" t="inlineStr">
-        <is>
-          <t>ق-08 يشرح صور مجيء الوحي للنبي ﷺ، لكنه لا يقدم تعريفاً تمهيدياً مستقلاً لمفهوم الوحي.</t>
-        </is>
-      </c>
-      <c r="F28" s="93" t="inlineStr">
-        <is>
-          <t>جزئي</t>
-        </is>
-      </c>
-      <c r="G28" s="93" t="inlineStr">
-        <is>
-          <t>PARTIAL أو إضافة تعريف مباشر قبل توسيع الوعد.</t>
-        </is>
-      </c>
-      <c r="H28" s="93" t="n"/>
-      <c r="I28" s="93" t="n"/>
-      <c r="J28" s="93" t="n"/>
-      <c r="K28" s="93" t="n"/>
-    </row>
-    <row r="29" ht="42" customHeight="1" s="49">
-      <c r="A29" s="94" t="inlineStr">
-        <is>
-          <t>ح5</t>
-        </is>
-      </c>
-      <c r="B29" s="94" t="inlineStr">
-        <is>
-          <t>كيف نعرف أن قصص القرآن حقيقية؟</t>
-        </is>
-      </c>
-      <c r="C29" s="94" t="inlineStr">
-        <is>
-          <t>استدلال/اعتراض غير مغطى</t>
-        </is>
-      </c>
-      <c r="D29" s="94" t="inlineStr">
-        <is>
-          <t>متوسطة</t>
-        </is>
-      </c>
-      <c r="E29" s="94" t="inlineStr">
-        <is>
-          <t>ق-06 يعرّف القصص وأنواعها وغاياتها، لكنه لا يقدم دليلاً مستقلاً لمن يطلب إثبات تاريخيتها.</t>
-        </is>
-      </c>
-      <c r="F29" s="94" t="inlineStr">
-        <is>
-          <t>غير مغطى</t>
-        </is>
-      </c>
-      <c r="G29" s="94" t="inlineStr">
-        <is>
-          <t>NOT_COVERED ضمن النسخة الحالية ما لم تضاف مادة استدلالية مستقلة.</t>
-        </is>
-      </c>
-      <c r="H29" s="94" t="n"/>
-      <c r="I29" s="94" t="n"/>
-      <c r="J29" s="94" t="n"/>
-      <c r="K29" s="94" t="n"/>
-    </row>
-    <row r="30">
-      <c r="A30" s="95" t="inlineStr">
-        <is>
-          <t>ح1</t>
-        </is>
-      </c>
-      <c r="B30" s="95" t="inlineStr">
-        <is>
-          <t>هل القرآن مثل الإنجيل عند المسيحيين؟</t>
-        </is>
-      </c>
-      <c r="C30" s="95" t="inlineStr">
-        <is>
-          <t>مقارنة غير مغطاة</t>
-        </is>
-      </c>
-      <c r="D30" s="95" t="inlineStr">
-        <is>
-          <t>متوسطة</t>
-        </is>
-      </c>
-      <c r="E30" s="95" t="inlineStr">
-        <is>
-          <t>v22: ق-03 يستبعدها صراحة؛ يجيب عن صلة القرآن بالكتب السابقة لا عن مقارنة دوره بدور الإنجيل.</t>
-        </is>
-      </c>
-      <c r="F30" s="95" t="inlineStr">
-        <is>
-          <t>غير مغطى</t>
-        </is>
-      </c>
-      <c r="G30" s="95" t="inlineStr">
-        <is>
-          <t>حُذفت من صياغات ح1 النشطة؛ تُضاف مادة مقارنة مباشرة أو يبقى الامتناع.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="3">
-    <mergeCell ref="A2:K2"/>
-    <mergeCell ref="A1:K1"/>
-    <mergeCell ref="A15:G15"/>
-  </mergeCells>
-  <conditionalFormatting sqref="D17:D26">
-    <cfRule type="expression" priority="1" dxfId="0">
-      <formula>D17="عالية"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <tableParts count="2">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
-  </tableParts>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Prepare (local only) library v24 (ق-37: count question becomes PARTIAL, not a negative match) and the unified development gold (62 cases) as eval/cases_dev_unified.jsonl, converted verbatim; not wired to the judge yet
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RkXtRf8o9rcFbV2XzFoBFz
</commit_message>
<xml_diff>
--- a/data/register.xlsx
+++ b/data/register.xlsx
@@ -867,7 +867,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F15"/>
+  <dimension ref="A1:F16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" style="49" min="1" max="1"/>
@@ -1075,6 +1075,18 @@
       <c r="B15" t="inlineStr">
         <is>
           <t>v23 (المرشحة النهائية، 5 أكتوبر 2026): v22 + قرارات المنع والاستيضاح الأخيرة (ق-14، ق-25، ق-06)، وقالبا استيضاح مرجعيان غير مفعّلين (ست-07، ست-08)، وفجوات جديدة، و«سجل التغييرات». صفر تغييرات في النص المرجعي. القاعدة: المنع لما لا يصلح للسؤال أصلاً؛ PARTIAL لما يفيد دون أن يكمل؛ CLARIFY لما يحتمل معنى يجيب عنه المقطع ومعنى لا يجيب عنه.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>النسخة v24</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>v24 (5 أكتوبر 2026): v23 + إزالة منع «كم مرة تحديداً نزل القرآن؟» من ق-37 (PARTIAL). صفر تغييرات في النص المرجعي.</t>
         </is>
       </c>
     </row>
@@ -1143,7 +1155,6 @@
       <c r="J2" s="1" t="n"/>
       <c r="K2" s="1" t="n"/>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="63" t="inlineStr">
         <is>
@@ -1474,9 +1485,6 @@
         </is>
       </c>
     </row>
-    <row r="12"/>
-    <row r="13"/>
-    <row r="14"/>
     <row r="15">
       <c r="A15" s="45" t="inlineStr">
         <is>
@@ -5385,7 +5393,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E36"/>
+  <dimension ref="A1:E38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" style="49" min="1" max="1"/>
@@ -6362,6 +6370,60 @@
         </is>
       </c>
       <c r="E36" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>v24</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>ق-37</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>أسئلة قريبة لا يجيب عنها</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>حُذف «كم مرة تحديداً نزل القرآن؟»؛ وأُضيف «لا يحدد عددًا معينًا لمرات نزول القرآن.» إلى «لا يجيب عن»</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>PARTIAL بـ ق-37 لا منع (ملف Unified Gold: Library Preconditions)</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>v24</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>النص المرجعي</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>0 تغييرات</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -8894,12 +8956,12 @@
       </c>
       <c r="X18" s="67" t="inlineStr">
         <is>
-          <t>لا يجيب عن شهر النزول أو كيفية مجيء الوحي للنبي.</t>
+          <t>لا يجيب عن شهر النزول أو كيفية مجيء الوحي للنبي. لا يحدد عددًا معينًا لمرات نزول القرآن.</t>
         </is>
       </c>
       <c r="Y18" s="67" t="inlineStr">
         <is>
-          <t>في أي شهر نزل القرآن؟ | كيف كان الوحي يأتي النبي؟ | كم مرة تحديداً نزل القرآن؟</t>
+          <t>في أي شهر نزل القرآن؟ | كيف كان الوحي يأتي النبي؟</t>
         </is>
       </c>
       <c r="Z18" s="67" t="inlineStr">
@@ -12256,8 +12318,8 @@
   <mergeCells count="6">
     <mergeCell ref="A2:AH2"/>
     <mergeCell ref="A3:D3"/>
+    <mergeCell ref="N3:AA3"/>
     <mergeCell ref="AB3:AH3"/>
-    <mergeCell ref="N3:AA3"/>
     <mergeCell ref="A1:AH1"/>
     <mergeCell ref="E3:M3"/>
   </mergeCells>
@@ -12346,7 +12408,6 @@
       <c r="N2" s="1" t="n"/>
       <c r="O2" s="1" t="n"/>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="63" t="inlineStr">
         <is>
@@ -13319,7 +13380,6 @@
       <c r="G2" s="1" t="n"/>
       <c r="H2" s="1" t="n"/>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="63" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Batch 1 (library cleanup, v25): drop «ما الرسالة الأساسية في القرآن؟» from ق-05 and record it as a gap; ق-30 keeps «لماذا لم ير الناس جبريل؟» (already present); archive the v24 pre-fix baselines; gold v1.1 with the Changes vs Dev43 sheet completed mechanically. Engine unchanged; 0 reference-text changes
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RkXtRf8o9rcFbV2XzFoBFz
</commit_message>
<xml_diff>
--- a/data/register.xlsx
+++ b/data/register.xlsx
@@ -867,7 +867,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:F17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" style="49" min="1" max="1"/>
@@ -1087,6 +1087,18 @@
       <c r="B16" t="inlineStr">
         <is>
           <t>v24 (5 أكتوبر 2026): v23 + إزالة منع «كم مرة تحديداً نزل القرآن؟» من ق-37 (PARTIAL). صفر تغييرات في النص المرجعي.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>النسخة v25</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>v25 (5 أكتوبر 2026): v24 + حذف «ما الرسالة الأساسية في القرآن؟» من ق-05 وتسجيله فجوة. صفر تغييرات في النص المرجعي.</t>
         </is>
       </c>
     </row>
@@ -1105,7 +1117,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K33"/>
+  <dimension ref="A1:K34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" style="49" min="1" max="1"/>
@@ -1155,6 +1167,7 @@
       <c r="J2" s="1" t="n"/>
       <c r="K2" s="1" t="n"/>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="63" t="inlineStr">
         <is>
@@ -1485,6 +1498,9 @@
         </is>
       </c>
     </row>
+    <row r="12"/>
+    <row r="13"/>
+    <row r="14"/>
     <row r="15">
       <c r="A15" s="45" t="inlineStr">
         <is>
@@ -2173,6 +2189,43 @@
       <c r="G33" s="95" t="inlineStr">
         <is>
           <t>إضافة مادة أو الامتناع.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="95" t="inlineStr">
+        <is>
+          <t>ح5</t>
+        </is>
+      </c>
+      <c r="B34" s="95" t="inlineStr">
+        <is>
+          <t>ما الرسالة الأساسية في القرآن؟</t>
+        </is>
+      </c>
+      <c r="C34" s="95" t="inlineStr">
+        <is>
+          <t>تحديد مفقود</t>
+        </is>
+      </c>
+      <c r="D34" s="95" t="inlineStr">
+        <is>
+          <t>متوسطة</t>
+        </is>
+      </c>
+      <c r="E34" s="95" t="inlineStr">
+        <is>
+          <t>v25: ق-05 يعدد أبرز الموضوعات ولا يحدد رسالة واحدة؛ حُذفت الصياغة من ق-05 (قياس السجل v24: ق-05/r2).</t>
+        </is>
+      </c>
+      <c r="F34" s="95" t="inlineStr">
+        <is>
+          <t>غير مغطى</t>
+        </is>
+      </c>
+      <c r="G34" s="95" t="inlineStr">
+        <is>
+          <t>إضافة مادة مباشرة أو الامتناع.</t>
         </is>
       </c>
     </row>
@@ -5393,7 +5446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E38"/>
+  <dimension ref="A1:E42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" style="49" min="1" max="1"/>
@@ -6424,6 +6477,114 @@
         </is>
       </c>
       <c r="E38" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>v25</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>ق-05</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>صياغات المستخدم</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>حُذف «ما الرسالة الأساسية في القرآن؟»؛ وأُضيف «يعدد أبرز موضوعات القرآن، ولا يحدد رسالة واحدة بوصفها الرسالة الأساسية للقرآن.» إلى الحدود و«لا يجيب عن»</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>ق-05 لا يحدد رسالة واحدة (قياس السجل v24)</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>v25</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>ح5</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>صياغات المستخدم</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>«ما الرسالة الأساسية في القرآن؟» موسوم [فجوة]</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>لا يُصدَّر للموجّه</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>v25</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>ق-30</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>صياغات المستخدم</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>لا تغيير: «لماذا لم ير الناس جبريل؟» موجود أصلاً في صياغاته</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>ق-30 يجيب عنه (حكمة خفاء الوحي والابتلاء)</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>v25</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>النص المرجعي</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>0 تغييرات</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -7787,7 +7948,7 @@
       </c>
       <c r="O11" s="67" t="inlineStr">
         <is>
-          <t>عن ماذا يتكلم القرآن؟ | ما الرسالة الأساسية في القرآن؟ | هل القرآن كتاب أحكام فقط؟ | هل يتكلم القرآن عن يوم القيامة؟ | ماذا يطلب القرآن من الإنسان؟</t>
+          <t>عن ماذا يتكلم القرآن؟ | هل القرآن كتاب أحكام فقط؟ | هل يتكلم القرآن عن يوم القيامة؟ | ماذا يطلب القرآن من الإنسان؟</t>
         </is>
       </c>
       <c r="P11" s="67" t="inlineStr">
@@ -7827,12 +7988,12 @@
       </c>
       <c r="W11" s="67" t="inlineStr">
         <is>
-          <t>يلخص أبرز موضوعات القرآن، ولا يفسر سورة أو قصة بعينها.</t>
+          <t>يلخص أبرز موضوعات القرآن، ولا يفسر سورة أو قصة بعينها. يعدد أبرز موضوعات القرآن، ولا يحدد رسالة واحدة بوصفها الرسالة الأساسية للقرآن.</t>
         </is>
       </c>
       <c r="X11" s="67" t="inlineStr">
         <is>
-          <t>لا يجيب عن قصة نبي بعينه ولا عن تفسير سورة محددة.</t>
+          <t>لا يجيب عن قصة نبي بعينه ولا عن تفسير سورة محددة. يعدد أبرز موضوعات القرآن، ولا يحدد رسالة واحدة بوصفها الرسالة الأساسية للقرآن.</t>
         </is>
       </c>
       <c r="Y11" s="67" t="inlineStr">
@@ -12317,8 +12478,8 @@
   </sheetData>
   <mergeCells count="6">
     <mergeCell ref="A2:AH2"/>
+    <mergeCell ref="N3:AA3"/>
     <mergeCell ref="A3:D3"/>
-    <mergeCell ref="N3:AA3"/>
     <mergeCell ref="AB3:AH3"/>
     <mergeCell ref="A1:AH1"/>
     <mergeCell ref="E3:M3"/>
@@ -12408,6 +12569,7 @@
       <c r="N2" s="1" t="n"/>
       <c r="O2" s="1" t="n"/>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="63" t="inlineStr">
         <is>
@@ -12588,7 +12750,7 @@
       </c>
       <c r="F6" s="67" t="inlineStr">
         <is>
-          <t>«عن ماذا يتكلم القرآن؟» · «ما الرسالة الأساسية في القرآن؟» · «هل القرآن فيه قصص؟» · «هل القرآن كتاب أحكام فقط؟» · «ماذا يطلب القرآن من الإنسان؟» · «هل يتكلم القرآن عن يوم القيامة؟»</t>
+          <t>«عن ماذا يتكلم القرآن؟» · «ما الرسالة الأساسية في القرآن؟» [فجوة] · «هل القرآن فيه قصص؟» · «هل القرآن كتاب أحكام فقط؟» · «ماذا يطلب القرآن من الإنسان؟» · «هل يتكلم القرآن عن يوم القيامة؟»</t>
         </is>
       </c>
       <c r="G6" s="67" t="inlineStr">

</xml_diff>